<commit_message>
Model: hiển thị số kỳ chiết khấu DCF dạng thập phân (0,25–4,25)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018d4TrajAJ6BNPb7i8Se7c9
</commit_message>
<xml_diff>
--- a/AgriPack_Model_final.xlsx
+++ b/AgriPack_Model_final.xlsx
@@ -2471,7 +2471,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="28">
+  <numFmts count="30">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* \-??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="0%"/>
@@ -2496,10 +2496,12 @@
     <numFmt numFmtId="185" formatCode="_(* #,##0_);_(* \(#,##0\);_(* \-_);_(@_)"/>
     <numFmt numFmtId="186" formatCode="#,##0.00"/>
     <numFmt numFmtId="187" formatCode="0.000"/>
-    <numFmt numFmtId="188" formatCode="0.0\x"/>
-    <numFmt numFmtId="189" formatCode="0.0"/>
-    <numFmt numFmtId="190" formatCode="\+#,##0.0;\-#,##0.0;0.0"/>
-    <numFmt numFmtId="191" formatCode="\+0%;\-0%;0%"/>
+    <numFmt numFmtId="188" formatCode="[$-409]0.00"/>
+    <numFmt numFmtId="189" formatCode="[$-409]0%"/>
+    <numFmt numFmtId="190" formatCode="0.0\x"/>
+    <numFmt numFmtId="191" formatCode="0.0"/>
+    <numFmt numFmtId="192" formatCode="\+#,##0.0;\-#,##0.0;0.0"/>
+    <numFmt numFmtId="193" formatCode="\+0%;\-0%;0%"/>
   </numFmts>
   <fonts count="61">
     <font>
@@ -3688,7 +3690,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="888">
+  <cellXfs count="892">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -6397,6 +6399,14 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="188" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="188" fontId="0" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -6457,94 +6467,102 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="189" fontId="0" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="189" fontId="44" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="15" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="186" fontId="0" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="37" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="46" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="47" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="46" fillId="5" borderId="40" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="46" fillId="5" borderId="40" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="46" fillId="3" borderId="40" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="46" fillId="3" borderId="40" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="8" borderId="30" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="8" fillId="8" borderId="30" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="47" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="37" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="59" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="38" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="40" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="37" fillId="5" borderId="2" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="37" fillId="5" borderId="3" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="177" fontId="44" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="15" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="186" fontId="0" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="37" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="46" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="47" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="46" fillId="5" borderId="40" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="177" fontId="46" fillId="5" borderId="40" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="177" fontId="46" fillId="3" borderId="40" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="46" fillId="3" borderId="40" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="30" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="177" fontId="8" fillId="8" borderId="30" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="177" fontId="47" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="177" fontId="0" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="177" fontId="37" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="59" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="177" fontId="38" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="177" fontId="40" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="21" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="37" fillId="5" borderId="2" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="177" fontId="37" fillId="5" borderId="3" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="37" fillId="5" borderId="6" xfId="21" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="2" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -6621,7 +6639,7 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="2" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="188" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="190" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6793,7 +6811,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="188" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="190" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6809,7 +6827,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="188" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="190" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6849,7 +6867,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="189" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="191" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6873,7 +6891,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="189" fontId="9" fillId="3" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="191" fontId="9" fillId="3" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -7169,11 +7187,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="190" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="192" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="190" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="192" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -7181,7 +7199,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="190" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="192" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -7213,11 +7231,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="191" fontId="7" fillId="7" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="193" fontId="7" fillId="7" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="191" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="193" fontId="7" fillId="7" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -7327,9 +7345,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>775440</xdr:colOff>
+      <xdr:colOff>775080</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>195120</xdr:rowOff>
+      <xdr:rowOff>194760</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7343,7 +7361,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="277560" y="317160"/>
-          <a:ext cx="1051560" cy="289440"/>
+          <a:ext cx="1051200" cy="289080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -9407,26 +9425,26 @@
       <c r="A3" s="676" t="s">
         <v>548</v>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="677" t="n">
         <v>0.25</v>
       </c>
-      <c r="C3" s="599" t="n">
+      <c r="C3" s="678" t="n">
         <f aca="false">B3</f>
         <v>0.25</v>
       </c>
-      <c r="D3" s="599" t="n">
+      <c r="D3" s="678" t="n">
         <f aca="false">C3+1</f>
         <v>1.25</v>
       </c>
-      <c r="E3" s="599" t="n">
+      <c r="E3" s="678" t="n">
         <f aca="false">D3+1</f>
         <v>2.25</v>
       </c>
-      <c r="F3" s="599" t="n">
+      <c r="F3" s="678" t="n">
         <f aca="false">E3+1</f>
         <v>3.25</v>
       </c>
-      <c r="G3" s="599" t="n">
+      <c r="G3" s="678" t="n">
         <f aca="false">F3+1</f>
         <v>4.25</v>
       </c>
@@ -9436,32 +9454,32 @@
       <c r="K3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="677"/>
-      <c r="B4" s="678" t="n">
+      <c r="A4" s="679"/>
+      <c r="B4" s="680" t="n">
         <f aca="false">'Income Statement'!D2</f>
         <v>2025</v>
       </c>
-      <c r="C4" s="678" t="n">
+      <c r="C4" s="680" t="n">
         <f aca="false">B4+1</f>
         <v>2026</v>
       </c>
-      <c r="D4" s="678" t="n">
+      <c r="D4" s="680" t="n">
         <f aca="false">C4+1</f>
         <v>2027</v>
       </c>
-      <c r="E4" s="678" t="n">
+      <c r="E4" s="680" t="n">
         <f aca="false">D4+1</f>
         <v>2028</v>
       </c>
-      <c r="F4" s="678" t="n">
+      <c r="F4" s="680" t="n">
         <f aca="false">E4+1</f>
         <v>2029</v>
       </c>
-      <c r="G4" s="678" t="n">
+      <c r="G4" s="680" t="n">
         <f aca="false">F4+1</f>
         <v>2030</v>
       </c>
-      <c r="H4" s="679" t="n">
+      <c r="H4" s="681" t="n">
         <f aca="false">G4+1</f>
         <v>2031</v>
       </c>
@@ -9470,134 +9488,134 @@
       <c r="K4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="680" t="s">
+      <c r="A5" s="682" t="s">
         <v>549</v>
       </c>
-      <c r="B5" s="681"/>
-      <c r="C5" s="682" t="n">
+      <c r="B5" s="683"/>
+      <c r="C5" s="684" t="n">
         <f aca="false">'Pro Forma'!C10-Drivers!F136*MAX(0,'Pro Forma'!C10-Drivers!F134)</f>
         <v>6712155.67662171</v>
       </c>
-      <c r="D5" s="682" t="n">
+      <c r="D5" s="684" t="n">
         <f aca="false">'Pro Forma'!D10-Drivers!G136*MAX(0,'Pro Forma'!D10-Drivers!G134)</f>
         <v>8583370.39044625</v>
       </c>
-      <c r="E5" s="682" t="n">
+      <c r="E5" s="684" t="n">
         <f aca="false">'Pro Forma'!E10-Drivers!H136*MAX(0,'Pro Forma'!E10-Drivers!H134)</f>
         <v>10267189.2831959</v>
       </c>
-      <c r="F5" s="682" t="n">
+      <c r="F5" s="684" t="n">
         <f aca="false">'Pro Forma'!F10-Drivers!I136*MAX(0,'Pro Forma'!F10-Drivers!I134)</f>
         <v>8109168.20303413</v>
       </c>
-      <c r="G5" s="682" t="n">
+      <c r="G5" s="684" t="n">
         <f aca="false">'Pro Forma'!G10-Drivers!J136*MAX(0,'Pro Forma'!G10-Drivers!J134)</f>
         <v>16321728.8378721</v>
       </c>
-      <c r="H5" s="683"/>
+      <c r="H5" s="685"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="684" t="s">
+      <c r="A6" s="686" t="s">
         <v>550</v>
       </c>
-      <c r="B6" s="681"/>
-      <c r="C6" s="682" t="n">
+      <c r="B6" s="683"/>
+      <c r="C6" s="684" t="n">
         <f aca="false">'Pro Forma'!C9</f>
         <v>3742094.4</v>
       </c>
-      <c r="D6" s="682" t="n">
+      <c r="D6" s="684" t="n">
         <f aca="false">'Pro Forma'!D9</f>
         <v>5270266.00775904</v>
       </c>
-      <c r="E6" s="682" t="n">
+      <c r="E6" s="684" t="n">
         <f aca="false">'Pro Forma'!E9</f>
         <v>6736300.28805754</v>
       </c>
-      <c r="F6" s="682" t="n">
+      <c r="F6" s="684" t="n">
         <f aca="false">'Pro Forma'!F9</f>
         <v>14567897.0477264</v>
       </c>
-      <c r="G6" s="682" t="n">
+      <c r="G6" s="684" t="n">
         <f aca="false">'Pro Forma'!G9</f>
         <v>16573405.0090052</v>
       </c>
-      <c r="H6" s="683"/>
+      <c r="H6" s="685"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="684" t="s">
+      <c r="A7" s="686" t="s">
         <v>551</v>
       </c>
-      <c r="B7" s="681"/>
-      <c r="C7" s="682" t="n">
+      <c r="B7" s="683"/>
+      <c r="C7" s="684" t="n">
         <f aca="false">'Pro Forma'!C37</f>
         <v>2584386.32806608</v>
       </c>
-      <c r="D7" s="682" t="n">
+      <c r="D7" s="684" t="n">
         <f aca="false">'Pro Forma'!D37</f>
         <v>3454529.79565908</v>
       </c>
-      <c r="E7" s="682" t="n">
+      <c r="E7" s="684" t="n">
         <f aca="false">'Pro Forma'!E37</f>
         <v>4040072.02117552</v>
       </c>
-      <c r="F7" s="682" t="n">
+      <c r="F7" s="684" t="n">
         <f aca="false">'Pro Forma'!F37</f>
         <v>9368456.35975228</v>
       </c>
-      <c r="G7" s="682" t="n">
+      <c r="G7" s="684" t="n">
         <f aca="false">'Pro Forma'!G37</f>
         <v>6556463.86375452</v>
       </c>
-      <c r="H7" s="683"/>
+      <c r="H7" s="685"/>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="684" t="s">
+      <c r="A8" s="686" t="s">
         <v>552</v>
       </c>
-      <c r="B8" s="681"/>
-      <c r="C8" s="682" t="n">
+      <c r="B8" s="683"/>
+      <c r="C8" s="684" t="n">
         <f aca="false">'Pro Forma'!C25</f>
         <v>12734763.397992</v>
       </c>
-      <c r="D8" s="682" t="n">
+      <c r="D8" s="684" t="n">
         <f aca="false">'Pro Forma'!D25</f>
         <v>12216952.3358209</v>
       </c>
-      <c r="E8" s="682" t="n">
+      <c r="E8" s="684" t="n">
         <f aca="false">'Pro Forma'!E25</f>
         <v>65263306.3305742</v>
       </c>
-      <c r="F8" s="682" t="n">
+      <c r="F8" s="684" t="n">
         <f aca="false">'Pro Forma'!F25</f>
         <v>16712566.34399</v>
       </c>
-      <c r="G8" s="682" t="n">
+      <c r="G8" s="684" t="n">
         <f aca="false">'Pro Forma'!G25</f>
         <v>17889220.9029689</v>
       </c>
-      <c r="H8" s="683"/>
+      <c r="H8" s="685"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="685"/>
-      <c r="B9" s="681"/>
-      <c r="C9" s="681"/>
-      <c r="D9" s="681"/>
-      <c r="E9" s="681"/>
-      <c r="F9" s="681"/>
-      <c r="G9" s="681"/>
-      <c r="H9" s="686" t="s">
+      <c r="A9" s="687"/>
+      <c r="B9" s="683"/>
+      <c r="C9" s="683"/>
+      <c r="D9" s="683"/>
+      <c r="E9" s="683"/>
+      <c r="F9" s="683"/>
+      <c r="G9" s="683"/>
+      <c r="H9" s="688" t="s">
         <v>553</v>
       </c>
       <c r="I9" s="2"/>
@@ -9605,68 +9623,68 @@
       <c r="K9" s="2"/>
     </row>
     <row r="10" s="604" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="687" t="s">
+      <c r="A10" s="689" t="s">
         <v>554</v>
       </c>
-      <c r="B10" s="688"/>
-      <c r="C10" s="688" t="n">
+      <c r="B10" s="690"/>
+      <c r="C10" s="690" t="n">
         <f aca="false">C5+C6-C7-C8</f>
         <v>-4864899.64943637</v>
       </c>
-      <c r="D10" s="688" t="n">
+      <c r="D10" s="690" t="n">
         <f aca="false">D5+D6-D7-D8</f>
         <v>-1817845.73327466</v>
       </c>
-      <c r="E10" s="688" t="n">
+      <c r="E10" s="690" t="n">
         <f aca="false">E5+E6-E7-E8</f>
         <v>-52299888.7804963</v>
       </c>
-      <c r="F10" s="688" t="n">
+      <c r="F10" s="690" t="n">
         <f aca="false">F5+F6-F7-F8</f>
         <v>-3403957.45298173</v>
       </c>
-      <c r="G10" s="688" t="n">
+      <c r="G10" s="690" t="n">
         <f aca="false">G5+G6-G7-G8</f>
         <v>8449449.08015391</v>
       </c>
-      <c r="H10" s="689" t="n">
+      <c r="H10" s="691" t="n">
         <f aca="false">G5*(1+Assumption!B14)*(1-Assumption!B14/Assumption!B17)</f>
         <v>10177781.0310875</v>
       </c>
       <c r="I10" s="336" t="s">
         <v>555</v>
       </c>
-      <c r="J10" s="690"/>
-      <c r="K10" s="691"/>
+      <c r="J10" s="692"/>
+      <c r="K10" s="693"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="676" t="s">
         <v>556</v>
       </c>
       <c r="B11" s="599"/>
-      <c r="C11" s="599" t="n">
+      <c r="C11" s="694" t="n">
         <f aca="false">B3</f>
         <v>0.25</v>
       </c>
-      <c r="D11" s="599" t="n">
+      <c r="D11" s="694" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="599" t="n">
+      <c r="E11" s="694" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="599" t="n">
+      <c r="F11" s="694" t="n">
         <v>1</v>
       </c>
-      <c r="G11" s="692" t="n">
+      <c r="G11" s="695" t="n">
         <v>1</v>
       </c>
       <c r="H11" s="599"/>
       <c r="I11" s="2"/>
-      <c r="J11" s="693"/>
-      <c r="K11" s="694"/>
+      <c r="J11" s="696"/>
+      <c r="K11" s="697"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="695" t="s">
+      <c r="A12" s="698" t="s">
         <v>557</v>
       </c>
       <c r="B12" s="599"/>
@@ -9674,11 +9692,11 @@
       <c r="D12" s="599"/>
       <c r="E12" s="599"/>
       <c r="F12" s="2"/>
-      <c r="G12" s="696" t="n">
+      <c r="G12" s="699" t="n">
         <f aca="false">H10/(Assumption!B16-Assumption!B14)</f>
         <v>111464230.849885</v>
       </c>
-      <c r="H12" s="697"/>
+      <c r="H12" s="700"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
@@ -9697,27 +9715,27 @@
       <c r="K13" s="2"/>
     </row>
     <row r="14" s="604" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="698" t="s">
+      <c r="A14" s="701" t="s">
         <v>558</v>
       </c>
-      <c r="B14" s="699"/>
-      <c r="C14" s="700" t="n">
+      <c r="B14" s="702"/>
+      <c r="C14" s="703" t="n">
         <f aca="false">C10*C11/(1+Assumption!$B$16)^C3</f>
         <v>-1176692.55216926</v>
       </c>
-      <c r="D14" s="700" t="n">
+      <c r="D14" s="703" t="n">
         <f aca="false">D10*D11/(1+Assumption!$B$16)^D3</f>
         <v>-1540999.76815546</v>
       </c>
-      <c r="E14" s="700" t="n">
+      <c r="E14" s="703" t="n">
         <f aca="false">E10*E11/(1+Assumption!$B$16)^E3</f>
         <v>-38845682.1299611</v>
       </c>
-      <c r="F14" s="700" t="n">
+      <c r="F14" s="703" t="n">
         <f aca="false">F10*F11/(1+Assumption!$B$16)^F3</f>
         <v>-2215248.99593255</v>
       </c>
-      <c r="G14" s="701" t="n">
+      <c r="G14" s="704" t="n">
         <f aca="false">(G10*G11+G12)/(1+Assumption!$B$16)^G3</f>
         <v>68375984.852971</v>
       </c>
@@ -9736,25 +9754,25 @@
       <c r="G15" s="599"/>
       <c r="H15" s="599"/>
       <c r="I15" s="2"/>
-      <c r="J15" s="702"/>
+      <c r="J15" s="705"/>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" s="708" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="703" t="s">
+    <row r="16" s="711" customFormat="true" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="706" t="s">
         <v>559</v>
       </c>
-      <c r="B16" s="704"/>
-      <c r="C16" s="704" t="n">
+      <c r="B16" s="707"/>
+      <c r="C16" s="707" t="n">
         <f aca="false">SUM(C14:G14)</f>
         <v>24597361.4067526</v>
       </c>
-      <c r="D16" s="705"/>
-      <c r="E16" s="706"/>
-      <c r="F16" s="706"/>
-      <c r="G16" s="707"/>
-      <c r="H16" s="707"/>
+      <c r="D16" s="708"/>
+      <c r="E16" s="709"/>
+      <c r="F16" s="709"/>
+      <c r="G16" s="710"/>
+      <c r="H16" s="710"/>
       <c r="I16" s="2"/>
-      <c r="J16" s="693"/>
+      <c r="J16" s="696"/>
       <c r="K16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9764,53 +9782,53 @@
       <c r="D17" s="599"/>
       <c r="E17" s="599"/>
       <c r="F17" s="599"/>
-      <c r="G17" s="702"/>
-      <c r="H17" s="702"/>
+      <c r="G17" s="705"/>
+      <c r="H17" s="705"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="676"/>
-      <c r="B18" s="709"/>
-      <c r="C18" s="710"/>
-      <c r="D18" s="711"/>
+      <c r="B18" s="712"/>
+      <c r="C18" s="713"/>
+      <c r="D18" s="714"/>
       <c r="E18" s="599"/>
       <c r="F18" s="599"/>
-      <c r="G18" s="702"/>
-      <c r="H18" s="702"/>
+      <c r="G18" s="705"/>
+      <c r="H18" s="705"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="712" t="s">
+      <c r="A19" s="715" t="s">
         <v>544</v>
       </c>
-      <c r="B19" s="713" t="n">
+      <c r="B19" s="716" t="n">
         <f aca="false">'Pro Forma'!B61</f>
         <v>40464671.3598887</v>
       </c>
-      <c r="C19" s="692"/>
-      <c r="D19" s="711"/>
+      <c r="C19" s="717"/>
+      <c r="D19" s="714"/>
       <c r="E19" s="599"/>
       <c r="F19" s="599"/>
-      <c r="G19" s="702"/>
-      <c r="H19" s="702"/>
+      <c r="G19" s="705"/>
+      <c r="H19" s="705"/>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="714" t="s">
+      <c r="A20" s="718" t="s">
         <v>560</v>
       </c>
-      <c r="B20" s="715" t="n">
+      <c r="B20" s="719" t="n">
         <f aca="false">B19/B21</f>
         <v>0.637646281974959</v>
       </c>
-      <c r="C20" s="716"/>
-      <c r="D20" s="711"/>
+      <c r="C20" s="720"/>
+      <c r="D20" s="714"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -9820,15 +9838,15 @@
       <c r="K20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="714" t="s">
+      <c r="A21" s="718" t="s">
         <v>561</v>
       </c>
-      <c r="B21" s="717" t="n">
+      <c r="B21" s="721" t="n">
         <f aca="false">SUM(B22,B19)</f>
         <v>63459432.7666413</v>
       </c>
-      <c r="C21" s="718"/>
-      <c r="D21" s="711"/>
+      <c r="C21" s="722"/>
+      <c r="D21" s="714"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -9838,29 +9856,29 @@
       <c r="K21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="719" t="s">
+      <c r="A22" s="723" t="s">
         <v>562</v>
       </c>
-      <c r="B22" s="720" t="n">
+      <c r="B22" s="724" t="n">
         <f aca="false">B33</f>
         <v>22994761.4067526</v>
       </c>
-      <c r="C22" s="718"/>
-      <c r="D22" s="721" t="s">
+      <c r="C22" s="722"/>
+      <c r="D22" s="725" t="s">
         <v>563</v>
       </c>
-      <c r="E22" s="722" t="n">
+      <c r="E22" s="726" t="n">
         <f aca="false">B19</f>
         <v>40464671.3598887</v>
       </c>
-      <c r="F22" s="723" t="s">
+      <c r="F22" s="727" t="s">
         <v>564</v>
       </c>
-      <c r="G22" s="724" t="n">
+      <c r="G22" s="728" t="n">
         <f aca="false">B20</f>
         <v>0.637646281974959</v>
       </c>
-      <c r="H22" s="725" t="s">
+      <c r="H22" s="729" t="s">
         <v>565</v>
       </c>
       <c r="I22" s="2"/>
@@ -9882,8 +9900,8 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="676"/>
-      <c r="B24" s="711"/>
-      <c r="C24" s="726"/>
+      <c r="B24" s="714"/>
+      <c r="C24" s="730"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
@@ -9907,10 +9925,10 @@
       <c r="K25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="727" t="s">
+      <c r="A26" s="731" t="s">
         <v>566</v>
       </c>
-      <c r="B26" s="728"/>
+      <c r="B26" s="732"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -9922,10 +9940,10 @@
       <c r="K26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="729" t="s">
+      <c r="A27" s="733" t="s">
         <v>567</v>
       </c>
-      <c r="B27" s="730" t="n">
+      <c r="B27" s="734" t="n">
         <f aca="false">SUM(C14:F14)+G10*G11/(1+Assumption!B16)^G3</f>
         <v>-38960662.7043112</v>
       </c>
@@ -9940,10 +9958,10 @@
       <c r="K27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="729" t="s">
+      <c r="A28" s="733" t="s">
         <v>568</v>
       </c>
-      <c r="B28" s="730" t="n">
+      <c r="B28" s="734" t="n">
         <f aca="false">G12/(1+Assumption!B16)^G3</f>
         <v>63558024.1110638</v>
       </c>
@@ -9958,10 +9976,10 @@
       <c r="K28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="729" t="s">
+      <c r="A29" s="733" t="s">
         <v>569</v>
       </c>
-      <c r="B29" s="730" t="n">
+      <c r="B29" s="734" t="n">
         <f aca="false">C16</f>
         <v>24597361.4067526</v>
       </c>
@@ -9976,10 +9994,10 @@
       <c r="K29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="729" t="s">
+      <c r="A30" s="733" t="s">
         <v>570</v>
       </c>
-      <c r="B30" s="731" t="n">
+      <c r="B30" s="735" t="n">
         <f aca="false">B28/B29</f>
         <v>2.58393666946795</v>
       </c>
@@ -9994,10 +10012,10 @@
       <c r="K30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="729" t="s">
+      <c r="A31" s="733" t="s">
         <v>571</v>
       </c>
-      <c r="B31" s="730" t="n">
+      <c r="B31" s="734" t="n">
         <f aca="false">MAX(0,'Balance Sheet'!F6+(1-B3)*C10)</f>
         <v>0</v>
       </c>
@@ -10012,10 +10030,10 @@
       <c r="K31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="729" t="s">
+      <c r="A32" s="733" t="s">
         <v>572</v>
       </c>
-      <c r="B32" s="730" t="n">
+      <c r="B32" s="734" t="n">
         <f aca="false">SUM('Balance Sheet'!F45,'Balance Sheet'!F58)</f>
         <v>1602600</v>
       </c>
@@ -10030,10 +10048,10 @@
       <c r="K32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="732" t="s">
+      <c r="A33" s="736" t="s">
         <v>573</v>
       </c>
-      <c r="B33" s="730" t="n">
+      <c r="B33" s="734" t="n">
         <f aca="false">B29+B31-B32</f>
         <v>22994761.4067526</v>
       </c>
@@ -10048,10 +10066,10 @@
       <c r="K33" s="2"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="729" t="s">
+      <c r="A34" s="733" t="s">
         <v>574</v>
       </c>
-      <c r="B34" s="733" t="n">
+      <c r="B34" s="737" t="n">
         <f aca="false">B29/Drivers!E77</f>
         <v>3.19669222750901</v>
       </c>
@@ -10066,10 +10084,10 @@
       <c r="K34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="729" t="s">
+      <c r="A35" s="733" t="s">
         <v>575</v>
       </c>
-      <c r="B35" s="733" t="n">
+      <c r="B35" s="737" t="n">
         <f aca="false">B29/Drivers!F77</f>
         <v>2.16065711154623</v>
       </c>
@@ -10084,10 +10102,10 @@
       <c r="K35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="729" t="s">
+      <c r="A36" s="733" t="s">
         <v>576</v>
       </c>
-      <c r="B36" s="733" t="n">
+      <c r="B36" s="737" t="n">
         <f aca="false">B33/'Income Statement'!E78</f>
         <v>3.49510146280095</v>
       </c>
@@ -10102,7 +10120,7 @@
       <c r="K36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="729" t="s">
+      <c r="A37" s="733" t="s">
         <v>577</v>
       </c>
       <c r="B37" s="490" t="n">
@@ -10120,10 +10138,10 @@
       <c r="K37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="732" t="s">
+      <c r="A38" s="736" t="s">
         <v>578</v>
       </c>
-      <c r="B38" s="730" t="n">
+      <c r="B38" s="734" t="n">
         <f aca="false">G10*(1+Assumption!B14)/(Assumption!B16-Assumption!B14)</f>
         <v>97162820.3579258</v>
       </c>
@@ -10138,10 +10156,10 @@
       <c r="K38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="729" t="s">
+      <c r="A39" s="733" t="s">
         <v>579</v>
       </c>
-      <c r="B39" s="731" t="n">
+      <c r="B39" s="735" t="n">
         <f aca="false">G5/SUM('Pro Forma'!G24,'Pro Forma'!G36)</f>
         <v>0.123115883251726</v>
       </c>
@@ -10156,10 +10174,10 @@
       <c r="K39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="734" t="s">
+      <c r="A40" s="738" t="s">
         <v>580</v>
       </c>
-      <c r="B40" s="735" t="n">
+      <c r="B40" s="739" t="n">
         <f aca="false">Assumption!B14/Assumption!B17</f>
         <v>0.406121441680834</v>
       </c>
@@ -10213,15 +10231,15 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="736" t="s">
+      <c r="A1" s="740" t="s">
         <v>581</v>
       </c>
-      <c r="B1" s="737"/>
-      <c r="C1" s="738" t="n">
+      <c r="B1" s="741"/>
+      <c r="C1" s="742" t="n">
         <f aca="false">DCF!G4</f>
         <v>2030</v>
       </c>
-      <c r="D1" s="739"/>
+      <c r="D1" s="743"/>
       <c r="E1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10234,104 +10252,104 @@
       <c r="E2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="740" t="s">
+      <c r="A3" s="744" t="s">
         <v>583</v>
       </c>
-      <c r="B3" s="741" t="n">
+      <c r="B3" s="745" t="n">
         <f aca="false">DCF!G3</f>
         <v>4.25</v>
       </c>
       <c r="C3" s="2"/>
-      <c r="D3" s="742" t="s">
+      <c r="D3" s="746" t="s">
         <v>544</v>
       </c>
-      <c r="E3" s="743" t="n">
+      <c r="E3" s="747" t="n">
         <f aca="false">DCF!B19</f>
         <v>40464671.3598887</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="744" t="s">
+      <c r="A4" s="748" t="s">
         <v>584</v>
       </c>
-      <c r="B4" s="745" t="n">
+      <c r="B4" s="749" t="n">
         <v>0.4</v>
       </c>
-      <c r="C4" s="746" t="s">
+      <c r="C4" s="750" t="s">
         <v>585</v>
       </c>
-      <c r="D4" s="747" t="s">
+      <c r="D4" s="751" t="s">
         <v>586</v>
       </c>
-      <c r="E4" s="748" t="n">
+      <c r="E4" s="752" t="n">
         <f aca="false">B35</f>
         <v>200607865.396057</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="744" t="s">
+      <c r="A5" s="748" t="s">
         <v>587</v>
       </c>
-      <c r="B5" s="749" t="n">
+      <c r="B5" s="753" t="n">
         <f aca="false">'Discount rate'!E4</f>
         <v>0.141309839519679</v>
       </c>
       <c r="C5" s="2"/>
-      <c r="D5" s="750" t="s">
+      <c r="D5" s="754" t="s">
         <v>588</v>
       </c>
-      <c r="E5" s="751" t="n">
+      <c r="E5" s="755" t="n">
         <f aca="false">E4/(1+B7)^B3</f>
         <v>68633171.9969417</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="752"/>
-      <c r="B6" s="753"/>
+      <c r="A6" s="756"/>
+      <c r="B6" s="757"/>
       <c r="C6" s="2"/>
-      <c r="D6" s="747" t="s">
+      <c r="D6" s="751" t="s">
         <v>589</v>
       </c>
-      <c r="E6" s="754" t="n">
+      <c r="E6" s="758" t="n">
         <f aca="false">E3/E5</f>
         <v>0.589578919093115</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="755" t="s">
+      <c r="A7" s="759" t="s">
         <v>590</v>
       </c>
-      <c r="B7" s="756" t="n">
+      <c r="B7" s="760" t="n">
         <f aca="false">(1+B5)/(1-B4)^(1/B3)-1</f>
         <v>0.287073258984758</v>
       </c>
       <c r="C7" s="415"/>
-      <c r="D7" s="750" t="s">
+      <c r="D7" s="754" t="s">
         <v>562</v>
       </c>
-      <c r="E7" s="757" t="n">
+      <c r="E7" s="761" t="n">
         <f aca="false">E5-E3</f>
         <v>28168500.6370529</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="339"/>
-      <c r="B8" s="758"/>
+      <c r="B8" s="762"/>
       <c r="C8" s="2"/>
-      <c r="D8" s="759" t="s">
+      <c r="D8" s="763" t="s">
         <v>591</v>
       </c>
-      <c r="E8" s="760" t="n">
+      <c r="E8" s="764" t="n">
         <f aca="false">1-E6</f>
         <v>0.410421080906885</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="339"/>
-      <c r="B9" s="758"/>
+      <c r="B9" s="762"/>
       <c r="C9" s="2"/>
       <c r="D9" s="339"/>
-      <c r="E9" s="761"/>
+      <c r="E9" s="765"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="2"/>
@@ -10341,21 +10359,21 @@
       <c r="E10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="762" t="s">
+      <c r="A11" s="766" t="s">
         <v>563</v>
       </c>
-      <c r="B11" s="722" t="n">
+      <c r="B11" s="726" t="n">
         <f aca="false">E3</f>
         <v>40464671.3598887</v>
       </c>
-      <c r="C11" s="723" t="s">
+      <c r="C11" s="727" t="s">
         <v>564</v>
       </c>
-      <c r="D11" s="724" t="n">
+      <c r="D11" s="728" t="n">
         <f aca="false">E6</f>
         <v>0.589578919093115</v>
       </c>
-      <c r="E11" s="725" t="s">
+      <c r="E11" s="729" t="s">
         <v>565</v>
       </c>
     </row>
@@ -10381,7 +10399,7 @@
       <c r="E14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="763" t="s">
+      <c r="A15" s="767" t="s">
         <v>592</v>
       </c>
       <c r="B15" s="567" t="s">
@@ -10399,45 +10417,45 @@
       <c r="A16" s="436" t="s">
         <v>596</v>
       </c>
-      <c r="B16" s="764" t="n">
+      <c r="B16" s="768" t="n">
         <v>0.65</v>
       </c>
-      <c r="C16" s="764" t="n">
+      <c r="C16" s="768" t="n">
         <v>0.8</v>
       </c>
-      <c r="D16" s="731" t="n">
+      <c r="D16" s="735" t="n">
         <f aca="false">AVERAGE(B16:C16)</f>
         <v>0.725</v>
       </c>
-      <c r="E16" s="765"/>
+      <c r="E16" s="769"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="436" t="s">
         <v>597</v>
       </c>
-      <c r="B17" s="764" t="n">
+      <c r="B17" s="768" t="n">
         <v>0.5</v>
       </c>
-      <c r="C17" s="764" t="n">
+      <c r="C17" s="768" t="n">
         <v>0.65</v>
       </c>
-      <c r="D17" s="731" t="n">
+      <c r="D17" s="735" t="n">
         <f aca="false">AVERAGE(B17:C17)</f>
         <v>0.575</v>
       </c>
-      <c r="E17" s="766"/>
+      <c r="E17" s="770"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="436" t="s">
         <v>598</v>
       </c>
-      <c r="B18" s="764" t="n">
+      <c r="B18" s="768" t="n">
         <v>0.35</v>
       </c>
-      <c r="C18" s="764" t="n">
+      <c r="C18" s="768" t="n">
         <v>0.45</v>
       </c>
-      <c r="D18" s="731" t="n">
+      <c r="D18" s="735" t="n">
         <f aca="false">AVERAGE(B18:C18)</f>
         <v>0.4</v>
       </c>
@@ -10447,13 +10465,13 @@
       <c r="A19" s="485" t="s">
         <v>599</v>
       </c>
-      <c r="B19" s="767" t="n">
+      <c r="B19" s="771" t="n">
         <v>0.2</v>
       </c>
-      <c r="C19" s="767" t="n">
+      <c r="C19" s="771" t="n">
         <v>0.3</v>
       </c>
-      <c r="D19" s="735" t="n">
+      <c r="D19" s="739" t="n">
         <f aca="false">AVERAGE(B19:C19)</f>
         <v>0.25</v>
       </c>
@@ -10470,16 +10488,16 @@
       <c r="A21" s="414" t="s">
         <v>600</v>
       </c>
-      <c r="B21" s="768" t="s">
+      <c r="B21" s="772" t="s">
         <v>598</v>
       </c>
-      <c r="C21" s="769" t="s">
+      <c r="C21" s="773" t="s">
         <v>601</v>
       </c>
-      <c r="D21" s="770"/>
-      <c r="E21" s="770"/>
-      <c r="F21" s="771"/>
-      <c r="G21" s="771"/>
+      <c r="D21" s="774"/>
+      <c r="E21" s="774"/>
+      <c r="F21" s="775"/>
+      <c r="G21" s="775"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="2"/>
@@ -10489,11 +10507,11 @@
       <c r="E22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="772" t="s">
+      <c r="A23" s="776" t="s">
         <v>602</v>
       </c>
-      <c r="B23" s="773"/>
-      <c r="C23" s="774"/>
+      <c r="B23" s="777"/>
+      <c r="C23" s="778"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
     </row>
@@ -10501,7 +10519,7 @@
       <c r="A24" s="18" t="s">
         <v>603</v>
       </c>
-      <c r="B24" s="775" t="n">
+      <c r="B24" s="779" t="n">
         <f aca="false">'Income Statement'!I78</f>
         <v>13374146.0043913</v>
       </c>
@@ -10513,10 +10531,10 @@
       <c r="A25" s="18" t="s">
         <v>604</v>
       </c>
-      <c r="B25" s="776" t="n">
+      <c r="B25" s="780" t="n">
         <v>9.4</v>
       </c>
-      <c r="C25" s="777" t="s">
+      <c r="C25" s="781" t="s">
         <v>605</v>
       </c>
       <c r="D25" s="2"/>
@@ -10526,7 +10544,7 @@
       <c r="A26" s="18" t="s">
         <v>606</v>
       </c>
-      <c r="B26" s="778" t="n">
+      <c r="B26" s="782" t="n">
         <f aca="false">B24*B25</f>
         <v>125716972.441279</v>
       </c>
@@ -10538,7 +10556,7 @@
       <c r="A27" s="18" t="s">
         <v>607</v>
       </c>
-      <c r="B27" s="775" t="n">
+      <c r="B27" s="779" t="n">
         <f aca="false">'Income Statement'!I80</f>
         <v>36975566.0563454</v>
       </c>
@@ -10550,10 +10568,10 @@
       <c r="A28" s="18" t="s">
         <v>608</v>
       </c>
-      <c r="B28" s="776" t="n">
+      <c r="B28" s="780" t="n">
         <v>8</v>
       </c>
-      <c r="C28" s="777" t="s">
+      <c r="C28" s="781" t="s">
         <v>609</v>
       </c>
       <c r="D28" s="2"/>
@@ -10563,7 +10581,7 @@
       <c r="A29" s="18" t="s">
         <v>610</v>
       </c>
-      <c r="B29" s="778" t="n">
+      <c r="B29" s="782" t="n">
         <f aca="false">B27*B28</f>
         <v>295804528.450763</v>
       </c>
@@ -10575,7 +10593,7 @@
       <c r="A30" s="18" t="s">
         <v>611</v>
       </c>
-      <c r="B30" s="775" t="n">
+      <c r="B30" s="779" t="n">
         <f aca="false">'Balance Sheet'!K6</f>
         <v>12623216.9387471</v>
       </c>
@@ -10587,7 +10605,7 @@
       <c r="A31" s="18" t="s">
         <v>612</v>
       </c>
-      <c r="B31" s="775" t="n">
+      <c r="B31" s="779" t="n">
         <f aca="false">SUM('Balance Sheet'!K45,'Balance Sheet'!K58)</f>
         <v>32928987.0386756</v>
       </c>
@@ -10599,7 +10617,7 @@
       <c r="A32" s="18" t="s">
         <v>613</v>
       </c>
-      <c r="B32" s="778" t="n">
+      <c r="B32" s="782" t="n">
         <f aca="false">B29+B30-B31</f>
         <v>275498758.350835</v>
       </c>
@@ -10608,10 +10626,10 @@
       <c r="E32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="779" t="s">
+      <c r="A33" s="783" t="s">
         <v>614</v>
       </c>
-      <c r="B33" s="778" t="n">
+      <c r="B33" s="782" t="n">
         <f aca="false">DCF!G12+B30-B31</f>
         <v>91158460.7499564</v>
       </c>
@@ -10623,7 +10641,7 @@
       <c r="A34" s="18" t="s">
         <v>615</v>
       </c>
-      <c r="B34" s="780" t="n">
+      <c r="B34" s="784" t="n">
         <f aca="false">(B26-B30+B31)/B27</f>
         <v>3.94916854872998</v>
       </c>
@@ -10632,10 +10650,10 @@
       <c r="E34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="779" t="s">
+      <c r="A35" s="783" t="s">
         <v>616</v>
       </c>
-      <c r="B35" s="778" t="n">
+      <c r="B35" s="782" t="n">
         <f aca="false">AVERAGE(B26,B32)</f>
         <v>200607865.396057</v>
       </c>
@@ -10654,7 +10672,7 @@
       <c r="A37" s="18" t="s">
         <v>617</v>
       </c>
-      <c r="B37" s="781" t="n">
+      <c r="B37" s="785" t="n">
         <f aca="false">(E4*E6/E3)^(1/B3)-1</f>
         <v>0.287073258984758</v>
       </c>
@@ -10663,10 +10681,10 @@
       <c r="E37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="782" t="s">
+      <c r="A38" s="786" t="s">
         <v>618</v>
       </c>
-      <c r="B38" s="783" t="n">
+      <c r="B38" s="787" t="n">
         <f aca="false">((1-B4)*E4*E6/E3)^(1/B3)-1</f>
         <v>0.141309839519679</v>
       </c>
@@ -10675,15 +10693,15 @@
       <c r="E38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="784"/>
-      <c r="B39" s="781"/>
+      <c r="A39" s="788"/>
+      <c r="B39" s="785"/>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="784"/>
-      <c r="B40" s="778"/>
+      <c r="A40" s="788"/>
+      <c r="B40" s="782"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2"/>
@@ -10696,7 +10714,7 @@
       <c r="E41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="785"/>
+      <c r="A42" s="789"/>
       <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
@@ -10732,7 +10750,7 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="786" t="s">
+      <c r="A1" s="790" t="s">
         <v>619</v>
       </c>
       <c r="B1" s="226"/>
@@ -10775,7 +10793,7 @@
       <c r="K3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="787" t="s">
+      <c r="A4" s="791" t="s">
         <v>621</v>
       </c>
       <c r="B4" s="419" t="s">
@@ -10810,19 +10828,19 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="788" t="s">
+      <c r="A5" s="792" t="s">
         <v>632</v>
       </c>
-      <c r="B5" s="784" t="s">
+      <c r="B5" s="788" t="s">
         <v>633</v>
       </c>
-      <c r="C5" s="784" t="s">
+      <c r="C5" s="788" t="s">
         <v>634</v>
       </c>
-      <c r="D5" s="789" t="n">
+      <c r="D5" s="793" t="n">
         <v>3938</v>
       </c>
-      <c r="E5" s="790" t="n">
+      <c r="E5" s="794" t="n">
         <v>18.9</v>
       </c>
       <c r="F5" s="569" t="n">
@@ -10831,35 +10849,35 @@
       <c r="G5" s="569" t="n">
         <v>7.48</v>
       </c>
-      <c r="H5" s="791" t="n">
+      <c r="H5" s="795" t="n">
         <v>1</v>
       </c>
-      <c r="I5" s="792" t="n">
+      <c r="I5" s="796" t="n">
         <f aca="false">IF(H5=1,F5,"")</f>
         <v>6.35</v>
       </c>
-      <c r="J5" s="792" t="n">
+      <c r="J5" s="796" t="n">
         <f aca="false">IF(H5=1,G5,"")</f>
         <v>7.48</v>
       </c>
-      <c r="K5" s="777" t="s">
+      <c r="K5" s="781" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="788" t="s">
+      <c r="A6" s="792" t="s">
         <v>636</v>
       </c>
-      <c r="B6" s="784" t="s">
+      <c r="B6" s="788" t="s">
         <v>633</v>
       </c>
-      <c r="C6" s="784" t="s">
+      <c r="C6" s="788" t="s">
         <v>637</v>
       </c>
-      <c r="D6" s="789" t="n">
+      <c r="D6" s="793" t="n">
         <v>5488</v>
       </c>
-      <c r="E6" s="790" t="n">
+      <c r="E6" s="794" t="n">
         <v>8.3</v>
       </c>
       <c r="F6" s="569" t="n">
@@ -10868,35 +10886,35 @@
       <c r="G6" s="569" t="n">
         <v>20.51</v>
       </c>
-      <c r="H6" s="791" t="n">
+      <c r="H6" s="795" t="n">
         <v>1</v>
       </c>
-      <c r="I6" s="792" t="n">
+      <c r="I6" s="796" t="n">
         <f aca="false">IF(H6=1,F6,"")</f>
         <v>8.98</v>
       </c>
-      <c r="J6" s="792" t="n">
+      <c r="J6" s="796" t="n">
         <f aca="false">IF(H6=1,G6,"")</f>
         <v>20.51</v>
       </c>
-      <c r="K6" s="777" t="s">
+      <c r="K6" s="781" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="788" t="s">
+      <c r="A7" s="792" t="s">
         <v>638</v>
       </c>
-      <c r="B7" s="784" t="s">
+      <c r="B7" s="788" t="s">
         <v>633</v>
       </c>
-      <c r="C7" s="784" t="s">
+      <c r="C7" s="788" t="s">
         <v>639</v>
       </c>
-      <c r="D7" s="789" t="n">
+      <c r="D7" s="793" t="n">
         <v>9243</v>
       </c>
-      <c r="E7" s="790" t="n">
+      <c r="E7" s="794" t="n">
         <v>14.2</v>
       </c>
       <c r="F7" s="569" t="n">
@@ -10905,35 +10923,35 @@
       <c r="G7" s="569" t="n">
         <v>5.16</v>
       </c>
-      <c r="H7" s="791" t="n">
+      <c r="H7" s="795" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="792" t="n">
+      <c r="I7" s="796" t="n">
         <f aca="false">IF(H7=1,F7,"")</f>
         <v>3.85</v>
       </c>
-      <c r="J7" s="792" t="n">
+      <c r="J7" s="796" t="n">
         <f aca="false">IF(H7=1,G7,"")</f>
         <v>5.16</v>
       </c>
-      <c r="K7" s="777" t="s">
+      <c r="K7" s="781" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="788" t="s">
+      <c r="A8" s="792" t="s">
         <v>640</v>
       </c>
-      <c r="B8" s="784" t="s">
+      <c r="B8" s="788" t="s">
         <v>633</v>
       </c>
-      <c r="C8" s="784" t="s">
+      <c r="C8" s="788" t="s">
         <v>641</v>
       </c>
-      <c r="D8" s="789" t="n">
+      <c r="D8" s="793" t="n">
         <v>9252</v>
       </c>
-      <c r="E8" s="790" t="n">
+      <c r="E8" s="794" t="n">
         <v>14</v>
       </c>
       <c r="F8" s="569" t="n">
@@ -10942,35 +10960,35 @@
       <c r="G8" s="569" t="n">
         <v>6.98</v>
       </c>
-      <c r="H8" s="791" t="n">
+      <c r="H8" s="795" t="n">
         <v>1</v>
       </c>
-      <c r="I8" s="792" t="n">
+      <c r="I8" s="796" t="n">
         <f aca="false">IF(H8=1,F8,"")</f>
         <v>5.05</v>
       </c>
-      <c r="J8" s="792" t="n">
+      <c r="J8" s="796" t="n">
         <f aca="false">IF(H8=1,G8,"")</f>
         <v>6.98</v>
       </c>
-      <c r="K8" s="777" t="s">
+      <c r="K8" s="781" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="788" t="s">
+      <c r="A9" s="792" t="s">
         <v>642</v>
       </c>
-      <c r="B9" s="784" t="s">
+      <c r="B9" s="788" t="s">
         <v>633</v>
       </c>
-      <c r="C9" s="784" t="s">
+      <c r="C9" s="788" t="s">
         <v>643</v>
       </c>
-      <c r="D9" s="789" t="n">
+      <c r="D9" s="793" t="n">
         <v>3112</v>
       </c>
-      <c r="E9" s="790" t="n">
+      <c r="E9" s="794" t="n">
         <v>9.3</v>
       </c>
       <c r="F9" s="569" t="n">
@@ -10979,35 +10997,35 @@
       <c r="G9" s="569" t="n">
         <v>32.9</v>
       </c>
-      <c r="H9" s="791" t="n">
+      <c r="H9" s="795" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="792" t="n">
+      <c r="I9" s="796" t="n">
         <f aca="false">IF(H9=1,F9,"")</f>
         <v>13.71</v>
       </c>
-      <c r="J9" s="792" t="n">
+      <c r="J9" s="796" t="n">
         <f aca="false">IF(H9=1,G9,"")</f>
         <v>32.9</v>
       </c>
-      <c r="K9" s="777" t="s">
+      <c r="K9" s="781" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="788" t="s">
+      <c r="A10" s="792" t="s">
         <v>644</v>
       </c>
-      <c r="B10" s="784" t="s">
+      <c r="B10" s="788" t="s">
         <v>645</v>
       </c>
-      <c r="C10" s="784" t="s">
+      <c r="C10" s="788" t="s">
         <v>646</v>
       </c>
-      <c r="D10" s="789" t="n">
+      <c r="D10" s="793" t="n">
         <v>1921</v>
       </c>
-      <c r="E10" s="790" t="n">
+      <c r="E10" s="794" t="n">
         <v>14.9</v>
       </c>
       <c r="F10" s="569" t="n">
@@ -11016,35 +11034,35 @@
       <c r="G10" s="569" t="n">
         <v>7.29</v>
       </c>
-      <c r="H10" s="791" t="n">
+      <c r="H10" s="795" t="n">
         <v>1</v>
       </c>
-      <c r="I10" s="792" t="n">
+      <c r="I10" s="796" t="n">
         <f aca="false">IF(H10=1,F10,"")</f>
         <v>2.66</v>
       </c>
-      <c r="J10" s="792" t="n">
+      <c r="J10" s="796" t="n">
         <f aca="false">IF(H10=1,G10,"")</f>
         <v>7.29</v>
       </c>
-      <c r="K10" s="777" t="s">
+      <c r="K10" s="781" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="788" t="s">
+      <c r="A11" s="792" t="s">
         <v>647</v>
       </c>
-      <c r="B11" s="784" t="s">
+      <c r="B11" s="788" t="s">
         <v>648</v>
       </c>
-      <c r="C11" s="784" t="s">
+      <c r="C11" s="788" t="s">
         <v>649</v>
       </c>
-      <c r="D11" s="789" t="n">
+      <c r="D11" s="793" t="n">
         <v>319</v>
       </c>
-      <c r="E11" s="790" t="n">
+      <c r="E11" s="794" t="n">
         <v>16.4</v>
       </c>
       <c r="F11" s="569" t="n">
@@ -11053,35 +11071,35 @@
       <c r="G11" s="569" t="n">
         <v>16.64</v>
       </c>
-      <c r="H11" s="791" t="n">
+      <c r="H11" s="795" t="n">
         <v>1</v>
       </c>
-      <c r="I11" s="792" t="n">
+      <c r="I11" s="796" t="n">
         <f aca="false">IF(H11=1,F11,"")</f>
         <v>13.33</v>
       </c>
-      <c r="J11" s="792" t="n">
+      <c r="J11" s="796" t="n">
         <f aca="false">IF(H11=1,G11,"")</f>
         <v>16.64</v>
       </c>
-      <c r="K11" s="777" t="s">
+      <c r="K11" s="781" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="788" t="s">
+      <c r="A12" s="792" t="s">
         <v>650</v>
       </c>
-      <c r="B12" s="784" t="s">
+      <c r="B12" s="788" t="s">
         <v>645</v>
       </c>
-      <c r="C12" s="784" t="s">
+      <c r="C12" s="788" t="s">
         <v>637</v>
       </c>
-      <c r="D12" s="789" t="n">
+      <c r="D12" s="793" t="n">
         <v>3179</v>
       </c>
-      <c r="E12" s="790" t="n">
+      <c r="E12" s="794" t="n">
         <v>15.9</v>
       </c>
       <c r="F12" s="569" t="n">
@@ -11090,35 +11108,35 @@
       <c r="G12" s="569" t="n">
         <v>2.54</v>
       </c>
-      <c r="H12" s="791" t="n">
+      <c r="H12" s="795" t="n">
         <v>1</v>
       </c>
-      <c r="I12" s="792" t="n">
+      <c r="I12" s="796" t="n">
         <f aca="false">IF(H12=1,F12,"")</f>
         <v>3.28</v>
       </c>
-      <c r="J12" s="792" t="n">
+      <c r="J12" s="796" t="n">
         <f aca="false">IF(H12=1,G12,"")</f>
         <v>2.54</v>
       </c>
-      <c r="K12" s="777" t="s">
+      <c r="K12" s="781" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="788" t="s">
+      <c r="A13" s="792" t="s">
         <v>651</v>
       </c>
-      <c r="B13" s="784" t="s">
+      <c r="B13" s="788" t="s">
         <v>633</v>
       </c>
-      <c r="C13" s="784" t="s">
+      <c r="C13" s="788" t="s">
         <v>652</v>
       </c>
-      <c r="D13" s="789" t="n">
+      <c r="D13" s="793" t="n">
         <v>431</v>
       </c>
-      <c r="E13" s="790" t="n">
+      <c r="E13" s="794" t="n">
         <v>2.9</v>
       </c>
       <c r="F13" s="569" t="n">
@@ -11127,35 +11145,35 @@
       <c r="G13" s="569" t="n">
         <v>84.23</v>
       </c>
-      <c r="H13" s="791" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="792" t="str">
+      <c r="H13" s="795" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="796" t="str">
         <f aca="false">IF(H13=1,F13,"")</f>
         <v/>
       </c>
-      <c r="J13" s="792" t="str">
+      <c r="J13" s="796" t="str">
         <f aca="false">IF(H13=1,G13,"")</f>
         <v/>
       </c>
-      <c r="K13" s="777" t="s">
+      <c r="K13" s="781" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="788" t="s">
+      <c r="A14" s="792" t="s">
         <v>654</v>
       </c>
-      <c r="B14" s="784" t="s">
+      <c r="B14" s="788" t="s">
         <v>648</v>
       </c>
-      <c r="C14" s="784" t="s">
+      <c r="C14" s="788" t="s">
         <v>655</v>
       </c>
-      <c r="D14" s="789" t="n">
+      <c r="D14" s="793" t="n">
         <v>2042</v>
       </c>
-      <c r="E14" s="790" t="n">
+      <c r="E14" s="794" t="n">
         <v>1.9</v>
       </c>
       <c r="F14" s="569" t="n">
@@ -11164,35 +11182,35 @@
       <c r="G14" s="569" t="n">
         <v>9.97</v>
       </c>
-      <c r="H14" s="791" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="792" t="str">
+      <c r="H14" s="795" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="796" t="str">
         <f aca="false">IF(H14=1,F14,"")</f>
         <v/>
       </c>
-      <c r="J14" s="792" t="str">
+      <c r="J14" s="796" t="str">
         <f aca="false">IF(H14=1,G14,"")</f>
         <v/>
       </c>
-      <c r="K14" s="777" t="s">
+      <c r="K14" s="781" t="s">
         <v>653</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="788" t="s">
+      <c r="A15" s="792" t="s">
         <v>656</v>
       </c>
-      <c r="B15" s="784" t="s">
+      <c r="B15" s="788" t="s">
         <v>633</v>
       </c>
-      <c r="C15" s="784" t="s">
+      <c r="C15" s="788" t="s">
         <v>657</v>
       </c>
-      <c r="D15" s="789" t="n">
+      <c r="D15" s="793" t="n">
         <v>490</v>
       </c>
-      <c r="E15" s="790" t="n">
+      <c r="E15" s="794" t="n">
         <v>7</v>
       </c>
       <c r="F15" s="569" t="n">
@@ -11201,70 +11219,70 @@
       <c r="G15" s="569" t="n">
         <v>20.41</v>
       </c>
-      <c r="H15" s="791" t="n">
+      <c r="H15" s="795" t="n">
         <v>1</v>
       </c>
-      <c r="I15" s="792" t="n">
+      <c r="I15" s="796" t="n">
         <f aca="false">IF(H15=1,F15,"")</f>
         <v>4.21</v>
       </c>
-      <c r="J15" s="792" t="n">
+      <c r="J15" s="796" t="n">
         <f aca="false">IF(H15=1,G15,"")</f>
         <v>20.41</v>
       </c>
-      <c r="K15" s="777" t="s">
+      <c r="K15" s="781" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="788" t="s">
+      <c r="A16" s="792" t="s">
         <v>658</v>
       </c>
-      <c r="B16" s="784" t="s">
+      <c r="B16" s="788" t="s">
         <v>645</v>
       </c>
-      <c r="C16" s="784" t="s">
+      <c r="C16" s="788" t="s">
         <v>637</v>
       </c>
-      <c r="D16" s="789" t="n">
+      <c r="D16" s="793" t="n">
         <v>913</v>
       </c>
-      <c r="E16" s="790"/>
+      <c r="E16" s="794"/>
       <c r="F16" s="569" t="n">
         <v>4.17</v>
       </c>
       <c r="G16" s="569" t="n">
         <v>4.85</v>
       </c>
-      <c r="H16" s="791" t="n">
+      <c r="H16" s="795" t="n">
         <v>1</v>
       </c>
-      <c r="I16" s="792" t="n">
+      <c r="I16" s="796" t="n">
         <f aca="false">IF(H16=1,F16,"")</f>
         <v>4.17</v>
       </c>
-      <c r="J16" s="792" t="n">
+      <c r="J16" s="796" t="n">
         <f aca="false">IF(H16=1,G16,"")</f>
         <v>4.85</v>
       </c>
-      <c r="K16" s="777" t="s">
+      <c r="K16" s="781" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="788" t="s">
+      <c r="A17" s="792" t="s">
         <v>659</v>
       </c>
-      <c r="B17" s="784" t="s">
+      <c r="B17" s="788" t="s">
         <v>645</v>
       </c>
-      <c r="C17" s="784" t="s">
+      <c r="C17" s="788" t="s">
         <v>660</v>
       </c>
-      <c r="D17" s="789" t="n">
+      <c r="D17" s="793" t="n">
         <v>484</v>
       </c>
-      <c r="E17" s="790" t="n">
+      <c r="E17" s="794" t="n">
         <v>6.5</v>
       </c>
       <c r="F17" s="569" t="n">
@@ -11273,70 +11291,70 @@
       <c r="G17" s="569" t="n">
         <v>9.19</v>
       </c>
-      <c r="H17" s="791" t="n">
+      <c r="H17" s="795" t="n">
         <v>1</v>
       </c>
-      <c r="I17" s="792" t="n">
+      <c r="I17" s="796" t="n">
         <f aca="false">IF(H17=1,F17,"")</f>
         <v>5.5</v>
       </c>
-      <c r="J17" s="792" t="n">
+      <c r="J17" s="796" t="n">
         <f aca="false">IF(H17=1,G17,"")</f>
         <v>9.19</v>
       </c>
-      <c r="K17" s="777" t="s">
+      <c r="K17" s="781" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="788" t="s">
+      <c r="A18" s="792" t="s">
         <v>661</v>
       </c>
-      <c r="B18" s="784" t="s">
+      <c r="B18" s="788" t="s">
         <v>645</v>
       </c>
-      <c r="C18" s="784" t="s">
+      <c r="C18" s="788" t="s">
         <v>662</v>
       </c>
-      <c r="D18" s="789" t="n">
+      <c r="D18" s="793" t="n">
         <v>212</v>
       </c>
-      <c r="E18" s="790"/>
+      <c r="E18" s="794"/>
       <c r="F18" s="569" t="n">
         <v>2.96</v>
       </c>
       <c r="G18" s="569" t="n">
         <v>6.65</v>
       </c>
-      <c r="H18" s="791" t="n">
+      <c r="H18" s="795" t="n">
         <v>1</v>
       </c>
-      <c r="I18" s="792" t="n">
+      <c r="I18" s="796" t="n">
         <f aca="false">IF(H18=1,F18,"")</f>
         <v>2.96</v>
       </c>
-      <c r="J18" s="792" t="n">
+      <c r="J18" s="796" t="n">
         <f aca="false">IF(H18=1,G18,"")</f>
         <v>6.65</v>
       </c>
-      <c r="K18" s="777" t="s">
+      <c r="K18" s="781" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="788" t="s">
+      <c r="A19" s="792" t="s">
         <v>663</v>
       </c>
-      <c r="B19" s="784" t="s">
+      <c r="B19" s="788" t="s">
         <v>645</v>
       </c>
-      <c r="C19" s="784" t="s">
+      <c r="C19" s="788" t="s">
         <v>664</v>
       </c>
-      <c r="D19" s="789" t="n">
+      <c r="D19" s="793" t="n">
         <v>372</v>
       </c>
-      <c r="E19" s="790" t="n">
+      <c r="E19" s="794" t="n">
         <v>5.3</v>
       </c>
       <c r="F19" s="569" t="n">
@@ -11345,55 +11363,55 @@
       <c r="G19" s="569" t="n">
         <v>6.46</v>
       </c>
-      <c r="H19" s="791" t="n">
+      <c r="H19" s="795" t="n">
         <v>1</v>
       </c>
-      <c r="I19" s="792" t="n">
+      <c r="I19" s="796" t="n">
         <f aca="false">IF(H19=1,F19,"")</f>
         <v>2.06</v>
       </c>
-      <c r="J19" s="792" t="n">
+      <c r="J19" s="796" t="n">
         <f aca="false">IF(H19=1,G19,"")</f>
         <v>6.46</v>
       </c>
-      <c r="K19" s="777" t="s">
+      <c r="K19" s="781" t="s">
         <v>635</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="793" t="s">
+      <c r="A20" s="797" t="s">
         <v>665</v>
       </c>
-      <c r="B20" s="794" t="s">
+      <c r="B20" s="798" t="s">
         <v>645</v>
       </c>
-      <c r="C20" s="794" t="s">
+      <c r="C20" s="798" t="s">
         <v>664</v>
       </c>
-      <c r="D20" s="795" t="n">
+      <c r="D20" s="799" t="n">
         <v>746</v>
       </c>
-      <c r="E20" s="796" t="n">
+      <c r="E20" s="800" t="n">
         <v>4</v>
       </c>
-      <c r="F20" s="797" t="n">
+      <c r="F20" s="801" t="n">
         <v>5.4</v>
       </c>
-      <c r="G20" s="797" t="n">
+      <c r="G20" s="801" t="n">
         <v>5.53</v>
       </c>
-      <c r="H20" s="798" t="n">
+      <c r="H20" s="802" t="n">
         <v>1</v>
       </c>
-      <c r="I20" s="799" t="n">
+      <c r="I20" s="803" t="n">
         <f aca="false">IF(H20=1,F20,"")</f>
         <v>5.4</v>
       </c>
-      <c r="J20" s="799" t="n">
+      <c r="J20" s="803" t="n">
         <f aca="false">IF(H20=1,G20,"")</f>
         <v>5.53</v>
       </c>
-      <c r="K20" s="800" t="s">
+      <c r="K20" s="804" t="s">
         <v>635</v>
       </c>
     </row>
@@ -11418,15 +11436,15 @@
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
-      <c r="F22" s="801" t="n">
+      <c r="F22" s="805" t="n">
         <f aca="false">MEDIAN(I5:I20)</f>
         <v>4.63</v>
       </c>
-      <c r="G22" s="801" t="n">
+      <c r="G22" s="805" t="n">
         <f aca="false">MEDIAN(J5:J20)</f>
         <v>7.135</v>
       </c>
-      <c r="H22" s="802" t="n">
+      <c r="H22" s="806" t="n">
         <f aca="false">SUM(H5:H20)</f>
         <v>14</v>
       </c>
@@ -11442,10 +11460,10 @@
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
-      <c r="F23" s="803" t="n">
+      <c r="F23" s="807" t="n">
         <v>7.99</v>
       </c>
-      <c r="G23" s="803" t="n">
+      <c r="G23" s="807" t="n">
         <v>9.43</v>
       </c>
       <c r="H23" s="336" t="s">
@@ -11484,10 +11502,10 @@
       <c r="K25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="772" t="s">
+      <c r="A26" s="776" t="s">
         <v>670</v>
       </c>
-      <c r="B26" s="774"/>
+      <c r="B26" s="778"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -11502,7 +11520,7 @@
       <c r="A27" s="18" t="s">
         <v>671</v>
       </c>
-      <c r="B27" s="804" t="n">
+      <c r="B27" s="808" t="n">
         <f aca="false">'Income Statement'!D80/1000000</f>
         <v>7.6946292155</v>
       </c>
@@ -11520,7 +11538,7 @@
       <c r="A28" s="18" t="s">
         <v>672</v>
       </c>
-      <c r="B28" s="804" t="n">
+      <c r="B28" s="808" t="n">
         <f aca="false">'Income Statement'!D74/1000000</f>
         <v>4.4204952155</v>
       </c>
@@ -11538,7 +11556,7 @@
       <c r="A29" s="18" t="s">
         <v>673</v>
       </c>
-      <c r="B29" s="805" t="n">
+      <c r="B29" s="809" t="n">
         <f aca="false">Assumption!B13</f>
         <v>0.2</v>
       </c>
@@ -11556,7 +11574,7 @@
       <c r="A30" s="18" t="s">
         <v>674</v>
       </c>
-      <c r="B30" s="806" t="n">
+      <c r="B30" s="810" t="n">
         <f aca="false">B28*(1-B29)</f>
         <v>3.5363961724</v>
       </c>
@@ -11574,7 +11592,7 @@
       <c r="A31" s="18" t="s">
         <v>675</v>
       </c>
-      <c r="B31" s="804" t="n">
+      <c r="B31" s="808" t="n">
         <f aca="false">'Balance Sheet'!F6/1000000</f>
         <v>2.93348176549999</v>
       </c>
@@ -11592,7 +11610,7 @@
       <c r="A32" s="18" t="s">
         <v>676</v>
       </c>
-      <c r="B32" s="804" t="n">
+      <c r="B32" s="808" t="n">
         <f aca="false">SUM('Balance Sheet'!F45,'Balance Sheet'!F58)/1000000</f>
         <v>1.6026</v>
       </c>
@@ -11607,10 +11625,10 @@
       <c r="K32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="782" t="s">
+      <c r="A33" s="786" t="s">
         <v>677</v>
       </c>
-      <c r="B33" s="807" t="n">
+      <c r="B33" s="811" t="n">
         <v>0.3</v>
       </c>
       <c r="C33" s="336" t="s">
@@ -11639,7 +11657,7 @@
       <c r="K34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="808" t="s">
+      <c r="A35" s="812" t="s">
         <v>679</v>
       </c>
       <c r="B35" s="2"/>
@@ -11654,7 +11672,7 @@
       <c r="K35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="809" t="s">
+      <c r="A36" s="813" t="s">
         <v>680</v>
       </c>
       <c r="B36" s="567" t="s">
@@ -11680,19 +11698,19 @@
       <c r="A37" s="18" t="s">
         <v>685</v>
       </c>
-      <c r="B37" s="792" t="n">
+      <c r="B37" s="796" t="n">
         <f aca="false">F22</f>
         <v>4.63</v>
       </c>
-      <c r="C37" s="810" t="n">
+      <c r="C37" s="814" t="n">
         <f aca="false">B27</f>
         <v>7.6946292155</v>
       </c>
-      <c r="D37" s="811" t="n">
+      <c r="D37" s="815" t="n">
         <f aca="false">B37*C37+B31-B32</f>
         <v>36.957015033265</v>
       </c>
-      <c r="E37" s="812" t="n">
+      <c r="E37" s="816" t="n">
         <f aca="false">D37*(1-$B$33)</f>
         <v>25.8699105232855</v>
       </c>
@@ -11707,19 +11725,19 @@
       <c r="A38" s="18" t="s">
         <v>686</v>
       </c>
-      <c r="B38" s="792" t="n">
+      <c r="B38" s="796" t="n">
         <f aca="false">F23</f>
         <v>7.99</v>
       </c>
-      <c r="C38" s="810" t="n">
+      <c r="C38" s="814" t="n">
         <f aca="false">B27</f>
         <v>7.6946292155</v>
       </c>
-      <c r="D38" s="811" t="n">
+      <c r="D38" s="815" t="n">
         <f aca="false">B38*C38+B31-B32</f>
         <v>62.810969197345</v>
       </c>
-      <c r="E38" s="812" t="n">
+      <c r="E38" s="816" t="n">
         <f aca="false">D38*(1-$B$33)</f>
         <v>43.9676784381415</v>
       </c>
@@ -11734,19 +11752,19 @@
       <c r="A39" s="18" t="s">
         <v>687</v>
       </c>
-      <c r="B39" s="792" t="n">
+      <c r="B39" s="796" t="n">
         <f aca="false">G22</f>
         <v>7.135</v>
       </c>
-      <c r="C39" s="810" t="n">
+      <c r="C39" s="814" t="n">
         <f aca="false">B30</f>
         <v>3.5363961724</v>
       </c>
-      <c r="D39" s="811" t="n">
+      <c r="D39" s="815" t="n">
         <f aca="false">B39*C39</f>
         <v>25.232186690074</v>
       </c>
-      <c r="E39" s="812" t="n">
+      <c r="E39" s="816" t="n">
         <f aca="false">D39*(1-$B$33)</f>
         <v>17.6625306830518</v>
       </c>
@@ -11758,22 +11776,22 @@
       <c r="K39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="779" t="s">
+      <c r="A40" s="783" t="s">
         <v>688</v>
       </c>
-      <c r="B40" s="792" t="n">
+      <c r="B40" s="796" t="n">
         <f aca="false">G23</f>
         <v>9.43</v>
       </c>
-      <c r="C40" s="810" t="n">
+      <c r="C40" s="814" t="n">
         <f aca="false">B30</f>
         <v>3.5363961724</v>
       </c>
-      <c r="D40" s="811" t="n">
+      <c r="D40" s="815" t="n">
         <f aca="false">B40*C40</f>
         <v>33.348215905732</v>
       </c>
-      <c r="E40" s="812" t="n">
+      <c r="E40" s="816" t="n">
         <f aca="false">D40*(1-$B$33)</f>
         <v>23.3437511340124</v>
       </c>
@@ -11785,13 +11803,13 @@
       <c r="K40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="788" t="s">
+      <c r="A41" s="792" t="s">
         <v>689</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
-      <c r="E41" s="812" t="n">
+      <c r="E41" s="816" t="n">
         <f aca="false">AVERAGE(E37:E40)</f>
         <v>27.7109676946228</v>
       </c>
@@ -11803,16 +11821,16 @@
       <c r="K41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="813" t="s">
+      <c r="A42" s="817" t="s">
         <v>690</v>
       </c>
       <c r="B42" s="498"/>
       <c r="C42" s="498"/>
-      <c r="D42" s="814" t="n">
+      <c r="D42" s="818" t="n">
         <f aca="false">MIN(E37:E40)</f>
         <v>17.6625306830518</v>
       </c>
-      <c r="E42" s="815" t="n">
+      <c r="E42" s="819" t="n">
         <f aca="false">MAX(E37:E40)</f>
         <v>43.9676784381415</v>
       </c>
@@ -11852,14 +11870,14 @@
       <c r="K44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="772" t="s">
+      <c r="A45" s="776" t="s">
         <v>569</v>
       </c>
-      <c r="B45" s="816" t="n">
+      <c r="B45" s="820" t="n">
         <f aca="false">B49-B31+B32</f>
         <v>26.3800859291228</v>
       </c>
-      <c r="C45" s="785" t="s">
+      <c r="C45" s="789" t="s">
         <v>692</v>
       </c>
       <c r="D45" s="2"/>
@@ -11872,14 +11890,14 @@
       <c r="K45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="817" t="s">
+      <c r="A46" s="821" t="s">
         <v>544</v>
       </c>
-      <c r="B46" s="818" t="n">
+      <c r="B46" s="822" t="n">
         <f aca="false">DCF!B19/1000000</f>
         <v>40.4646713598887</v>
       </c>
-      <c r="C46" s="785" t="s">
+      <c r="C46" s="789" t="s">
         <v>693</v>
       </c>
       <c r="D46" s="2"/>
@@ -11892,10 +11910,10 @@
       <c r="K46" s="2"/>
     </row>
     <row r="47" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="817" t="s">
+      <c r="A47" s="821" t="s">
         <v>589</v>
       </c>
-      <c r="B47" s="819" t="n">
+      <c r="B47" s="823" t="n">
         <f aca="false">B46/B48</f>
         <v>0.593535637084886</v>
       </c>
@@ -11910,10 +11928,10 @@
       <c r="K47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="817" t="s">
+      <c r="A48" s="821" t="s">
         <v>561</v>
       </c>
-      <c r="B48" s="820" t="n">
+      <c r="B48" s="824" t="n">
         <f aca="false">SUM(B49,B46)</f>
         <v>68.1756390545115</v>
       </c>
@@ -11928,14 +11946,14 @@
       <c r="K48" s="2"/>
     </row>
     <row r="49" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="817" t="s">
+      <c r="A49" s="821" t="s">
         <v>562</v>
       </c>
-      <c r="B49" s="820" t="n">
+      <c r="B49" s="824" t="n">
         <f aca="false">E41</f>
         <v>27.7109676946228</v>
       </c>
-      <c r="C49" s="785" t="s">
+      <c r="C49" s="789" t="s">
         <v>694</v>
       </c>
       <c r="D49" s="2"/>
@@ -11948,10 +11966,10 @@
       <c r="K49" s="2"/>
     </row>
     <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="821" t="s">
+      <c r="A50" s="825" t="s">
         <v>591</v>
       </c>
-      <c r="B50" s="822" t="n">
+      <c r="B50" s="826" t="n">
         <f aca="false">1-B47</f>
         <v>0.406464362915114</v>
       </c>
@@ -11979,21 +11997,21 @@
       <c r="K51" s="2"/>
     </row>
     <row r="52" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="823" t="s">
+      <c r="A52" s="827" t="s">
         <v>563</v>
       </c>
-      <c r="B52" s="824" t="n">
+      <c r="B52" s="828" t="n">
         <f aca="false">B46</f>
         <v>40.4646713598887</v>
       </c>
-      <c r="C52" s="825" t="s">
+      <c r="C52" s="829" t="s">
         <v>695</v>
       </c>
-      <c r="D52" s="826" t="n">
+      <c r="D52" s="830" t="n">
         <f aca="false">B47</f>
         <v>0.593535637084886</v>
       </c>
-      <c r="E52" s="825" t="s">
+      <c r="E52" s="829" t="s">
         <v>565</v>
       </c>
       <c r="F52" s="2"/>
@@ -12030,10 +12048,10 @@
       <c r="K54" s="2"/>
     </row>
     <row r="55" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="784"/>
+      <c r="A55" s="788"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
-      <c r="D55" s="811"/>
+      <c r="D55" s="815"/>
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
@@ -12085,7 +12103,7 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="786" t="s">
+      <c r="A1" s="790" t="s">
         <v>696</v>
       </c>
       <c r="B1" s="226"/>
@@ -12137,7 +12155,7 @@
       <c r="N3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="809" t="s">
+      <c r="A4" s="813" t="s">
         <v>698</v>
       </c>
       <c r="B4" s="567" t="s">
@@ -12155,7 +12173,7 @@
       <c r="F4" s="575" t="s">
         <v>703</v>
       </c>
-      <c r="G4" s="827" t="s">
+      <c r="G4" s="831" t="s">
         <v>704</v>
       </c>
       <c r="H4" s="2"/>
@@ -12170,23 +12188,23 @@
       <c r="A5" s="18" t="s">
         <v>705</v>
       </c>
-      <c r="B5" s="811" t="n">
+      <c r="B5" s="815" t="n">
         <f aca="false">DCF!B22/1000000</f>
         <v>22.9947614067526</v>
       </c>
-      <c r="C5" s="811" t="n">
+      <c r="C5" s="815" t="n">
         <f aca="false">DCF!B19/1000000</f>
         <v>40.4646713598887</v>
       </c>
-      <c r="D5" s="811" t="n">
+      <c r="D5" s="815" t="n">
         <f aca="false">SUM(B5:C5)</f>
         <v>63.4594327666413</v>
       </c>
-      <c r="E5" s="781" t="n">
+      <c r="E5" s="785" t="n">
         <f aca="false">IF(B5&lt;=0,"n.m.",C5/D5)</f>
         <v>0.637646281974959</v>
       </c>
-      <c r="F5" s="828" t="n">
+      <c r="F5" s="832" t="n">
         <v>0.4</v>
       </c>
       <c r="G5" s="336" t="s">
@@ -12204,23 +12222,23 @@
       <c r="A6" s="18" t="s">
         <v>707</v>
       </c>
-      <c r="B6" s="811" t="n">
+      <c r="B6" s="815" t="n">
         <f aca="false">VCM!E7/1000000</f>
         <v>28.1685006370529</v>
       </c>
-      <c r="C6" s="811" t="n">
+      <c r="C6" s="815" t="n">
         <f aca="false">VCM!E3/1000000</f>
         <v>40.4646713598887</v>
       </c>
-      <c r="D6" s="811" t="n">
+      <c r="D6" s="815" t="n">
         <f aca="false">SUM(B6:C6)</f>
         <v>68.6331719969417</v>
       </c>
-      <c r="E6" s="781" t="n">
+      <c r="E6" s="785" t="n">
         <f aca="false">IF(B6&lt;=0,"n.m.",C6/D6)</f>
         <v>0.589578919093115</v>
       </c>
-      <c r="F6" s="828" t="n">
+      <c r="F6" s="832" t="n">
         <v>0.4</v>
       </c>
       <c r="G6" s="336" t="s">
@@ -12235,26 +12253,26 @@
       <c r="N6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="779" t="s">
+      <c r="A7" s="783" t="s">
         <v>709</v>
       </c>
-      <c r="B7" s="829" t="n">
+      <c r="B7" s="833" t="n">
         <f aca="false">Multiples!B49</f>
         <v>27.7109676946228</v>
       </c>
-      <c r="C7" s="829" t="n">
+      <c r="C7" s="833" t="n">
         <f aca="false">Multiples!B46</f>
         <v>40.4646713598887</v>
       </c>
-      <c r="D7" s="811" t="n">
+      <c r="D7" s="815" t="n">
         <f aca="false">SUM(B7:C7)</f>
         <v>68.1756390545115</v>
       </c>
-      <c r="E7" s="781" t="n">
+      <c r="E7" s="785" t="n">
         <f aca="false">IF(B7&lt;=0,"n.m.",C7/D7)</f>
         <v>0.593535637084886</v>
       </c>
-      <c r="F7" s="828" t="n">
+      <c r="F7" s="832" t="n">
         <v>0.2</v>
       </c>
       <c r="G7" s="336" t="s">
@@ -12269,26 +12287,26 @@
       <c r="N7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="830" t="s">
+      <c r="A8" s="834" t="s">
         <v>711</v>
       </c>
-      <c r="B8" s="831" t="n">
+      <c r="B8" s="835" t="n">
         <f aca="false">(B5*F5+B6*F6+B7*F7)/SUM(F5:F7)</f>
         <v>26.0074983564468</v>
       </c>
-      <c r="C8" s="831" t="n">
+      <c r="C8" s="835" t="n">
         <f aca="false">C5</f>
         <v>40.4646713598887</v>
       </c>
-      <c r="D8" s="831" t="n">
+      <c r="D8" s="835" t="n">
         <f aca="false">SUM(B8:C8)</f>
         <v>66.4721697163355</v>
       </c>
-      <c r="E8" s="832" t="n">
+      <c r="E8" s="836" t="n">
         <f aca="false">IF(B8&lt;=0,"n.m.",C8/D8)</f>
         <v>0.608746059178877</v>
       </c>
-      <c r="F8" s="833" t="n">
+      <c r="F8" s="837" t="n">
         <f aca="false">SUM(F5:F7)</f>
         <v>1</v>
       </c>
@@ -12302,12 +12320,12 @@
       <c r="N8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="834"/>
-      <c r="B9" s="835"/>
-      <c r="C9" s="835"/>
-      <c r="D9" s="835"/>
-      <c r="E9" s="836"/>
-      <c r="F9" s="837"/>
+      <c r="A9" s="838"/>
+      <c r="B9" s="839"/>
+      <c r="C9" s="839"/>
+      <c r="D9" s="839"/>
+      <c r="E9" s="840"/>
+      <c r="F9" s="841"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -12318,7 +12336,7 @@
       <c r="N9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="808" t="s">
+      <c r="A10" s="812" t="s">
         <v>712</v>
       </c>
       <c r="B10" s="2"/>
@@ -12336,17 +12354,17 @@
       <c r="N10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="838" t="s">
+      <c r="A11" s="842" t="s">
         <v>713</v>
       </c>
-      <c r="B11" s="839" t="n">
+      <c r="B11" s="843" t="n">
         <f aca="false">(1-VCM!B4)*B5+VCM!B4*B12</f>
         <v>19.7912983971515</v>
       </c>
-      <c r="C11" s="840"/>
-      <c r="D11" s="841"/>
-      <c r="E11" s="841"/>
-      <c r="F11" s="841"/>
+      <c r="C11" s="844"/>
+      <c r="D11" s="845"/>
+      <c r="E11" s="845"/>
+      <c r="F11" s="845"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -12357,21 +12375,21 @@
       <c r="N11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="838" t="s">
+      <c r="A12" s="842" t="s">
         <v>714</v>
       </c>
-      <c r="B12" s="839" t="n">
+      <c r="B12" s="843" t="n">
         <f aca="false">C12*'Balance Sheet'!F73/1000000</f>
         <v>14.98610388275</v>
       </c>
-      <c r="C12" s="842" t="n">
+      <c r="C12" s="846" t="n">
         <v>0.5</v>
       </c>
-      <c r="D12" s="843" t="s">
+      <c r="D12" s="847" t="s">
         <v>715</v>
       </c>
-      <c r="E12" s="843"/>
-      <c r="F12" s="843"/>
+      <c r="E12" s="847"/>
+      <c r="F12" s="847"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -12382,8 +12400,8 @@
       <c r="N12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="844"/>
-      <c r="B13" s="811"/>
+      <c r="A13" s="848"/>
+      <c r="B13" s="815"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -12446,7 +12464,7 @@
       <c r="N16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="808" t="s">
+      <c r="A17" s="812" t="s">
         <v>716</v>
       </c>
       <c r="B17" s="2"/>
@@ -12464,7 +12482,7 @@
       <c r="N17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="809" t="s">
+      <c r="A18" s="813" t="s">
         <v>698</v>
       </c>
       <c r="B18" s="567" t="s">
@@ -12490,22 +12508,22 @@
       <c r="N18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="845" t="s">
+      <c r="A19" s="849" t="s">
         <v>48</v>
       </c>
-      <c r="B19" s="846" t="n">
+      <c r="B19" s="850" t="n">
         <f aca="false">MIN(Sensitivity!C7:E9)</f>
         <v>13.4694523430269</v>
       </c>
-      <c r="C19" s="847" t="n">
+      <c r="C19" s="851" t="n">
         <f aca="false">B5</f>
         <v>22.9947614067526</v>
       </c>
-      <c r="D19" s="846" t="n">
+      <c r="D19" s="850" t="n">
         <f aca="false">MAX(Sensitivity!C7:E9)</f>
         <v>33.0495622160443</v>
       </c>
-      <c r="E19" s="848" t="s">
+      <c r="E19" s="852" t="s">
         <v>719</v>
       </c>
       <c r="F19" s="2"/>
@@ -12519,22 +12537,22 @@
       <c r="N19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="845" t="s">
+      <c r="A20" s="849" t="s">
         <v>720</v>
       </c>
-      <c r="B20" s="846" t="n">
+      <c r="B20" s="850" t="n">
         <f aca="false">MIN(Sensitivity!C16:E18)</f>
         <v>13.0120084877283</v>
       </c>
-      <c r="C20" s="847" t="n">
+      <c r="C20" s="851" t="n">
         <f aca="false">B6</f>
         <v>28.1685006370529</v>
       </c>
-      <c r="D20" s="846" t="n">
+      <c r="D20" s="850" t="n">
         <f aca="false">MAX(Sensitivity!C16:E18)</f>
         <v>45.0408220863011</v>
       </c>
-      <c r="E20" s="848" t="s">
+      <c r="E20" s="852" t="s">
         <v>721</v>
       </c>
       <c r="F20" s="2"/>
@@ -12548,22 +12566,22 @@
       <c r="N20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="845" t="s">
+      <c r="A21" s="849" t="s">
         <v>722</v>
       </c>
-      <c r="B21" s="846" t="n">
+      <c r="B21" s="850" t="n">
         <f aca="false">Multiples!D42</f>
         <v>17.6625306830518</v>
       </c>
-      <c r="C21" s="847" t="n">
+      <c r="C21" s="851" t="n">
         <f aca="false">B7</f>
         <v>27.7109676946228</v>
       </c>
-      <c r="D21" s="846" t="n">
+      <c r="D21" s="850" t="n">
         <f aca="false">Multiples!E42</f>
         <v>43.9676784381415</v>
       </c>
-      <c r="E21" s="848" t="s">
+      <c r="E21" s="852" t="s">
         <v>723</v>
       </c>
       <c r="F21" s="2"/>
@@ -12577,22 +12595,22 @@
       <c r="N21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="849" t="s">
+      <c r="A22" s="853" t="s">
         <v>724</v>
       </c>
-      <c r="B22" s="850" t="n">
+      <c r="B22" s="854" t="n">
         <f aca="false">(B19*F5+B20*F6+B21*F7)/F8</f>
         <v>14.1250904689124</v>
       </c>
-      <c r="C22" s="851" t="n">
+      <c r="C22" s="855" t="n">
         <f aca="false">B8</f>
         <v>26.0074983564468</v>
       </c>
-      <c r="D22" s="850" t="n">
+      <c r="D22" s="854" t="n">
         <f aca="false">(D19*F5+D20*F6+D21*F7)/F8</f>
         <v>40.0296894085664</v>
       </c>
-      <c r="E22" s="852" t="s">
+      <c r="E22" s="856" t="s">
         <v>725</v>
       </c>
       <c r="F22" s="2"/>
@@ -12622,7 +12640,7 @@
       <c r="N23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="772" t="s">
+      <c r="A24" s="776" t="s">
         <v>726</v>
       </c>
       <c r="B24" s="548"/>
@@ -12640,10 +12658,10 @@
       <c r="N24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="845" t="s">
+      <c r="A25" s="849" t="s">
         <v>727</v>
       </c>
-      <c r="B25" s="853" t="n">
+      <c r="B25" s="857" t="n">
         <f aca="false">C8</f>
         <v>40.4646713598887</v>
       </c>
@@ -12661,10 +12679,10 @@
       <c r="N25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="845" t="s">
+      <c r="A26" s="849" t="s">
         <v>728</v>
       </c>
-      <c r="B26" s="854" t="n">
+      <c r="B26" s="858" t="n">
         <f aca="false">E8</f>
         <v>0.608746059178877</v>
       </c>
@@ -12682,10 +12700,10 @@
       <c r="N26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="855" t="s">
+      <c r="A27" s="859" t="s">
         <v>729</v>
       </c>
-      <c r="B27" s="856" t="n">
+      <c r="B27" s="860" t="n">
         <f aca="false">SUM(Drivers!F125:J125)/1000000</f>
         <v>39.1579837983445</v>
       </c>
@@ -12703,10 +12721,10 @@
       <c r="N27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="857" t="s">
+      <c r="A28" s="861" t="s">
         <v>730</v>
       </c>
-      <c r="B28" s="858" t="n">
+      <c r="B28" s="862" t="n">
         <f aca="false">SUM(B25,B27)</f>
         <v>79.6226551582333</v>
       </c>
@@ -12756,7 +12774,7 @@
       <c r="N30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="808" t="s">
+      <c r="A31" s="812" t="s">
         <v>731</v>
       </c>
       <c r="B31" s="2"/>
@@ -12792,7 +12810,7 @@
       <c r="N32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="62.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="809" t="s">
+      <c r="A33" s="813" t="s">
         <v>287</v>
       </c>
       <c r="B33" s="567" t="str">
@@ -12824,20 +12842,20 @@
       <c r="A34" s="18" t="s">
         <v>737</v>
       </c>
-      <c r="B34" s="859" t="n">
+      <c r="B34" s="863" t="n">
         <f aca="false">'Income Statement'!I11/1000000</f>
         <v>178.89220902969</v>
       </c>
-      <c r="C34" s="860" t="n">
+      <c r="C34" s="864" t="n">
         <v>121.163880717148</v>
       </c>
-      <c r="D34" s="860" t="n">
+      <c r="D34" s="864" t="n">
         <v>227.441176895844</v>
       </c>
-      <c r="E34" s="860" t="n">
+      <c r="E34" s="864" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="F34" s="861" t="n">
+      <c r="F34" s="865" t="n">
         <v>178.89220902969</v>
       </c>
       <c r="G34" s="2"/>
@@ -12853,20 +12871,20 @@
       <c r="A35" s="18" t="s">
         <v>738</v>
       </c>
-      <c r="B35" s="862" t="n">
+      <c r="B35" s="866" t="n">
         <f aca="false">('Income Statement'!I11/'Income Statement'!D11)^(1/5)-1</f>
         <v>0.303450441286468</v>
       </c>
-      <c r="C35" s="863" t="n">
+      <c r="C35" s="867" t="n">
         <v>0.205732238215002</v>
       </c>
-      <c r="D35" s="863" t="n">
+      <c r="D35" s="867" t="n">
         <v>0.367571548032998</v>
       </c>
-      <c r="E35" s="863" t="n">
+      <c r="E35" s="867" t="n">
         <v>0.303450441286468</v>
       </c>
-      <c r="F35" s="864" t="n">
+      <c r="F35" s="868" t="n">
         <v>0.303450441286468</v>
       </c>
       <c r="G35" s="2"/>
@@ -12882,20 +12900,20 @@
       <c r="A36" s="18" t="s">
         <v>739</v>
       </c>
-      <c r="B36" s="862" t="n">
+      <c r="B36" s="866" t="n">
         <f aca="false">'Income Statement'!I80/'Income Statement'!I11</f>
         <v>0.20669187471551</v>
       </c>
-      <c r="C36" s="863" t="n">
+      <c r="C36" s="867" t="n">
         <v>0.13983212556253</v>
       </c>
-      <c r="D36" s="863" t="n">
+      <c r="D36" s="867" t="n">
         <v>0.240698731755984</v>
       </c>
-      <c r="E36" s="863" t="n">
+      <c r="E36" s="867" t="n">
         <v>0.20669187471551</v>
       </c>
-      <c r="F36" s="864" t="n">
+      <c r="F36" s="868" t="n">
         <v>0.20669187471551</v>
       </c>
       <c r="G36" s="2"/>
@@ -12911,20 +12929,20 @@
       <c r="A37" s="18" t="s">
         <v>740</v>
       </c>
-      <c r="B37" s="859" t="n">
+      <c r="B37" s="863" t="n">
         <f aca="false">'Income Statement'!I78/1000000</f>
         <v>13.3741460043913</v>
       </c>
-      <c r="C37" s="860" t="n">
+      <c r="C37" s="864" t="n">
         <v>-0.188144670982913</v>
       </c>
-      <c r="D37" s="860" t="n">
+      <c r="D37" s="864" t="n">
         <v>25.7416742613056</v>
       </c>
-      <c r="E37" s="860" t="n">
+      <c r="E37" s="864" t="n">
         <v>16.1935208378721</v>
       </c>
-      <c r="F37" s="861" t="n">
+      <c r="F37" s="865" t="n">
         <v>12.6693022960211</v>
       </c>
       <c r="G37" s="2"/>
@@ -12940,20 +12958,20 @@
       <c r="A38" s="18" t="s">
         <v>741</v>
       </c>
-      <c r="B38" s="859" t="n">
+      <c r="B38" s="863" t="n">
         <f aca="false">SUM(DCF!C10:G10)/1000000</f>
         <v>-53.9371425360351</v>
       </c>
-      <c r="C38" s="860" t="n">
+      <c r="C38" s="864" t="n">
         <v>-57.6325593720804</v>
       </c>
-      <c r="D38" s="860" t="n">
+      <c r="D38" s="864" t="n">
         <v>-49.3917978554204</v>
       </c>
-      <c r="E38" s="860" t="n">
+      <c r="E38" s="864" t="n">
         <v>-53.9371425360351</v>
       </c>
-      <c r="F38" s="861" t="n">
+      <c r="F38" s="865" t="n">
         <v>-53.9371425360351</v>
       </c>
       <c r="G38" s="2"/>
@@ -12969,20 +12987,20 @@
       <c r="A39" s="18" t="s">
         <v>742</v>
       </c>
-      <c r="B39" s="859" t="n">
+      <c r="B39" s="863" t="n">
         <f aca="false">'Pro Forma'!B61/1000000</f>
         <v>40.4646713598887</v>
       </c>
-      <c r="C39" s="860" t="n">
+      <c r="C39" s="864" t="n">
         <v>47.3094743775238</v>
       </c>
-      <c r="D39" s="860" t="n">
+      <c r="D39" s="864" t="n">
         <v>34.3242588002227</v>
       </c>
-      <c r="E39" s="860" t="n">
+      <c r="E39" s="864" t="n">
         <v>73.6277508567534</v>
       </c>
-      <c r="F39" s="861" t="n">
+      <c r="F39" s="865" t="n">
         <v>33.9174564688055</v>
       </c>
       <c r="G39" s="2"/>
@@ -12998,20 +13016,20 @@
       <c r="A40" s="18" t="s">
         <v>743</v>
       </c>
-      <c r="B40" s="859" t="n">
+      <c r="B40" s="863" t="n">
         <f aca="false">SUM(Drivers!F125:J125)/1000000</f>
         <v>39.1579837983445</v>
       </c>
-      <c r="C40" s="860" t="n">
+      <c r="C40" s="864" t="n">
         <v>31.4016790921057</v>
       </c>
-      <c r="D40" s="860" t="n">
+      <c r="D40" s="864" t="n">
         <v>44.8558406219516</v>
       </c>
-      <c r="E40" s="860" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" s="861" t="n">
+      <c r="E40" s="864" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="865" t="n">
         <v>48.9474797479307</v>
       </c>
       <c r="G40" s="2"/>
@@ -13027,20 +13045,20 @@
       <c r="A41" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="B41" s="862" t="n">
+      <c r="B41" s="866" t="n">
         <f aca="false">'Discount rate'!E4</f>
         <v>0.141309839519679</v>
       </c>
-      <c r="C41" s="863" t="n">
+      <c r="C41" s="867" t="n">
         <v>0.140795536109349</v>
       </c>
-      <c r="D41" s="863" t="n">
+      <c r="D41" s="867" t="n">
         <v>0.14166079659066</v>
       </c>
-      <c r="E41" s="863" t="n">
+      <c r="E41" s="867" t="n">
         <v>0.136668124116301</v>
       </c>
-      <c r="F41" s="864" t="n">
+      <c r="F41" s="868" t="n">
         <v>0.142347620348559</v>
       </c>
       <c r="G41" s="2"/>
@@ -13056,20 +13074,20 @@
       <c r="A42" s="18" t="s">
         <v>744</v>
       </c>
-      <c r="B42" s="859" t="n">
+      <c r="B42" s="863" t="n">
         <f aca="false">B5</f>
         <v>22.9947614067526</v>
       </c>
-      <c r="C42" s="860" t="n">
+      <c r="C42" s="864" t="n">
         <v>-60.2877610097098</v>
       </c>
-      <c r="D42" s="860" t="n">
+      <c r="D42" s="864" t="n">
         <v>99.8206222064367</v>
       </c>
-      <c r="E42" s="860" t="n">
+      <c r="E42" s="864" t="n">
         <v>27.2563852914441</v>
       </c>
-      <c r="F42" s="861" t="n">
+      <c r="F42" s="865" t="n">
         <v>22.1075648881229</v>
       </c>
       <c r="G42" s="2"/>
@@ -13085,20 +13103,20 @@
       <c r="A43" s="18" t="s">
         <v>745</v>
       </c>
-      <c r="B43" s="859" t="n">
+      <c r="B43" s="863" t="n">
         <f aca="false">B6</f>
         <v>28.1685006370529</v>
       </c>
-      <c r="C43" s="860" t="n">
+      <c r="C43" s="864" t="n">
         <v>-27.1869051180712</v>
       </c>
-      <c r="D43" s="860" t="n">
+      <c r="D43" s="864" t="n">
         <v>77.9063327224381</v>
       </c>
-      <c r="E43" s="860" t="n">
+      <c r="E43" s="864" t="n">
         <v>7.89790782077882</v>
       </c>
-      <c r="F43" s="861" t="n">
+      <c r="F43" s="865" t="n">
         <v>31.8861460935203</v>
       </c>
       <c r="G43" s="2"/>
@@ -13114,20 +13132,20 @@
       <c r="A44" s="18" t="s">
         <v>746</v>
       </c>
-      <c r="B44" s="859" t="n">
+      <c r="B44" s="863" t="n">
         <f aca="false">B8</f>
         <v>26.0074983564468</v>
       </c>
-      <c r="C44" s="860" t="n">
+      <c r="C44" s="864" t="n">
         <v>-29.4476729121878</v>
       </c>
-      <c r="D44" s="860" t="n">
+      <c r="D44" s="864" t="n">
         <v>76.6329755104745</v>
       </c>
-      <c r="E44" s="860" t="n">
+      <c r="E44" s="864" t="n">
         <v>19.6039107838137</v>
       </c>
-      <c r="F44" s="861" t="n">
+      <c r="F44" s="865" t="n">
         <v>27.1396779315818</v>
       </c>
       <c r="G44" s="2"/>
@@ -13143,20 +13161,20 @@
       <c r="A45" s="18" t="s">
         <v>747</v>
       </c>
-      <c r="B45" s="862" t="n">
+      <c r="B45" s="866" t="n">
         <f aca="false">E8</f>
         <v>0.608746059178877</v>
       </c>
-      <c r="C45" s="863" t="s">
+      <c r="C45" s="867" t="s">
         <v>748</v>
       </c>
-      <c r="D45" s="863" t="n">
+      <c r="D45" s="867" t="n">
         <v>0.309346740782215</v>
       </c>
-      <c r="E45" s="863" t="n">
+      <c r="E45" s="867" t="n">
         <v>0.789729042271154</v>
       </c>
-      <c r="F45" s="864" t="n">
+      <c r="F45" s="868" t="n">
         <v>0.555503575493552</v>
       </c>
       <c r="G45" s="2"/>
@@ -13169,23 +13187,23 @@
       <c r="N45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="813" t="s">
+      <c r="A46" s="817" t="s">
         <v>749</v>
       </c>
-      <c r="B46" s="865" t="n">
+      <c r="B46" s="869" t="n">
         <f aca="false">IF(B8&lt;=0,"n.m.",1-E8)</f>
         <v>0.391253940821123</v>
       </c>
-      <c r="C46" s="866" t="s">
+      <c r="C46" s="870" t="s">
         <v>748</v>
       </c>
-      <c r="D46" s="866" t="n">
+      <c r="D46" s="870" t="n">
         <v>0.690653259217785</v>
       </c>
-      <c r="E46" s="866" t="n">
+      <c r="E46" s="870" t="n">
         <v>0.210270957728846</v>
       </c>
-      <c r="F46" s="867" t="n">
+      <c r="F46" s="871" t="n">
         <v>0.444496424506448</v>
       </c>
       <c r="G46" s="2"/>
@@ -13230,7 +13248,7 @@
       <c r="N48" s="2"/>
     </row>
     <row r="49" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="808" t="s">
+      <c r="A49" s="812" t="s">
         <v>750</v>
       </c>
       <c r="B49" s="2"/>
@@ -13266,396 +13284,396 @@
       <c r="N50" s="2"/>
     </row>
     <row r="51" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="827" t="s">
+      <c r="A51" s="831" t="s">
         <v>752</v>
       </c>
-      <c r="B51" s="827" t="s">
+      <c r="B51" s="831" t="s">
         <v>753</v>
       </c>
-      <c r="C51" s="827" t="s">
+      <c r="C51" s="831" t="s">
         <v>754</v>
       </c>
-      <c r="D51" s="827" t="s">
+      <c r="D51" s="831" t="s">
         <v>755</v>
       </c>
-      <c r="E51" s="827" t="s">
+      <c r="E51" s="831" t="s">
         <v>756</v>
       </c>
-      <c r="F51" s="827" t="s">
+      <c r="F51" s="831" t="s">
         <v>757</v>
       </c>
-      <c r="G51" s="827" t="s">
+      <c r="G51" s="831" t="s">
         <v>758</v>
       </c>
-      <c r="H51" s="827" t="s">
+      <c r="H51" s="831" t="s">
         <v>759</v>
       </c>
-      <c r="I51" s="827" t="s">
+      <c r="I51" s="831" t="s">
         <v>760</v>
       </c>
-      <c r="J51" s="827" t="s">
+      <c r="J51" s="831" t="s">
         <v>761</v>
       </c>
-      <c r="K51" s="827" t="s">
+      <c r="K51" s="831" t="s">
         <v>762</v>
       </c>
-      <c r="L51" s="827" t="s">
+      <c r="L51" s="831" t="s">
         <v>763</v>
       </c>
-      <c r="M51" s="827" t="s">
+      <c r="M51" s="831" t="s">
         <v>764</v>
       </c>
-      <c r="N51" s="827" t="s">
+      <c r="N51" s="831" t="s">
         <v>765</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="868" t="s">
+      <c r="A52" s="872" t="s">
         <v>766</v>
       </c>
-      <c r="B52" s="869" t="n">
+      <c r="B52" s="873" t="n">
         <v>26.0074983564468</v>
       </c>
-      <c r="C52" s="869" t="n">
+      <c r="C52" s="873" t="n">
         <v>26.0074983564468</v>
       </c>
-      <c r="D52" s="870" t="n">
-        <v>0</v>
-      </c>
-      <c r="E52" s="870" t="n">
-        <v>0</v>
-      </c>
-      <c r="F52" s="869" t="n">
+      <c r="D52" s="874" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="874" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="873" t="n">
         <v>22.9947614067526</v>
       </c>
-      <c r="G52" s="869" t="n">
+      <c r="G52" s="873" t="n">
         <v>22.9947614067526</v>
       </c>
-      <c r="H52" s="869" t="n">
+      <c r="H52" s="873" t="n">
         <v>28.1685006370529</v>
       </c>
-      <c r="I52" s="869" t="n">
+      <c r="I52" s="873" t="n">
         <v>28.1685006370529</v>
       </c>
-      <c r="J52" s="869" t="n">
+      <c r="J52" s="873" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="K52" s="869" t="n">
+      <c r="K52" s="873" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="L52" s="869" t="n">
+      <c r="L52" s="873" t="n">
         <v>13.3741460043913</v>
       </c>
-      <c r="M52" s="869" t="n">
+      <c r="M52" s="873" t="n">
         <v>13.3741460043913</v>
       </c>
       <c r="N52" s="465"/>
     </row>
     <row r="53" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="779" t="s">
+      <c r="A53" s="783" t="s">
         <v>767</v>
       </c>
-      <c r="B53" s="860" t="n">
+      <c r="B53" s="864" t="n">
         <v>-1.96554644080494</v>
       </c>
-      <c r="C53" s="860" t="n">
+      <c r="C53" s="864" t="n">
         <v>59.9233919574906</v>
       </c>
-      <c r="D53" s="871" t="n">
+      <c r="D53" s="875" t="n">
         <v>-27.9730447972517</v>
       </c>
-      <c r="E53" s="871" t="n">
+      <c r="E53" s="875" t="n">
         <v>33.9158936010438</v>
       </c>
-      <c r="F53" s="860" t="n">
+      <c r="F53" s="864" t="n">
         <v>-20.312298248552</v>
       </c>
-      <c r="G53" s="860" t="n">
+      <c r="G53" s="864" t="n">
         <v>75.8171447729884</v>
       </c>
-      <c r="H53" s="860" t="n">
+      <c r="H53" s="864" t="n">
         <v>1.5429482992283</v>
       </c>
-      <c r="I53" s="860" t="n">
+      <c r="I53" s="864" t="n">
         <v>60.1358512734266</v>
       </c>
-      <c r="J53" s="860" t="n">
+      <c r="J53" s="864" t="n">
         <v>142.915944245401</v>
       </c>
-      <c r="K53" s="860" t="n">
+      <c r="K53" s="864" t="n">
         <v>221.944073516401</v>
       </c>
-      <c r="L53" s="860" t="n">
+      <c r="L53" s="864" t="n">
         <v>5.87980417282567</v>
       </c>
-      <c r="M53" s="860" t="n">
+      <c r="M53" s="864" t="n">
         <v>22.5009174886484</v>
       </c>
-      <c r="N53" s="777" t="s">
+      <c r="N53" s="781" t="s">
         <v>768</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="779" t="s">
+      <c r="A54" s="783" t="s">
         <v>769</v>
       </c>
-      <c r="B54" s="860" t="n">
+      <c r="B54" s="864" t="n">
         <v>19.3741392318594</v>
       </c>
-      <c r="C54" s="860" t="n">
+      <c r="C54" s="864" t="n">
         <v>32.925863476306</v>
       </c>
-      <c r="D54" s="871" t="n">
+      <c r="D54" s="875" t="n">
         <v>-6.63335912458738</v>
       </c>
-      <c r="E54" s="871" t="n">
+      <c r="E54" s="875" t="n">
         <v>6.91836511985926</v>
       </c>
-      <c r="F54" s="860" t="n">
+      <c r="F54" s="864" t="n">
         <v>12.7144146114538</v>
       </c>
-      <c r="G54" s="860" t="n">
+      <c r="G54" s="864" t="n">
         <v>33.7306141755154</v>
       </c>
-      <c r="H54" s="860" t="n">
+      <c r="H54" s="864" t="n">
         <v>21.8654496208832</v>
       </c>
-      <c r="I54" s="860" t="n">
+      <c r="I54" s="864" t="n">
         <v>34.7285606679383</v>
       </c>
-      <c r="J54" s="860" t="n">
+      <c r="J54" s="864" t="n">
         <v>170.288003540798</v>
       </c>
-      <c r="K54" s="860" t="n">
+      <c r="K54" s="864" t="n">
         <v>187.840751522138</v>
       </c>
-      <c r="L54" s="860" t="n">
+      <c r="L54" s="864" t="n">
         <v>11.5840438628959</v>
       </c>
-      <c r="M54" s="860" t="n">
+      <c r="M54" s="864" t="n">
         <v>15.2430370919031</v>
       </c>
-      <c r="N54" s="777" t="s">
+      <c r="N54" s="781" t="s">
         <v>770</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="779" t="s">
+      <c r="A55" s="783" t="s">
         <v>771</v>
       </c>
-      <c r="B55" s="860" t="n">
+      <c r="B55" s="864" t="n">
         <v>16.991754813111</v>
       </c>
-      <c r="C55" s="860" t="n">
+      <c r="C55" s="864" t="n">
         <v>35.0041933420044</v>
       </c>
-      <c r="D55" s="871" t="n">
+      <c r="D55" s="875" t="n">
         <v>-9.01574354333572</v>
       </c>
-      <c r="E55" s="871" t="n">
+      <c r="E55" s="875" t="n">
         <v>8.99669498555765</v>
       </c>
-      <c r="F55" s="860" t="n">
+      <c r="F55" s="864" t="n">
         <v>10.5311256827794</v>
       </c>
-      <c r="G55" s="860" t="n">
+      <c r="G55" s="864" t="n">
         <v>35.4166973517185</v>
       </c>
-      <c r="H55" s="860" t="n">
+      <c r="H55" s="864" t="n">
         <v>18.0927775026868</v>
       </c>
-      <c r="I55" s="860" t="n">
+      <c r="I55" s="864" t="n">
         <v>38.2383021559811</v>
       </c>
-      <c r="J55" s="860" t="n">
+      <c r="J55" s="864" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="K55" s="860" t="n">
+      <c r="K55" s="864" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="L55" s="860" t="n">
+      <c r="L55" s="864" t="n">
         <v>11.9430083321538</v>
       </c>
-      <c r="M55" s="860" t="n">
+      <c r="M55" s="864" t="n">
         <v>14.8052836766288</v>
       </c>
-      <c r="N55" s="777" t="s">
+      <c r="N55" s="781" t="s">
         <v>772</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="779" t="s">
+      <c r="A56" s="783" t="s">
         <v>773</v>
       </c>
-      <c r="B56" s="860" t="n">
+      <c r="B56" s="864" t="n">
         <v>14.866604664728</v>
       </c>
-      <c r="C56" s="860" t="n">
+      <c r="C56" s="864" t="n">
         <v>37.1221726922844</v>
       </c>
-      <c r="D56" s="871" t="n">
+      <c r="D56" s="875" t="n">
         <v>-11.1408936917188</v>
       </c>
-      <c r="E56" s="871" t="n">
+      <c r="E56" s="875" t="n">
         <v>11.1146743358376</v>
       </c>
-      <c r="F56" s="860" t="n">
+      <c r="F56" s="864" t="n">
         <v>7.46763841904257</v>
       </c>
-      <c r="G56" s="860" t="n">
+      <c r="G56" s="864" t="n">
         <v>38.4644591134795</v>
       </c>
-      <c r="H56" s="860" t="n">
+      <c r="H56" s="864" t="n">
         <v>15.8433893954659</v>
       </c>
-      <c r="I56" s="860" t="n">
+      <c r="I56" s="864" t="n">
         <v>40.4854887699201</v>
       </c>
-      <c r="J56" s="860" t="n">
+      <c r="J56" s="864" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="K56" s="860" t="n">
+      <c r="K56" s="864" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="L56" s="860" t="n">
+      <c r="L56" s="864" t="n">
         <v>11.5422897839273</v>
       </c>
-      <c r="M56" s="860" t="n">
+      <c r="M56" s="864" t="n">
         <v>15.2060022248553</v>
       </c>
-      <c r="N56" s="777" t="s">
+      <c r="N56" s="781" t="s">
         <v>774</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="779" t="s">
+      <c r="A57" s="783" t="s">
         <v>775</v>
       </c>
-      <c r="B57" s="860" t="n">
+      <c r="B57" s="864" t="n">
         <v>21.6260696287263</v>
       </c>
-      <c r="C57" s="860" t="n">
+      <c r="C57" s="864" t="n">
         <v>31.198177127893</v>
       </c>
-      <c r="D57" s="871" t="n">
+      <c r="D57" s="875" t="n">
         <v>-4.38142872772042</v>
       </c>
-      <c r="E57" s="871" t="n">
+      <c r="E57" s="875" t="n">
         <v>5.19067877144628</v>
       </c>
-      <c r="F57" s="860" t="n">
+      <c r="F57" s="864" t="n">
         <v>15.7283531504832</v>
       </c>
-      <c r="G57" s="860" t="n">
+      <c r="G57" s="864" t="n">
         <v>32.1506176525824</v>
       </c>
-      <c r="H57" s="860" t="n">
+      <c r="H57" s="864" t="n">
         <v>24.4813370740213</v>
       </c>
-      <c r="I57" s="860" t="n">
+      <c r="I57" s="864" t="n">
         <v>31.9893413198388</v>
       </c>
-      <c r="J57" s="860" t="n">
+      <c r="J57" s="864" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="K57" s="860" t="n">
+      <c r="K57" s="864" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="L57" s="860" t="n">
+      <c r="L57" s="864" t="n">
         <v>13.0793877210432</v>
       </c>
-      <c r="M57" s="860" t="n">
+      <c r="M57" s="864" t="n">
         <v>13.6689042877394</v>
       </c>
-      <c r="N57" s="777" t="s">
+      <c r="N57" s="781" t="s">
         <v>776</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="779" t="s">
+      <c r="A58" s="783" t="s">
         <v>777</v>
       </c>
-      <c r="B58" s="860" t="n">
+      <c r="B58" s="864" t="n">
         <v>21.7559343776643</v>
       </c>
-      <c r="C58" s="860" t="n">
+      <c r="C58" s="864" t="n">
         <v>31.259573190541</v>
       </c>
-      <c r="D58" s="871" t="n">
+      <c r="D58" s="875" t="n">
         <v>-4.25156397878245</v>
       </c>
-      <c r="E58" s="871" t="n">
+      <c r="E58" s="875" t="n">
         <v>5.25207483409425</v>
       </c>
-      <c r="F58" s="860" t="n">
+      <c r="F58" s="864" t="n">
         <v>14.9782604607731</v>
       </c>
-      <c r="G58" s="860" t="n">
+      <c r="G58" s="864" t="n">
         <v>33.38364800817</v>
       </c>
-      <c r="H58" s="860" t="n">
+      <c r="H58" s="864" t="n">
         <v>25.5560916360763</v>
       </c>
-      <c r="I58" s="860" t="n">
+      <c r="I58" s="864" t="n">
         <v>30.9098011208712</v>
       </c>
-      <c r="J58" s="860" t="n">
+      <c r="J58" s="864" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="K58" s="860" t="n">
+      <c r="K58" s="864" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="L58" s="860" t="n">
+      <c r="L58" s="864" t="n">
         <v>13.3741460043913</v>
       </c>
-      <c r="M58" s="860" t="n">
+      <c r="M58" s="864" t="n">
         <v>13.3741460043913</v>
       </c>
-      <c r="N58" s="777" t="s">
+      <c r="N58" s="781" t="s">
         <v>778</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="782" t="s">
+      <c r="A59" s="786" t="s">
         <v>779</v>
       </c>
-      <c r="B59" s="872" t="n">
+      <c r="B59" s="876" t="n">
         <v>26.0074983564468</v>
       </c>
-      <c r="C59" s="872" t="n">
+      <c r="C59" s="876" t="n">
         <v>29.4860145263927</v>
       </c>
-      <c r="D59" s="873" t="n">
-        <v>0</v>
-      </c>
-      <c r="E59" s="873" t="n">
+      <c r="D59" s="877" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="877" t="n">
         <v>3.47851616994597</v>
       </c>
-      <c r="F59" s="872" t="n">
+      <c r="F59" s="876" t="n">
         <v>22.9947614067526</v>
       </c>
-      <c r="G59" s="872" t="n">
+      <c r="G59" s="876" t="n">
         <v>26.6177473961008</v>
       </c>
-      <c r="H59" s="872" t="n">
+      <c r="H59" s="876" t="n">
         <v>28.1685006370529</v>
       </c>
-      <c r="I59" s="872" t="n">
+      <c r="I59" s="876" t="n">
         <v>33.2418050725696</v>
       </c>
-      <c r="J59" s="872" t="n">
+      <c r="J59" s="876" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="K59" s="872" t="n">
+      <c r="K59" s="876" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="L59" s="872" t="n">
+      <c r="L59" s="876" t="n">
         <v>13.3741460043913</v>
       </c>
-      <c r="M59" s="872" t="n">
+      <c r="M59" s="876" t="n">
         <v>13.3741460043913</v>
       </c>
-      <c r="N59" s="800" t="s">
+      <c r="N59" s="804" t="s">
         <v>780</v>
       </c>
     </row>
@@ -13688,7 +13706,7 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="786" t="s">
+      <c r="A1" s="790" t="s">
         <v>781</v>
       </c>
       <c r="B1" s="226"/>
@@ -13726,165 +13744,165 @@
       <c r="F4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="809" t="s">
+      <c r="A5" s="813" t="s">
         <v>784</v>
       </c>
-      <c r="B5" s="874" t="n">
+      <c r="B5" s="878" t="n">
         <f aca="false">Assumption!$B$14+(-0.02)</f>
         <v>0.03</v>
       </c>
-      <c r="C5" s="874" t="n">
+      <c r="C5" s="878" t="n">
         <f aca="false">Assumption!$B$14+(-0.01)</f>
         <v>0.04</v>
       </c>
-      <c r="D5" s="874" t="n">
+      <c r="D5" s="878" t="n">
         <f aca="false">Assumption!$B$14+(0)</f>
         <v>0.05</v>
       </c>
-      <c r="E5" s="874" t="n">
+      <c r="E5" s="878" t="n">
         <f aca="false">Assumption!$B$14+(0.01)</f>
         <v>0.06</v>
       </c>
-      <c r="F5" s="875" t="n">
+      <c r="F5" s="879" t="n">
         <f aca="false">Assumption!$B$14+(0.02)</f>
         <v>0.07</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="876" t="n">
+      <c r="A6" s="880" t="n">
         <f aca="false">Assumption!$B$16+(-0.02)</f>
         <v>0.121309839519679</v>
       </c>
-      <c r="B6" s="877" t="n">
+      <c r="B6" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A6)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+B$5)*(1-B$5/Assumption!$B$17)/($A6-B$5))/(1+$A6)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>43.6632784026025</v>
       </c>
-      <c r="C6" s="877" t="n">
+      <c r="C6" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A6)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+C$5)*(1-C$5/Assumption!$B$17)/($A6-C$5))/(1+$A6)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>44.7004899324069</v>
       </c>
-      <c r="D6" s="877" t="n">
+      <c r="D6" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A6)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+D$5)*(1-D$5/Assumption!$B$17)/($A6-D$5))/(1+$A6)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>45.8000450628265</v>
       </c>
-      <c r="E6" s="877" t="n">
+      <c r="E6" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A6)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+E$5)*(1-E$5/Assumption!$B$17)/($A6-E$5))/(1+$A6)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>46.9924496316371</v>
       </c>
-      <c r="F6" s="878" t="n">
+      <c r="F6" s="882" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A6)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+F$5)*(1-F$5/Assumption!$B$17)/($A6-F$5))/(1+$A6)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>48.3319911434931</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="876" t="n">
+      <c r="A7" s="880" t="n">
         <f aca="false">Assumption!$B$16+(-0.01)</f>
         <v>0.131309839519679</v>
       </c>
-      <c r="B7" s="877" t="n">
+      <c r="B7" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A7)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+B$5)*(1-B$5/Assumption!$B$17)/($A7-B$5))/(1+$A7)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>33.051201020086</v>
       </c>
-      <c r="C7" s="877" t="n">
+      <c r="C7" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A7)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+C$5)*(1-C$5/Assumption!$B$17)/($A7-C$5))/(1+$A7)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>33.0495622160443</v>
       </c>
-      <c r="D7" s="877" t="n">
+      <c r="D7" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A7)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+D$5)*(1-D$5/Assumption!$B$17)/($A7-D$5))/(1+$A7)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>32.8544936419302</v>
       </c>
-      <c r="E7" s="877" t="n">
+      <c r="E7" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A7)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+E$5)*(1-E$5/Assumption!$B$17)/($A7-E$5))/(1+$A7)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>32.3846195277062</v>
       </c>
-      <c r="F7" s="878" t="n">
+      <c r="F7" s="882" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A7)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+F$5)*(1-F$5/Assumption!$B$17)/($A7-F$5))/(1+$A7)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>31.5054726121973</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="876" t="n">
+      <c r="A8" s="880" t="n">
         <f aca="false">Assumption!$B$16+(0)</f>
         <v>0.141309839519679</v>
       </c>
-      <c r="B8" s="877" t="n">
+      <c r="B8" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A8)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+B$5)*(1-B$5/Assumption!$B$17)/($A8-B$5))/(1+$A8)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>24.5717305276797</v>
       </c>
-      <c r="C8" s="877" t="n">
+      <c r="C8" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A8)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+C$5)*(1-C$5/Assumption!$B$17)/($A8-C$5))/(1+$A8)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>23.9356915628625</v>
       </c>
-      <c r="D8" s="879" t="n">
+      <c r="D8" s="883" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A8)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+D$5)*(1-D$5/Assumption!$B$17)/($A8-D$5))/(1+$A8)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>22.9947614067526</v>
       </c>
-      <c r="E8" s="877" t="n">
+      <c r="E8" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A8)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+E$5)*(1-E$5/Assumption!$B$17)/($A8-E$5))/(1+$A8)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>21.6364476993502</v>
       </c>
-      <c r="F8" s="878" t="n">
+      <c r="F8" s="882" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A8)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+F$5)*(1-F$5/Assumption!$B$17)/($A8-F$5))/(1+$A8)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>19.6851574702728</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="876" t="n">
+      <c r="A9" s="880" t="n">
         <f aca="false">Assumption!$B$16+(0.01)</f>
         <v>0.151309839519679</v>
       </c>
-      <c r="B9" s="877" t="n">
+      <c r="B9" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A9)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+B$5)*(1-B$5/Assumption!$B$17)/($A9-B$5))/(1+$A9)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>17.6880241299027</v>
       </c>
-      <c r="C9" s="877" t="n">
+      <c r="C9" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A9)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+C$5)*(1-C$5/Assumption!$B$17)/($A9-C$5))/(1+$A9)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>16.6653784440411</v>
       </c>
-      <c r="D9" s="877" t="n">
+      <c r="D9" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A9)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+D$5)*(1-D$5/Assumption!$B$17)/($A9-D$5))/(1+$A9)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>15.2970464524351</v>
       </c>
-      <c r="E9" s="877" t="n">
+      <c r="E9" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A9)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+E$5)*(1-E$5/Assumption!$B$17)/($A9-E$5))/(1+$A9)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>13.4694523430269</v>
       </c>
-      <c r="F9" s="878" t="n">
+      <c r="F9" s="882" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A9)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+F$5)*(1-F$5/Assumption!$B$17)/($A9-F$5))/(1+$A9)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>11.0131472075974</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="876" t="n">
+      <c r="A10" s="880" t="n">
         <f aca="false">Assumption!$B$16+(0.02)</f>
         <v>0.161309839519679</v>
       </c>
-      <c r="B10" s="877" t="n">
+      <c r="B10" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A10)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+B$5)*(1-B$5/Assumption!$B$17)/($A10-B$5))/(1+$A10)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>12.0272360755729</v>
       </c>
-      <c r="C10" s="877" t="n">
+      <c r="C10" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A10)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+C$5)*(1-C$5/Assumption!$B$17)/($A10-C$5))/(1+$A10)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>10.7742603486568</v>
       </c>
-      <c r="D10" s="877" t="n">
+      <c r="D10" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A10)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+D$5)*(1-D$5/Assumption!$B$17)/($A10-D$5))/(1+$A10)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>9.16999241407187</v>
       </c>
-      <c r="E10" s="877" t="n">
+      <c r="E10" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A10)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+E$5)*(1-E$5/Assumption!$B$17)/($A10-E$5))/(1+$A10)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>7.11040717139316</v>
       </c>
-      <c r="F10" s="878" t="n">
+      <c r="F10" s="882" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A10)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+F$5)*(1-F$5/Assumption!$B$17)/($A10-F$5))/(1+$A10)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>4.44590935997118</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="821" t="s">
+      <c r="A11" s="825" t="s">
         <v>785</v>
       </c>
-      <c r="B11" s="880" t="n">
+      <c r="B11" s="884" t="n">
         <f aca="false">ROUND(D8-DCF!B22/1000000,6)</f>
         <v>0</v>
       </c>
@@ -13912,155 +13930,155 @@
       <c r="F13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="809" t="s">
+      <c r="A14" s="813" t="s">
         <v>787</v>
       </c>
-      <c r="B14" s="881" t="n">
+      <c r="B14" s="885" t="n">
         <v>-0.3</v>
       </c>
-      <c r="C14" s="881" t="n">
+      <c r="C14" s="885" t="n">
         <v>-0.15</v>
       </c>
-      <c r="D14" s="881" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="881" t="n">
+      <c r="D14" s="885" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="885" t="n">
         <v>0.15</v>
       </c>
-      <c r="F14" s="882" t="n">
+      <c r="F14" s="886" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="883" t="n">
+      <c r="A15" s="887" t="n">
         <v>0.3</v>
       </c>
-      <c r="B15" s="877" t="n">
+      <c r="B15" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+B$14)*(1-$A15)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>15.5857524376136</v>
       </c>
-      <c r="C15" s="877" t="n">
+      <c r="C15" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+C$14)*(1-$A15)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>27.5965575370784</v>
       </c>
-      <c r="D15" s="877" t="n">
+      <c r="D15" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+D$14)*(1-$A15)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>39.6073626365432</v>
       </c>
-      <c r="E15" s="877" t="n">
+      <c r="E15" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+E$14)*(1-$A15)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>51.618167736008</v>
       </c>
-      <c r="F15" s="878" t="n">
+      <c r="F15" s="882" t="n">
         <f aca="false">(VCM!$E$4*(1+F$14)*(1-$A15)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>63.6289728354728</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="883" t="n">
+      <c r="A16" s="887" t="n">
         <v>0.35</v>
       </c>
-      <c r="B16" s="877" t="n">
+      <c r="B16" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+B$14)*(1-$A16)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>11.582150737792</v>
       </c>
-      <c r="C16" s="877" t="n">
+      <c r="C16" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+C$14)*(1-$A16)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>22.735041187295</v>
       </c>
-      <c r="D16" s="877" t="n">
+      <c r="D16" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+D$14)*(1-$A16)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>33.8879316367981</v>
       </c>
-      <c r="E16" s="877" t="n">
+      <c r="E16" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+E$14)*(1-$A16)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>45.0408220863011</v>
       </c>
-      <c r="F16" s="878" t="n">
+      <c r="F16" s="882" t="n">
         <f aca="false">(VCM!$E$4*(1+F$14)*(1-$A16)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>56.1937125358041</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="883" t="n">
+      <c r="A17" s="887" t="n">
         <v>0.4</v>
       </c>
-      <c r="B17" s="877" t="n">
+      <c r="B17" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+B$14)*(1-$A17)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>7.57854903797042</v>
       </c>
-      <c r="C17" s="877" t="n">
+      <c r="C17" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+C$14)*(1-$A17)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>17.8735248375117</v>
       </c>
-      <c r="D17" s="879" t="n">
+      <c r="D17" s="883" t="n">
         <f aca="false">(VCM!$E$4*(1+D$14)*(1-$A17)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>28.1685006370529</v>
       </c>
-      <c r="E17" s="877" t="n">
+      <c r="E17" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+E$14)*(1-$A17)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>38.4634764365942</v>
       </c>
-      <c r="F17" s="878" t="n">
+      <c r="F17" s="882" t="n">
         <f aca="false">(VCM!$E$4*(1+F$14)*(1-$A17)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>48.7584522361354</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="883" t="n">
+      <c r="A18" s="887" t="n">
         <v>0.45</v>
       </c>
-      <c r="B18" s="877" t="n">
+      <c r="B18" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+B$14)*(1-$A18)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>3.57494733814883</v>
       </c>
-      <c r="C18" s="877" t="n">
+      <c r="C18" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+C$14)*(1-$A18)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>13.0120084877283</v>
       </c>
-      <c r="D18" s="877" t="n">
+      <c r="D18" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+D$14)*(1-$A18)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>22.4490696373078</v>
       </c>
-      <c r="E18" s="877" t="n">
+      <c r="E18" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+E$14)*(1-$A18)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>31.8861307868873</v>
       </c>
-      <c r="F18" s="878" t="n">
+      <c r="F18" s="882" t="n">
         <f aca="false">(VCM!$E$4*(1+F$14)*(1-$A18)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>41.3231919364668</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="883" t="n">
+      <c r="A19" s="887" t="n">
         <v>0.5</v>
       </c>
-      <c r="B19" s="877" t="n">
+      <c r="B19" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+B$14)*(1-$A19)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>-0.428654361672774</v>
       </c>
-      <c r="C19" s="877" t="n">
+      <c r="C19" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+C$14)*(1-$A19)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>8.15049213794494</v>
       </c>
-      <c r="D19" s="877" t="n">
+      <c r="D19" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+D$14)*(1-$A19)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>16.7296386375626</v>
       </c>
-      <c r="E19" s="877" t="n">
+      <c r="E19" s="881" t="n">
         <f aca="false">(VCM!$E$4*(1+E$14)*(1-$A19)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>25.3087851371804</v>
       </c>
-      <c r="F19" s="878" t="n">
+      <c r="F19" s="882" t="n">
         <f aca="false">(VCM!$E$4*(1+F$14)*(1-$A19)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>33.8879316367981</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="821" t="s">
+      <c r="A20" s="825" t="s">
         <v>788</v>
       </c>
-      <c r="B20" s="880" t="n">
+      <c r="B20" s="884" t="n">
         <f aca="false">ROUND(D17-VCM!E7/1000000,6)</f>
         <v>0</v>
       </c>
@@ -14088,156 +14106,156 @@
       <c r="F22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="809" t="s">
+      <c r="A23" s="813" t="s">
         <v>790</v>
       </c>
-      <c r="B23" s="874" t="n">
+      <c r="B23" s="878" t="n">
         <f aca="false">Assumption!$B$17+(-0.04)</f>
         <v>0.0831158832517256</v>
       </c>
-      <c r="C23" s="874" t="n">
+      <c r="C23" s="878" t="n">
         <f aca="false">Assumption!$B$17+(-0.02)</f>
         <v>0.103115883251726</v>
       </c>
-      <c r="D23" s="874" t="n">
+      <c r="D23" s="878" t="n">
         <f aca="false">Assumption!$B$17+(0)</f>
         <v>0.123115883251726</v>
       </c>
-      <c r="E23" s="874" t="n">
+      <c r="E23" s="878" t="n">
         <f aca="false">Assumption!$B$17+(0.02)</f>
         <v>0.143115883251726</v>
       </c>
-      <c r="F23" s="875" t="n">
+      <c r="F23" s="879" t="n">
         <f aca="false">Assumption!$B$17+(0.04)</f>
         <v>0.163115883251726</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="876" t="n">
+      <c r="A24" s="880" t="n">
         <f aca="false">Assumption!$B$16+(-0.02)</f>
         <v>0.121309839519679</v>
       </c>
-      <c r="B24" s="877" t="n">
+      <c r="B24" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A24)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/B$23)/($A24-Assumption!$B$14))/(1+$A24)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>16.9262450704033</v>
       </c>
-      <c r="C24" s="877" t="n">
+      <c r="C24" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A24)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/C$23)/($A24-Assumption!$B$14))/(1+$A24)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>34.1632762473697</v>
       </c>
-      <c r="D24" s="877" t="n">
+      <c r="D24" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A24)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/D$23)/($A24-Assumption!$B$14))/(1+$A24)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>45.8000450628265</v>
       </c>
-      <c r="E24" s="877" t="n">
+      <c r="E24" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A24)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/E$23)/($A24-Assumption!$B$14))/(1+$A24)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>54.1844093090465</v>
       </c>
-      <c r="F24" s="878" t="n">
+      <c r="F24" s="882" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A24)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/F$23)/($A24-Assumption!$B$14))/(1+$A24)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>60.5127225860838</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="876" t="n">
+      <c r="A25" s="880" t="n">
         <f aca="false">Assumption!$B$16+(-0.01)</f>
         <v>0.131309839519679</v>
       </c>
-      <c r="B25" s="877" t="n">
+      <c r="B25" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A25)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/B$23)/($A25-Assumption!$B$14))/(1+$A25)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>8.46950312566897</v>
       </c>
-      <c r="C25" s="877" t="n">
+      <c r="C25" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A25)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/C$23)/($A25-Assumption!$B$14))/(1+$A25)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>23.026812585772</v>
       </c>
-      <c r="D25" s="877" t="n">
+      <c r="D25" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A25)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/D$23)/($A25-Assumption!$B$14))/(1+$A25)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>32.8544936419302</v>
       </c>
-      <c r="E25" s="877" t="n">
+      <c r="E25" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A25)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/E$23)/($A25-Assumption!$B$14))/(1+$A25)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>39.9353989153131</v>
       </c>
-      <c r="F25" s="878" t="n">
+      <c r="F25" s="882" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A25)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/F$23)/($A25-Assumption!$B$14))/(1+$A25)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>45.2798932071963</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="876" t="n">
+      <c r="A26" s="880" t="n">
         <f aca="false">Assumption!$B$16+(0)</f>
         <v>0.141309839519679</v>
       </c>
-      <c r="B26" s="877" t="n">
+      <c r="B26" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A26)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/B$23)/($A26-Assumption!$B$14))/(1+$A26)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>2.07750943539398</v>
       </c>
-      <c r="C26" s="877" t="n">
+      <c r="C26" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A26)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/C$23)/($A26-Assumption!$B$14))/(1+$A26)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>14.5646543370482</v>
       </c>
-      <c r="D26" s="879" t="n">
+      <c r="D26" s="883" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A26)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/D$23)/($A26-Assumption!$B$14))/(1+$A26)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>22.9947614067526</v>
       </c>
-      <c r="E26" s="877" t="n">
+      <c r="E26" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A26)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/E$23)/($A26-Assumption!$B$14))/(1+$A26)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>29.0687059379142</v>
       </c>
-      <c r="F26" s="878" t="n">
+      <c r="F26" s="882" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A26)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/F$23)/($A26-Assumption!$B$14))/(1+$A26)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>33.6531708647412</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="876" t="n">
+      <c r="A27" s="880" t="n">
         <f aca="false">Assumption!$B$16+(0.01)</f>
         <v>0.151309839519679</v>
       </c>
-      <c r="B27" s="877" t="n">
+      <c r="B27" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A27)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/B$23)/($A27-Assumption!$B$14))/(1+$A27)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>-2.86935038162652</v>
       </c>
-      <c r="C27" s="877" t="n">
+      <c r="C27" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A27)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/C$23)/($A27-Assumption!$B$14))/(1+$A27)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>7.9755937782705</v>
       </c>
-      <c r="D27" s="877" t="n">
+      <c r="D27" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A27)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/D$23)/($A27-Assumption!$B$14))/(1+$A27)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>15.2970464524351</v>
       </c>
-      <c r="E27" s="877" t="n">
+      <c r="E27" s="881" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A27)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/E$23)/($A27-Assumption!$B$14))/(1+$A27)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>20.5721986020697</v>
       </c>
-      <c r="F27" s="878" t="n">
+      <c r="F27" s="882" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A27)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/F$23)/($A27-Assumption!$B$14))/(1+$A27)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>24.5537545562942</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="884" t="n">
+      <c r="A28" s="888" t="n">
         <f aca="false">Assumption!$B$16+(0.02)</f>
         <v>0.161309839519679</v>
       </c>
-      <c r="B28" s="885" t="n">
+      <c r="B28" s="889" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A28)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/B$23)/($A28-Assumption!$B$14))/(1+$A28)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>-6.76765950913217</v>
       </c>
-      <c r="C28" s="885" t="n">
+      <c r="C28" s="889" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A28)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/C$23)/($A28-Assumption!$B$14))/(1+$A28)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>2.74677236890245</v>
       </c>
-      <c r="D28" s="885" t="n">
+      <c r="D28" s="889" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A28)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/D$23)/($A28-Assumption!$B$14))/(1+$A28)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>9.16999241407187</v>
       </c>
-      <c r="E28" s="885" t="n">
+      <c r="E28" s="889" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A28)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/E$23)/($A28-Assumption!$B$14))/(1+$A28)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>13.7979623726044</v>
       </c>
-      <c r="F28" s="886" t="n">
+      <c r="F28" s="890" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A28)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/F$23)/($A28-Assumption!$B$14))/(1+$A28)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
         <v>17.2910410216522</v>
       </c>
@@ -14572,11 +14590,11 @@
       <c r="A14" s="1" t="s">
         <v>804</v>
       </c>
-      <c r="B14" s="887" t="n">
+      <c r="B14" s="891" t="n">
         <f aca="false">Sensitivity!B11</f>
         <v>0</v>
       </c>
-      <c r="C14" s="887" t="n">
+      <c r="C14" s="891" t="n">
         <f aca="false">Sensitivity!B20</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Tiền mặt ròng tại t0 được phép âm; Multiples dùng tiền/nợ tại t0, thêm đối chiếu TTM
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018d4TrajAJ6BNPb7i8Se7c9
</commit_message>
<xml_diff>
--- a/AgriPack_Model_final.xlsx
+++ b/AgriPack_Model_final.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1027" uniqueCount="808">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1035" uniqueCount="817">
   <si>
     <t xml:space="preserve">Công ty Cổ phần AgriPack</t>
   </si>
@@ -1756,7 +1756,7 @@
     <t xml:space="preserve">Tỷ trọng giá trị cuối kỳ / EV</t>
   </si>
   <si>
-    <t xml:space="preserve">(+) Tiền mặt ước tính 30/09/2026 = tiền 31/12/2025 + 75% FCFF 2026 (≥ 0)</t>
+    <t xml:space="preserve">(+) Tiền mặt ròng ước tính 30/09/2026 = tiền 31/12/2025 + 75% FCFF 2026 (âm = thiếu hụt tài trợ tạm, coi như nợ)</t>
   </si>
   <si>
     <t xml:space="preserve">(−) Nợ vay 30/09/2026 (= 31/12/2025; không vay mới trong 2026)</t>
@@ -2068,10 +2068,10 @@
     <t xml:space="preserve">LNST chuẩn hóa 2025A</t>
   </si>
   <si>
-    <t xml:space="preserve">Tiền mặt 31/12/2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nợ vay 31/12/2025</t>
+    <t xml:space="preserve">Tiền mặt ròng tại t0 (30/09/2026, = DCF!B31)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nợ vay tại t0 (30/09/2026, = DCF!B32)</t>
   </si>
   <si>
     <t xml:space="preserve">Chiết khấu thiếu thanh khoản &amp; quy mô (DLOM)</t>
@@ -2119,7 +2119,7 @@
     <t xml:space="preserve">KẾT QUẢ: GIÁ TRỊ DOANH NGHIỆP, PRE-MONEY, POST-MONEY VÀ TỶ LỆ CỔ PHẦN</t>
   </si>
   <si>
-    <t xml:space="preserve">EV = pre-money − tiền mặt (B31) + nợ vay (B32) tại 31/12/2025, cùng cầu nối giữa EV và vốn CSH như DCF!B22.</t>
+    <t xml:space="preserve">EV = pre-money − tiền mặt (B31) + nợ vay (B32) tại t0 = 01/10/2026, cùng cầu nối giữa EV và vốn CSH như DCF!B22.</t>
   </si>
   <si>
     <t xml:space="preserve">Vốn cổ phần cần huy động năm 2026 (Pro Forma!B63), dùng chung cho DCF và VC Method.</t>
@@ -2128,7 +2128,34 @@
     <t xml:space="preserve">Lấy từ E41: bình quân 4 cách tính, sau chiết khấu thiếu thanh khoản 30%.</t>
   </si>
   <si>
+    <t xml:space="preserve">ĐỐI CHIẾU (không dùng trong pre-money): bội số áp lên TTM pro-rata đến 30/09/2026 = 25% × 2025A + 75% × 2026E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDA TTM</t>
+  </si>
+  <si>
     <t xml:space="preserve">tỷ đồng tương ứng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LNST chuẩn hóa TTM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV/EBITDA TTM × trung vị mẫu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV/EBITDA TTM × bình quân ngành</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P/E TTM × trung vị mẫu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P/E TTM × bình quân ngành</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-money theo Multiples TTM (bình quân 4 cách) – chỉ để đối chiếu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lý do không dùng: 75% số liệu là dự phóng 2026E, và EBITDA 2026 phụ thuộc khoản vốn đang cần gọi; giữ 2025A (12 tháng thực tế gần nhất) làm cơ sở.</t>
   </si>
   <si>
     <t xml:space="preserve">TỔNG HỢP ĐỊNH GIÁ &amp; ĐỀ XUẤT GỌI VỐN – AgriPack</t>
@@ -3690,7 +3717,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="892">
+  <cellXfs count="895">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -7003,7 +7030,7 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="186" fontId="47" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="169" fontId="47" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -7013,6 +7040,18 @@
     </xf>
     <xf numFmtId="174" fontId="47" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -7345,9 +7384,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>775080</xdr:colOff>
+      <xdr:colOff>774360</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>194760</xdr:rowOff>
+      <xdr:rowOff>194040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -7361,7 +7400,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="277560" y="317160"/>
-          <a:ext cx="1051200" cy="289080"/>
+          <a:ext cx="1050480" cy="288360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7807,7 +7846,7 @@
       </c>
       <c r="F19" s="34" t="n">
         <f aca="false">Summary!B8</f>
-        <v>26.0074983564468</v>
+        <v>25.4660139362204</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9825,7 +9864,7 @@
       </c>
       <c r="B20" s="719" t="n">
         <f aca="false">B19/B21</f>
-        <v>0.637646281974959</v>
+        <v>0.644914521110702</v>
       </c>
       <c r="C20" s="720"/>
       <c r="D20" s="714"/>
@@ -9843,7 +9882,7 @@
       </c>
       <c r="B21" s="721" t="n">
         <f aca="false">SUM(B22,B19)</f>
-        <v>63459432.7666413</v>
+        <v>62744239.795064</v>
       </c>
       <c r="C21" s="722"/>
       <c r="D21" s="714"/>
@@ -9861,7 +9900,7 @@
       </c>
       <c r="B22" s="724" t="n">
         <f aca="false">B33</f>
-        <v>22994761.4067526</v>
+        <v>22279568.4351753</v>
       </c>
       <c r="C22" s="722"/>
       <c r="D22" s="725" t="s">
@@ -9876,7 +9915,7 @@
       </c>
       <c r="G22" s="728" t="n">
         <f aca="false">B20</f>
-        <v>0.637646281974959</v>
+        <v>0.644914521110702</v>
       </c>
       <c r="H22" s="729" t="s">
         <v>565</v>
@@ -10016,8 +10055,8 @@
         <v>571</v>
       </c>
       <c r="B31" s="734" t="n">
-        <f aca="false">MAX(0,'Balance Sheet'!F6+(1-B3)*C10)</f>
-        <v>0</v>
+        <f aca="false">'Balance Sheet'!F6+(1-B3)*C10</f>
+        <v>-715192.97157729</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -10053,7 +10092,7 @@
       </c>
       <c r="B33" s="734" t="n">
         <f aca="false">B29+B31-B32</f>
-        <v>22994761.4067526</v>
+        <v>22279568.4351753</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -10107,7 +10146,7 @@
       </c>
       <c r="B36" s="737" t="n">
         <f aca="false">B33/'Income Statement'!E78</f>
-        <v>3.49510146280095</v>
+        <v>3.38639531199867</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -10125,7 +10164,7 @@
       </c>
       <c r="B37" s="490" t="n">
         <f aca="false">B33/'Balance Sheet'!F73</f>
-        <v>0.767202789552963</v>
+        <v>0.743340918009401</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -10738,7 +10777,7 @@
     <tabColor rgb="FF7B1E2B"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K58"/>
   <sheetFormatPr defaultColWidth="8.515625" defaultRowHeight="15.6" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="60.1"/>
@@ -11593,8 +11632,8 @@
         <v>675</v>
       </c>
       <c r="B31" s="808" t="n">
-        <f aca="false">'Balance Sheet'!F6/1000000</f>
-        <v>2.93348176549999</v>
+        <f aca="false">DCF!B31/1000000</f>
+        <v>-0.71519297157729</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -11611,7 +11650,7 @@
         <v>676</v>
       </c>
       <c r="B32" s="808" t="n">
-        <f aca="false">SUM('Balance Sheet'!F45,'Balance Sheet'!F58)/1000000</f>
+        <f aca="false">DCF!B32/1000000</f>
         <v>1.6026</v>
       </c>
       <c r="C32" s="2"/>
@@ -11708,11 +11747,11 @@
       </c>
       <c r="D37" s="815" t="n">
         <f aca="false">B37*C37+B31-B32</f>
-        <v>36.957015033265</v>
+        <v>33.3083402961877</v>
       </c>
       <c r="E37" s="816" t="n">
         <f aca="false">D37*(1-$B$33)</f>
-        <v>25.8699105232855</v>
+        <v>23.3158382073314</v>
       </c>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
@@ -11735,11 +11774,11 @@
       </c>
       <c r="D38" s="815" t="n">
         <f aca="false">B38*C38+B31-B32</f>
-        <v>62.810969197345</v>
+        <v>59.1622944602677</v>
       </c>
       <c r="E38" s="816" t="n">
         <f aca="false">D38*(1-$B$33)</f>
-        <v>43.9676784381415</v>
+        <v>41.4136061221874</v>
       </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
@@ -11811,7 +11850,7 @@
       <c r="D41" s="2"/>
       <c r="E41" s="816" t="n">
         <f aca="false">AVERAGE(E37:E40)</f>
-        <v>27.7109676946228</v>
+        <v>26.4339315366457</v>
       </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
@@ -11832,7 +11871,7 @@
       </c>
       <c r="E42" s="819" t="n">
         <f aca="false">MAX(E37:E40)</f>
-        <v>43.9676784381415</v>
+        <v>41.4136061221874</v>
       </c>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
@@ -11875,7 +11914,7 @@
       </c>
       <c r="B45" s="820" t="n">
         <f aca="false">B49-B31+B32</f>
-        <v>26.3800859291228</v>
+        <v>28.751724508223</v>
       </c>
       <c r="C45" s="789" t="s">
         <v>692</v>
@@ -11915,7 +11954,7 @@
       </c>
       <c r="B47" s="823" t="n">
         <f aca="false">B46/B48</f>
-        <v>0.593535637084886</v>
+        <v>0.604865716291138</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
@@ -11933,7 +11972,7 @@
       </c>
       <c r="B48" s="824" t="n">
         <f aca="false">SUM(B49,B46)</f>
-        <v>68.1756390545115</v>
+        <v>66.8986028965345</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
@@ -11951,7 +11990,7 @@
       </c>
       <c r="B49" s="824" t="n">
         <f aca="false">E41</f>
-        <v>27.7109676946228</v>
+        <v>26.4339315366457</v>
       </c>
       <c r="C49" s="789" t="s">
         <v>694</v>
@@ -11971,7 +12010,7 @@
       </c>
       <c r="B50" s="826" t="n">
         <f aca="false">1-B47</f>
-        <v>0.406464362915114</v>
+        <v>0.395134283708862</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
@@ -11984,7 +12023,9 @@
       <c r="K50" s="2"/>
     </row>
     <row r="51" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="2"/>
+      <c r="A51" s="265" t="s">
+        <v>695</v>
+      </c>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
@@ -11998,18 +12039,18 @@
     </row>
     <row r="52" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="827" t="s">
-        <v>563</v>
+        <v>696</v>
       </c>
       <c r="B52" s="828" t="n">
-        <f aca="false">B46</f>
-        <v>40.4646713598887</v>
+        <f aca="false">0.25*B27+0.75*'Income Statement'!E80/1000000</f>
+        <v>10.46181032986</v>
       </c>
       <c r="C52" s="829" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="D52" s="830" t="n">
         <f aca="false">B47</f>
-        <v>0.593535637084886</v>
+        <v>0.604865716291138</v>
       </c>
       <c r="E52" s="829" t="s">
         <v>565</v>
@@ -12022,8 +12063,13 @@
       <c r="K52" s="2"/>
     </row>
     <row r="53" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2"/>
+      <c r="A53" s="2" t="s">
+        <v>698</v>
+      </c>
+      <c r="B53" s="831" t="n">
+        <f aca="false">(0.25*B28+0.75*'Income Statement'!E74/1000000)*(1-B29)</f>
+        <v>5.37320882388798</v>
+      </c>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
@@ -12035,11 +12081,16 @@
       <c r="K53" s="2"/>
     </row>
     <row r="54" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="414"/>
+      <c r="A54" s="414" t="s">
+        <v>699</v>
+      </c>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
+      <c r="E54" s="831" t="n">
+        <f aca="false">(B37*B52+B31-B32)*(1-$B$33)</f>
+        <v>32.2842721989721</v>
+      </c>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
       <c r="H54" s="2"/>
@@ -12048,11 +12099,16 @@
       <c r="K54" s="2"/>
     </row>
     <row r="55" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="788"/>
+      <c r="A55" s="788" t="s">
+        <v>700</v>
+      </c>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="815"/>
-      <c r="E55" s="2"/>
+      <c r="E55" s="831" t="n">
+        <f aca="false">(B38*B52+B31-B32)*(1-$B$33)</f>
+        <v>56.8904500948027</v>
+      </c>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
@@ -12061,17 +12117,43 @@
       <c r="K55" s="2"/>
     </row>
     <row r="56" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="336"/>
+      <c r="A56" s="336" t="s">
+        <v>701</v>
+      </c>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
+      <c r="E56" s="831" t="n">
+        <f aca="false">B39*B53*(1-$B$33)</f>
+        <v>26.8364914709085</v>
+      </c>
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
+    </row>
+    <row r="57" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1" t="s">
+        <v>702</v>
+      </c>
+      <c r="E57" s="832" t="n">
+        <f aca="false">B40*B53*(1-$B$33)</f>
+        <v>35.4685514464846</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="329" t="s">
+        <v>703</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>704</v>
+      </c>
+      <c r="E58" s="833" t="n">
+        <f aca="false">AVERAGE(E54:E57)</f>
+        <v>37.869941302792</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -12104,7 +12186,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="790" t="s">
-        <v>696</v>
+        <v>705</v>
       </c>
       <c r="B1" s="226"/>
       <c r="C1" s="2"/>
@@ -12122,7 +12204,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="336" t="s">
-        <v>697</v>
+        <v>706</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -12156,25 +12238,25 @@
     </row>
     <row r="4" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="813" t="s">
-        <v>698</v>
+        <v>707</v>
       </c>
       <c r="B4" s="567" t="s">
-        <v>699</v>
+        <v>708</v>
       </c>
       <c r="C4" s="567" t="s">
-        <v>700</v>
+        <v>709</v>
       </c>
       <c r="D4" s="567" t="s">
-        <v>701</v>
+        <v>710</v>
       </c>
       <c r="E4" s="567" t="s">
-        <v>702</v>
+        <v>711</v>
       </c>
       <c r="F4" s="575" t="s">
-        <v>703</v>
-      </c>
-      <c r="G4" s="831" t="s">
-        <v>704</v>
+        <v>712</v>
+      </c>
+      <c r="G4" s="834" t="s">
+        <v>713</v>
       </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
@@ -12186,11 +12268,11 @@
     </row>
     <row r="5" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>705</v>
+        <v>714</v>
       </c>
       <c r="B5" s="815" t="n">
         <f aca="false">DCF!B22/1000000</f>
-        <v>22.9947614067526</v>
+        <v>22.2795684351753</v>
       </c>
       <c r="C5" s="815" t="n">
         <f aca="false">DCF!B19/1000000</f>
@@ -12198,17 +12280,17 @@
       </c>
       <c r="D5" s="815" t="n">
         <f aca="false">SUM(B5:C5)</f>
-        <v>63.4594327666413</v>
+        <v>62.744239795064</v>
       </c>
       <c r="E5" s="785" t="n">
         <f aca="false">IF(B5&lt;=0,"n.m.",C5/D5)</f>
-        <v>0.637646281974959</v>
-      </c>
-      <c r="F5" s="832" t="n">
+        <v>0.644914521110702</v>
+      </c>
+      <c r="F5" s="835" t="n">
         <v>0.4</v>
       </c>
       <c r="G5" s="336" t="s">
-        <v>706</v>
+        <v>715</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -12220,7 +12302,7 @@
     </row>
     <row r="6" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>707</v>
+        <v>716</v>
       </c>
       <c r="B6" s="815" t="n">
         <f aca="false">VCM!E7/1000000</f>
@@ -12238,11 +12320,11 @@
         <f aca="false">IF(B6&lt;=0,"n.m.",C6/D6)</f>
         <v>0.589578919093115</v>
       </c>
-      <c r="F6" s="832" t="n">
+      <c r="F6" s="835" t="n">
         <v>0.4</v>
       </c>
       <c r="G6" s="336" t="s">
-        <v>708</v>
+        <v>717</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -12254,29 +12336,29 @@
     </row>
     <row r="7" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="783" t="s">
-        <v>709</v>
-      </c>
-      <c r="B7" s="833" t="n">
+        <v>718</v>
+      </c>
+      <c r="B7" s="836" t="n">
         <f aca="false">Multiples!B49</f>
-        <v>27.7109676946228</v>
-      </c>
-      <c r="C7" s="833" t="n">
+        <v>26.4339315366457</v>
+      </c>
+      <c r="C7" s="836" t="n">
         <f aca="false">Multiples!B46</f>
         <v>40.4646713598887</v>
       </c>
       <c r="D7" s="815" t="n">
         <f aca="false">SUM(B7:C7)</f>
-        <v>68.1756390545115</v>
+        <v>66.8986028965345</v>
       </c>
       <c r="E7" s="785" t="n">
         <f aca="false">IF(B7&lt;=0,"n.m.",C7/D7)</f>
-        <v>0.593535637084886</v>
-      </c>
-      <c r="F7" s="832" t="n">
+        <v>0.604865716291138</v>
+      </c>
+      <c r="F7" s="835" t="n">
         <v>0.2</v>
       </c>
       <c r="G7" s="336" t="s">
-        <v>710</v>
+        <v>719</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
@@ -12287,26 +12369,26 @@
       <c r="N7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="834" t="s">
-        <v>711</v>
-      </c>
-      <c r="B8" s="835" t="n">
+      <c r="A8" s="837" t="s">
+        <v>720</v>
+      </c>
+      <c r="B8" s="838" t="n">
         <f aca="false">(B5*F5+B6*F6+B7*F7)/SUM(F5:F7)</f>
-        <v>26.0074983564468</v>
-      </c>
-      <c r="C8" s="835" t="n">
+        <v>25.4660139362204</v>
+      </c>
+      <c r="C8" s="838" t="n">
         <f aca="false">C5</f>
         <v>40.4646713598887</v>
       </c>
-      <c r="D8" s="835" t="n">
+      <c r="D8" s="838" t="n">
         <f aca="false">SUM(B8:C8)</f>
-        <v>66.4721697163355</v>
-      </c>
-      <c r="E8" s="836" t="n">
+        <v>65.9306852961092</v>
+      </c>
+      <c r="E8" s="839" t="n">
         <f aca="false">IF(B8&lt;=0,"n.m.",C8/D8)</f>
-        <v>0.608746059178877</v>
-      </c>
-      <c r="F8" s="837" t="n">
+        <v>0.613745650877934</v>
+      </c>
+      <c r="F8" s="840" t="n">
         <f aca="false">SUM(F5:F7)</f>
         <v>1</v>
       </c>
@@ -12320,12 +12402,12 @@
       <c r="N8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="838"/>
-      <c r="B9" s="839"/>
-      <c r="C9" s="839"/>
-      <c r="D9" s="839"/>
-      <c r="E9" s="840"/>
-      <c r="F9" s="841"/>
+      <c r="A9" s="841"/>
+      <c r="B9" s="842"/>
+      <c r="C9" s="842"/>
+      <c r="D9" s="842"/>
+      <c r="E9" s="843"/>
+      <c r="F9" s="844"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -12337,7 +12419,7 @@
     </row>
     <row r="10" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="812" t="s">
-        <v>712</v>
+        <v>721</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
@@ -12354,17 +12436,17 @@
       <c r="N10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="842" t="s">
-        <v>713</v>
-      </c>
-      <c r="B11" s="843" t="n">
+      <c r="A11" s="845" t="s">
+        <v>722</v>
+      </c>
+      <c r="B11" s="846" t="n">
         <f aca="false">(1-VCM!B4)*B5+VCM!B4*B12</f>
-        <v>19.7912983971515</v>
-      </c>
-      <c r="C11" s="844"/>
-      <c r="D11" s="845"/>
-      <c r="E11" s="845"/>
-      <c r="F11" s="845"/>
+        <v>19.3621826142052</v>
+      </c>
+      <c r="C11" s="847"/>
+      <c r="D11" s="848"/>
+      <c r="E11" s="848"/>
+      <c r="F11" s="848"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -12375,21 +12457,21 @@
       <c r="N11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="842" t="s">
-        <v>714</v>
-      </c>
-      <c r="B12" s="843" t="n">
+      <c r="A12" s="845" t="s">
+        <v>723</v>
+      </c>
+      <c r="B12" s="846" t="n">
         <f aca="false">C12*'Balance Sheet'!F73/1000000</f>
         <v>14.98610388275</v>
       </c>
-      <c r="C12" s="846" t="n">
+      <c r="C12" s="849" t="n">
         <v>0.5</v>
       </c>
-      <c r="D12" s="847" t="s">
-        <v>715</v>
-      </c>
-      <c r="E12" s="847"/>
-      <c r="F12" s="847"/>
+      <c r="D12" s="850" t="s">
+        <v>724</v>
+      </c>
+      <c r="E12" s="850"/>
+      <c r="F12" s="850"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -12400,7 +12482,7 @@
       <c r="N12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="848"/>
+      <c r="A13" s="851"/>
       <c r="B13" s="815"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -12465,7 +12547,7 @@
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="812" t="s">
-        <v>716</v>
+        <v>725</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -12483,19 +12565,19 @@
     </row>
     <row r="18" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="813" t="s">
-        <v>698</v>
+        <v>707</v>
       </c>
       <c r="B18" s="567" t="s">
         <v>593</v>
       </c>
       <c r="C18" s="567" t="s">
-        <v>717</v>
+        <v>726</v>
       </c>
       <c r="D18" s="567" t="s">
         <v>594</v>
       </c>
       <c r="E18" s="575" t="s">
-        <v>718</v>
+        <v>727</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -12508,23 +12590,23 @@
       <c r="N18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="849" t="s">
+      <c r="A19" s="852" t="s">
         <v>48</v>
       </c>
-      <c r="B19" s="850" t="n">
+      <c r="B19" s="853" t="n">
         <f aca="false">MIN(Sensitivity!C7:E9)</f>
-        <v>13.4694523430269</v>
-      </c>
-      <c r="C19" s="851" t="n">
+        <v>12.7542593714496</v>
+      </c>
+      <c r="C19" s="854" t="n">
         <f aca="false">B5</f>
-        <v>22.9947614067526</v>
-      </c>
-      <c r="D19" s="850" t="n">
+        <v>22.2795684351753</v>
+      </c>
+      <c r="D19" s="853" t="n">
         <f aca="false">MAX(Sensitivity!C7:E9)</f>
-        <v>33.0495622160443</v>
-      </c>
-      <c r="E19" s="852" t="s">
-        <v>719</v>
+        <v>32.334369244467</v>
+      </c>
+      <c r="E19" s="855" t="s">
+        <v>728</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
@@ -12537,23 +12619,23 @@
       <c r="N19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="849" t="s">
-        <v>720</v>
-      </c>
-      <c r="B20" s="850" t="n">
+      <c r="A20" s="852" t="s">
+        <v>729</v>
+      </c>
+      <c r="B20" s="853" t="n">
         <f aca="false">MIN(Sensitivity!C16:E18)</f>
         <v>13.0120084877283</v>
       </c>
-      <c r="C20" s="851" t="n">
+      <c r="C20" s="854" t="n">
         <f aca="false">B6</f>
         <v>28.1685006370529</v>
       </c>
-      <c r="D20" s="850" t="n">
+      <c r="D20" s="853" t="n">
         <f aca="false">MAX(Sensitivity!C16:E18)</f>
         <v>45.0408220863011</v>
       </c>
-      <c r="E20" s="852" t="s">
-        <v>721</v>
+      <c r="E20" s="855" t="s">
+        <v>730</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -12566,23 +12648,23 @@
       <c r="N20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="849" t="s">
-        <v>722</v>
-      </c>
-      <c r="B21" s="850" t="n">
+      <c r="A21" s="852" t="s">
+        <v>731</v>
+      </c>
+      <c r="B21" s="853" t="n">
         <f aca="false">Multiples!D42</f>
         <v>17.6625306830518</v>
       </c>
-      <c r="C21" s="851" t="n">
+      <c r="C21" s="854" t="n">
         <f aca="false">B7</f>
-        <v>27.7109676946228</v>
-      </c>
-      <c r="D21" s="850" t="n">
+        <v>26.4339315366457</v>
+      </c>
+      <c r="D21" s="853" t="n">
         <f aca="false">Multiples!E42</f>
-        <v>43.9676784381415</v>
-      </c>
-      <c r="E21" s="852" t="s">
-        <v>723</v>
+        <v>41.4136061221874</v>
+      </c>
+      <c r="E21" s="855" t="s">
+        <v>732</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -12595,23 +12677,23 @@
       <c r="N21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="853" t="s">
-        <v>724</v>
-      </c>
-      <c r="B22" s="854" t="n">
+      <c r="A22" s="856" t="s">
+        <v>733</v>
+      </c>
+      <c r="B22" s="857" t="n">
         <f aca="false">(B19*F5+B20*F6+B21*F7)/F8</f>
-        <v>14.1250904689124</v>
-      </c>
-      <c r="C22" s="855" t="n">
+        <v>13.8390132802815</v>
+      </c>
+      <c r="C22" s="858" t="n">
         <f aca="false">B8</f>
-        <v>26.0074983564468</v>
-      </c>
-      <c r="D22" s="854" t="n">
+        <v>25.4660139362204</v>
+      </c>
+      <c r="D22" s="857" t="n">
         <f aca="false">(D19*F5+D20*F6+D21*F7)/F8</f>
-        <v>40.0296894085664</v>
-      </c>
-      <c r="E22" s="856" t="s">
-        <v>725</v>
+        <v>39.2327977567447</v>
+      </c>
+      <c r="E22" s="859" t="s">
+        <v>734</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -12641,7 +12723,7 @@
     </row>
     <row r="24" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="776" t="s">
-        <v>726</v>
+        <v>735</v>
       </c>
       <c r="B24" s="548"/>
       <c r="C24" s="2"/>
@@ -12658,10 +12740,10 @@
       <c r="N24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="849" t="s">
-        <v>727</v>
-      </c>
-      <c r="B25" s="857" t="n">
+      <c r="A25" s="852" t="s">
+        <v>736</v>
+      </c>
+      <c r="B25" s="860" t="n">
         <f aca="false">C8</f>
         <v>40.4646713598887</v>
       </c>
@@ -12679,12 +12761,12 @@
       <c r="N25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="849" t="s">
-        <v>728</v>
-      </c>
-      <c r="B26" s="858" t="n">
+      <c r="A26" s="852" t="s">
+        <v>737</v>
+      </c>
+      <c r="B26" s="861" t="n">
         <f aca="false">E8</f>
-        <v>0.608746059178877</v>
+        <v>0.613745650877934</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -12700,10 +12782,10 @@
       <c r="N26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="859" t="s">
-        <v>729</v>
-      </c>
-      <c r="B27" s="860" t="n">
+      <c r="A27" s="862" t="s">
+        <v>738</v>
+      </c>
+      <c r="B27" s="863" t="n">
         <f aca="false">SUM(Drivers!F125:J125)/1000000</f>
         <v>39.1579837983445</v>
       </c>
@@ -12721,10 +12803,10 @@
       <c r="N27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="861" t="s">
-        <v>730</v>
-      </c>
-      <c r="B28" s="862" t="n">
+      <c r="A28" s="864" t="s">
+        <v>739</v>
+      </c>
+      <c r="B28" s="865" t="n">
         <f aca="false">SUM(B25,B27)</f>
         <v>79.6226551582333</v>
       </c>
@@ -12775,7 +12857,7 @@
     </row>
     <row r="31" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="812" t="s">
-        <v>731</v>
+        <v>740</v>
       </c>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -12793,7 +12875,7 @@
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="336" t="s">
-        <v>732</v>
+        <v>741</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -12818,16 +12900,16 @@
         <v>Đang chạy: Base</v>
       </c>
       <c r="C33" s="567" t="s">
-        <v>733</v>
+        <v>742</v>
       </c>
       <c r="D33" s="567" t="s">
-        <v>734</v>
+        <v>743</v>
       </c>
       <c r="E33" s="567" t="s">
-        <v>735</v>
+        <v>744</v>
       </c>
       <c r="F33" s="575" t="s">
-        <v>736</v>
+        <v>745</v>
       </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
@@ -12840,22 +12922,22 @@
     </row>
     <row r="34" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="18" t="s">
-        <v>737</v>
-      </c>
-      <c r="B34" s="863" t="n">
+        <v>746</v>
+      </c>
+      <c r="B34" s="866" t="n">
         <f aca="false">'Income Statement'!I11/1000000</f>
         <v>178.89220902969</v>
       </c>
-      <c r="C34" s="864" t="n">
+      <c r="C34" s="867" t="n">
         <v>121.163880717148</v>
       </c>
-      <c r="D34" s="864" t="n">
+      <c r="D34" s="867" t="n">
         <v>227.441176895844</v>
       </c>
-      <c r="E34" s="864" t="n">
+      <c r="E34" s="867" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="F34" s="865" t="n">
+      <c r="F34" s="868" t="n">
         <v>178.89220902969</v>
       </c>
       <c r="G34" s="2"/>
@@ -12869,22 +12951,22 @@
     </row>
     <row r="35" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="18" t="s">
-        <v>738</v>
-      </c>
-      <c r="B35" s="866" t="n">
+        <v>747</v>
+      </c>
+      <c r="B35" s="869" t="n">
         <f aca="false">('Income Statement'!I11/'Income Statement'!D11)^(1/5)-1</f>
         <v>0.303450441286468</v>
       </c>
-      <c r="C35" s="867" t="n">
+      <c r="C35" s="870" t="n">
         <v>0.205732238215002</v>
       </c>
-      <c r="D35" s="867" t="n">
+      <c r="D35" s="870" t="n">
         <v>0.367571548032998</v>
       </c>
-      <c r="E35" s="867" t="n">
+      <c r="E35" s="870" t="n">
         <v>0.303450441286468</v>
       </c>
-      <c r="F35" s="868" t="n">
+      <c r="F35" s="871" t="n">
         <v>0.303450441286468</v>
       </c>
       <c r="G35" s="2"/>
@@ -12898,22 +12980,22 @@
     </row>
     <row r="36" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="18" t="s">
-        <v>739</v>
-      </c>
-      <c r="B36" s="866" t="n">
+        <v>748</v>
+      </c>
+      <c r="B36" s="869" t="n">
         <f aca="false">'Income Statement'!I80/'Income Statement'!I11</f>
         <v>0.20669187471551</v>
       </c>
-      <c r="C36" s="867" t="n">
+      <c r="C36" s="870" t="n">
         <v>0.13983212556253</v>
       </c>
-      <c r="D36" s="867" t="n">
+      <c r="D36" s="870" t="n">
         <v>0.240698731755984</v>
       </c>
-      <c r="E36" s="867" t="n">
+      <c r="E36" s="870" t="n">
         <v>0.20669187471551</v>
       </c>
-      <c r="F36" s="868" t="n">
+      <c r="F36" s="871" t="n">
         <v>0.20669187471551</v>
       </c>
       <c r="G36" s="2"/>
@@ -12927,22 +13009,22 @@
     </row>
     <row r="37" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="18" t="s">
-        <v>740</v>
-      </c>
-      <c r="B37" s="863" t="n">
+        <v>749</v>
+      </c>
+      <c r="B37" s="866" t="n">
         <f aca="false">'Income Statement'!I78/1000000</f>
         <v>13.3741460043913</v>
       </c>
-      <c r="C37" s="864" t="n">
+      <c r="C37" s="867" t="n">
         <v>-0.188144670982913</v>
       </c>
-      <c r="D37" s="864" t="n">
+      <c r="D37" s="867" t="n">
         <v>25.7416742613056</v>
       </c>
-      <c r="E37" s="864" t="n">
+      <c r="E37" s="867" t="n">
         <v>16.1935208378721</v>
       </c>
-      <c r="F37" s="865" t="n">
+      <c r="F37" s="868" t="n">
         <v>12.6693022960211</v>
       </c>
       <c r="G37" s="2"/>
@@ -12956,22 +13038,22 @@
     </row>
     <row r="38" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="18" t="s">
-        <v>741</v>
-      </c>
-      <c r="B38" s="863" t="n">
+        <v>750</v>
+      </c>
+      <c r="B38" s="866" t="n">
         <f aca="false">SUM(DCF!C10:G10)/1000000</f>
         <v>-53.9371425360351</v>
       </c>
-      <c r="C38" s="864" t="n">
+      <c r="C38" s="867" t="n">
         <v>-57.6325593720804</v>
       </c>
-      <c r="D38" s="864" t="n">
+      <c r="D38" s="867" t="n">
         <v>-49.3917978554204</v>
       </c>
-      <c r="E38" s="864" t="n">
+      <c r="E38" s="867" t="n">
         <v>-53.9371425360351</v>
       </c>
-      <c r="F38" s="865" t="n">
+      <c r="F38" s="868" t="n">
         <v>-53.9371425360351</v>
       </c>
       <c r="G38" s="2"/>
@@ -12985,22 +13067,22 @@
     </row>
     <row r="39" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="18" t="s">
-        <v>742</v>
-      </c>
-      <c r="B39" s="863" t="n">
+        <v>751</v>
+      </c>
+      <c r="B39" s="866" t="n">
         <f aca="false">'Pro Forma'!B61/1000000</f>
         <v>40.4646713598887</v>
       </c>
-      <c r="C39" s="864" t="n">
+      <c r="C39" s="867" t="n">
         <v>47.3094743775238</v>
       </c>
-      <c r="D39" s="864" t="n">
+      <c r="D39" s="867" t="n">
         <v>34.3242588002227</v>
       </c>
-      <c r="E39" s="864" t="n">
+      <c r="E39" s="867" t="n">
         <v>73.6277508567534</v>
       </c>
-      <c r="F39" s="865" t="n">
+      <c r="F39" s="868" t="n">
         <v>33.9174564688055</v>
       </c>
       <c r="G39" s="2"/>
@@ -13014,22 +13096,22 @@
     </row>
     <row r="40" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="18" t="s">
-        <v>743</v>
-      </c>
-      <c r="B40" s="863" t="n">
+        <v>752</v>
+      </c>
+      <c r="B40" s="866" t="n">
         <f aca="false">SUM(Drivers!F125:J125)/1000000</f>
         <v>39.1579837983445</v>
       </c>
-      <c r="C40" s="864" t="n">
+      <c r="C40" s="867" t="n">
         <v>31.4016790921057</v>
       </c>
-      <c r="D40" s="864" t="n">
+      <c r="D40" s="867" t="n">
         <v>44.8558406219516</v>
       </c>
-      <c r="E40" s="864" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" s="865" t="n">
+      <c r="E40" s="867" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="868" t="n">
         <v>48.9474797479307</v>
       </c>
       <c r="G40" s="2"/>
@@ -13045,20 +13127,20 @@
       <c r="A41" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="B41" s="866" t="n">
+      <c r="B41" s="869" t="n">
         <f aca="false">'Discount rate'!E4</f>
         <v>0.141309839519679</v>
       </c>
-      <c r="C41" s="867" t="n">
+      <c r="C41" s="870" t="n">
         <v>0.140795536109349</v>
       </c>
-      <c r="D41" s="867" t="n">
+      <c r="D41" s="870" t="n">
         <v>0.14166079659066</v>
       </c>
-      <c r="E41" s="867" t="n">
+      <c r="E41" s="870" t="n">
         <v>0.136668124116301</v>
       </c>
-      <c r="F41" s="868" t="n">
+      <c r="F41" s="871" t="n">
         <v>0.142347620348559</v>
       </c>
       <c r="G41" s="2"/>
@@ -13072,23 +13154,23 @@
     </row>
     <row r="42" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="18" t="s">
-        <v>744</v>
-      </c>
-      <c r="B42" s="863" t="n">
+        <v>753</v>
+      </c>
+      <c r="B42" s="866" t="n">
         <f aca="false">B5</f>
-        <v>22.9947614067526</v>
-      </c>
-      <c r="C42" s="864" t="n">
-        <v>-60.2877610097098</v>
-      </c>
-      <c r="D42" s="864" t="n">
-        <v>99.8206222064367</v>
-      </c>
-      <c r="E42" s="864" t="n">
-        <v>27.2563852914441</v>
-      </c>
-      <c r="F42" s="865" t="n">
-        <v>22.1075648881229</v>
+        <v>22.2795684351753</v>
+      </c>
+      <c r="C42" s="867" t="n">
+        <v>-61.4323148226172</v>
+      </c>
+      <c r="D42" s="867" t="n">
+        <v>99.4620460335602</v>
+      </c>
+      <c r="E42" s="867" t="n">
+        <v>26.5411923198669</v>
+      </c>
+      <c r="F42" s="868" t="n">
+        <v>21.3923719165456</v>
       </c>
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
@@ -13101,22 +13183,22 @@
     </row>
     <row r="43" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="18" t="s">
-        <v>745</v>
-      </c>
-      <c r="B43" s="863" t="n">
+        <v>754</v>
+      </c>
+      <c r="B43" s="866" t="n">
         <f aca="false">B6</f>
         <v>28.1685006370529</v>
       </c>
-      <c r="C43" s="864" t="n">
+      <c r="C43" s="867" t="n">
         <v>-27.1869051180712</v>
       </c>
-      <c r="D43" s="864" t="n">
+      <c r="D43" s="867" t="n">
         <v>77.9063327224381</v>
       </c>
-      <c r="E43" s="864" t="n">
+      <c r="E43" s="867" t="n">
         <v>7.89790782077882</v>
       </c>
-      <c r="F43" s="865" t="n">
+      <c r="F43" s="868" t="n">
         <v>31.8861460935203</v>
       </c>
       <c r="G43" s="2"/>
@@ -13130,23 +13212,23 @@
     </row>
     <row r="44" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="18" t="s">
-        <v>746</v>
-      </c>
-      <c r="B44" s="863" t="n">
+        <v>755</v>
+      </c>
+      <c r="B44" s="866" t="n">
         <f aca="false">B8</f>
-        <v>26.0074983564468</v>
-      </c>
-      <c r="C44" s="864" t="n">
-        <v>-29.4476729121878</v>
-      </c>
-      <c r="D44" s="864" t="n">
-        <v>76.6329755104745</v>
-      </c>
-      <c r="E44" s="864" t="n">
-        <v>19.6039107838137</v>
-      </c>
-      <c r="F44" s="865" t="n">
-        <v>27.1396779315818</v>
+        <v>25.4660139362204</v>
+      </c>
+      <c r="C44" s="867" t="n">
+        <v>-30.1909569278393</v>
+      </c>
+      <c r="D44" s="867" t="n">
+        <v>76.2591009856375</v>
+      </c>
+      <c r="E44" s="867" t="n">
+        <v>19.0624263635874</v>
+      </c>
+      <c r="F44" s="868" t="n">
+        <v>26.5981935113555</v>
       </c>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
@@ -13159,23 +13241,23 @@
     </row>
     <row r="45" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="18" t="s">
-        <v>747</v>
-      </c>
-      <c r="B45" s="866" t="n">
+        <v>756</v>
+      </c>
+      <c r="B45" s="869" t="n">
         <f aca="false">E8</f>
-        <v>0.608746059178877</v>
-      </c>
-      <c r="C45" s="867" t="s">
-        <v>748</v>
-      </c>
-      <c r="D45" s="867" t="n">
-        <v>0.309346740782215</v>
-      </c>
-      <c r="E45" s="867" t="n">
-        <v>0.789729042271154</v>
-      </c>
-      <c r="F45" s="868" t="n">
-        <v>0.555503575493552</v>
+        <v>0.613745650877934</v>
+      </c>
+      <c r="C45" s="870" t="s">
+        <v>757</v>
+      </c>
+      <c r="D45" s="870" t="n">
+        <v>0.31039262025218</v>
+      </c>
+      <c r="E45" s="870" t="n">
+        <v>0.794342540544801</v>
+      </c>
+      <c r="F45" s="871" t="n">
+        <v>0.560474133218841</v>
       </c>
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
@@ -13188,23 +13270,23 @@
     </row>
     <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="817" t="s">
-        <v>749</v>
-      </c>
-      <c r="B46" s="869" t="n">
+        <v>758</v>
+      </c>
+      <c r="B46" s="872" t="n">
         <f aca="false">IF(B8&lt;=0,"n.m.",1-E8)</f>
-        <v>0.391253940821123</v>
-      </c>
-      <c r="C46" s="870" t="s">
-        <v>748</v>
-      </c>
-      <c r="D46" s="870" t="n">
-        <v>0.690653259217785</v>
-      </c>
-      <c r="E46" s="870" t="n">
-        <v>0.210270957728846</v>
-      </c>
-      <c r="F46" s="871" t="n">
-        <v>0.444496424506448</v>
+        <v>0.386254349122066</v>
+      </c>
+      <c r="C46" s="873" t="s">
+        <v>757</v>
+      </c>
+      <c r="D46" s="873" t="n">
+        <v>0.68960737974782</v>
+      </c>
+      <c r="E46" s="873" t="n">
+        <v>0.205657459455199</v>
+      </c>
+      <c r="F46" s="874" t="n">
+        <v>0.439525866781159</v>
       </c>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
@@ -13249,7 +13331,7 @@
     </row>
     <row r="49" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="812" t="s">
-        <v>750</v>
+        <v>759</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -13267,7 +13349,7 @@
     </row>
     <row r="50" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="336" t="s">
-        <v>751</v>
+        <v>760</v>
       </c>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -13284,397 +13366,397 @@
       <c r="N50" s="2"/>
     </row>
     <row r="51" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="831" t="s">
-        <v>752</v>
-      </c>
-      <c r="B51" s="831" t="s">
-        <v>753</v>
-      </c>
-      <c r="C51" s="831" t="s">
-        <v>754</v>
-      </c>
-      <c r="D51" s="831" t="s">
-        <v>755</v>
-      </c>
-      <c r="E51" s="831" t="s">
-        <v>756</v>
-      </c>
-      <c r="F51" s="831" t="s">
-        <v>757</v>
-      </c>
-      <c r="G51" s="831" t="s">
-        <v>758</v>
-      </c>
-      <c r="H51" s="831" t="s">
-        <v>759</v>
-      </c>
-      <c r="I51" s="831" t="s">
-        <v>760</v>
-      </c>
-      <c r="J51" s="831" t="s">
+      <c r="A51" s="834" t="s">
         <v>761</v>
       </c>
-      <c r="K51" s="831" t="s">
+      <c r="B51" s="834" t="s">
         <v>762</v>
       </c>
-      <c r="L51" s="831" t="s">
+      <c r="C51" s="834" t="s">
         <v>763</v>
       </c>
-      <c r="M51" s="831" t="s">
+      <c r="D51" s="834" t="s">
         <v>764</v>
       </c>
-      <c r="N51" s="831" t="s">
+      <c r="E51" s="834" t="s">
         <v>765</v>
       </c>
+      <c r="F51" s="834" t="s">
+        <v>766</v>
+      </c>
+      <c r="G51" s="834" t="s">
+        <v>767</v>
+      </c>
+      <c r="H51" s="834" t="s">
+        <v>768</v>
+      </c>
+      <c r="I51" s="834" t="s">
+        <v>769</v>
+      </c>
+      <c r="J51" s="834" t="s">
+        <v>770</v>
+      </c>
+      <c r="K51" s="834" t="s">
+        <v>771</v>
+      </c>
+      <c r="L51" s="834" t="s">
+        <v>772</v>
+      </c>
+      <c r="M51" s="834" t="s">
+        <v>773</v>
+      </c>
+      <c r="N51" s="834" t="s">
+        <v>774</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="872" t="s">
-        <v>766</v>
-      </c>
-      <c r="B52" s="873" t="n">
-        <v>26.0074983564468</v>
-      </c>
-      <c r="C52" s="873" t="n">
-        <v>26.0074983564468</v>
-      </c>
-      <c r="D52" s="874" t="n">
-        <v>0</v>
-      </c>
-      <c r="E52" s="874" t="n">
-        <v>0</v>
-      </c>
-      <c r="F52" s="873" t="n">
-        <v>22.9947614067526</v>
-      </c>
-      <c r="G52" s="873" t="n">
-        <v>22.9947614067526</v>
-      </c>
-      <c r="H52" s="873" t="n">
+      <c r="A52" s="875" t="s">
+        <v>775</v>
+      </c>
+      <c r="B52" s="876" t="n">
+        <v>25.4660139362204</v>
+      </c>
+      <c r="C52" s="876" t="n">
+        <v>25.4660139362204</v>
+      </c>
+      <c r="D52" s="877" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" s="877" t="n">
+        <v>0</v>
+      </c>
+      <c r="F52" s="876" t="n">
+        <v>22.2795684351753</v>
+      </c>
+      <c r="G52" s="876" t="n">
+        <v>22.2795684351753</v>
+      </c>
+      <c r="H52" s="876" t="n">
         <v>28.1685006370529</v>
       </c>
-      <c r="I52" s="873" t="n">
+      <c r="I52" s="876" t="n">
         <v>28.1685006370529</v>
       </c>
-      <c r="J52" s="873" t="n">
+      <c r="J52" s="876" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="K52" s="873" t="n">
+      <c r="K52" s="876" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="L52" s="873" t="n">
+      <c r="L52" s="876" t="n">
         <v>13.3741460043913</v>
       </c>
-      <c r="M52" s="873" t="n">
+      <c r="M52" s="876" t="n">
         <v>13.3741460043913</v>
       </c>
       <c r="N52" s="465"/>
     </row>
     <row r="53" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="783" t="s">
-        <v>767</v>
-      </c>
-      <c r="B53" s="864" t="n">
-        <v>-1.96554644080494</v>
-      </c>
-      <c r="C53" s="864" t="n">
-        <v>59.9233919574906</v>
-      </c>
-      <c r="D53" s="875" t="n">
-        <v>-27.9730447972517</v>
-      </c>
-      <c r="E53" s="875" t="n">
-        <v>33.9158936010438</v>
-      </c>
-      <c r="F53" s="864" t="n">
-        <v>-20.312298248552</v>
-      </c>
-      <c r="G53" s="864" t="n">
-        <v>75.8171447729884</v>
-      </c>
-      <c r="H53" s="864" t="n">
+        <v>776</v>
+      </c>
+      <c r="B53" s="867" t="n">
+        <v>-2.43017647090996</v>
+      </c>
+      <c r="C53" s="867" t="n">
+        <v>59.3050531471429</v>
+      </c>
+      <c r="D53" s="878" t="n">
+        <v>-27.8961904071304</v>
+      </c>
+      <c r="E53" s="878" t="n">
+        <v>33.8390392109225</v>
+      </c>
+      <c r="F53" s="867" t="n">
+        <v>-20.8639712411478</v>
+      </c>
+      <c r="G53" s="867" t="n">
+        <v>74.9384318224296</v>
+      </c>
+      <c r="H53" s="867" t="n">
         <v>1.5429482992283</v>
       </c>
-      <c r="I53" s="864" t="n">
+      <c r="I53" s="867" t="n">
         <v>60.1358512734266</v>
       </c>
-      <c r="J53" s="864" t="n">
+      <c r="J53" s="867" t="n">
         <v>142.915944245401</v>
       </c>
-      <c r="K53" s="864" t="n">
+      <c r="K53" s="867" t="n">
         <v>221.944073516401</v>
       </c>
-      <c r="L53" s="864" t="n">
+      <c r="L53" s="867" t="n">
         <v>5.87980417282567</v>
       </c>
-      <c r="M53" s="864" t="n">
+      <c r="M53" s="867" t="n">
         <v>22.5009174886484</v>
       </c>
       <c r="N53" s="781" t="s">
-        <v>768</v>
+        <v>777</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="783" t="s">
-        <v>769</v>
-      </c>
-      <c r="B54" s="864" t="n">
-        <v>19.3741392318594</v>
-      </c>
-      <c r="C54" s="864" t="n">
-        <v>32.925863476306</v>
-      </c>
-      <c r="D54" s="875" t="n">
-        <v>-6.63335912458738</v>
-      </c>
-      <c r="E54" s="875" t="n">
-        <v>6.91836511985926</v>
-      </c>
-      <c r="F54" s="864" t="n">
-        <v>12.7144146114538</v>
-      </c>
-      <c r="G54" s="864" t="n">
-        <v>33.7306141755154</v>
-      </c>
-      <c r="H54" s="864" t="n">
+        <v>778</v>
+      </c>
+      <c r="B54" s="867" t="n">
+        <v>18.8484476206593</v>
+      </c>
+      <c r="C54" s="867" t="n">
+        <v>32.3685862470535</v>
+      </c>
+      <c r="D54" s="878" t="n">
+        <v>-6.61756631556115</v>
+      </c>
+      <c r="E54" s="878" t="n">
+        <v>6.90257231083302</v>
+      </c>
+      <c r="F54" s="867" t="n">
+        <v>12.0328233612089</v>
+      </c>
+      <c r="G54" s="867" t="n">
+        <v>32.9818194826057</v>
+      </c>
+      <c r="H54" s="867" t="n">
         <v>21.8654496208832</v>
       </c>
-      <c r="I54" s="864" t="n">
+      <c r="I54" s="867" t="n">
         <v>34.7285606679383</v>
       </c>
-      <c r="J54" s="864" t="n">
+      <c r="J54" s="867" t="n">
         <v>170.288003540798</v>
       </c>
-      <c r="K54" s="864" t="n">
+      <c r="K54" s="867" t="n">
         <v>187.840751522138</v>
       </c>
-      <c r="L54" s="864" t="n">
+      <c r="L54" s="867" t="n">
         <v>11.5840438628959</v>
       </c>
-      <c r="M54" s="864" t="n">
+      <c r="M54" s="867" t="n">
         <v>15.2430370919031</v>
       </c>
       <c r="N54" s="781" t="s">
-        <v>770</v>
+        <v>779</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="783" t="s">
-        <v>771</v>
-      </c>
-      <c r="B55" s="864" t="n">
-        <v>16.991754813111</v>
-      </c>
-      <c r="C55" s="864" t="n">
-        <v>35.0041933420044</v>
-      </c>
-      <c r="D55" s="875" t="n">
-        <v>-9.01574354333572</v>
-      </c>
-      <c r="E55" s="875" t="n">
-        <v>8.99669498555765</v>
-      </c>
-      <c r="F55" s="864" t="n">
-        <v>10.5311256827794</v>
-      </c>
-      <c r="G55" s="864" t="n">
-        <v>35.4166973517185</v>
-      </c>
-      <c r="H55" s="864" t="n">
+        <v>780</v>
+      </c>
+      <c r="B55" s="867" t="n">
+        <v>16.2086328366892</v>
+      </c>
+      <c r="C55" s="867" t="n">
+        <v>34.7043464779736</v>
+      </c>
+      <c r="D55" s="878" t="n">
+        <v>-9.25738109953126</v>
+      </c>
+      <c r="E55" s="878" t="n">
+        <v>9.23833254175318</v>
+      </c>
+      <c r="F55" s="867" t="n">
+        <v>9.30181025121158</v>
+      </c>
+      <c r="G55" s="867" t="n">
+        <v>35.2156268401317</v>
+      </c>
+      <c r="H55" s="867" t="n">
         <v>18.0927775026868</v>
       </c>
-      <c r="I55" s="864" t="n">
+      <c r="I55" s="867" t="n">
         <v>38.2383021559811</v>
       </c>
-      <c r="J55" s="864" t="n">
+      <c r="J55" s="867" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="K55" s="864" t="n">
+      <c r="K55" s="867" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="L55" s="864" t="n">
+      <c r="L55" s="867" t="n">
         <v>11.9430083321538</v>
       </c>
-      <c r="M55" s="864" t="n">
+      <c r="M55" s="867" t="n">
         <v>14.8052836766288</v>
       </c>
       <c r="N55" s="781" t="s">
-        <v>772</v>
+        <v>781</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="783" t="s">
-        <v>773</v>
-      </c>
-      <c r="B56" s="864" t="n">
-        <v>14.866604664728</v>
-      </c>
-      <c r="C56" s="864" t="n">
-        <v>37.1221726922844</v>
-      </c>
-      <c r="D56" s="875" t="n">
-        <v>-11.1408936917188</v>
-      </c>
-      <c r="E56" s="875" t="n">
-        <v>11.1146743358376</v>
-      </c>
-      <c r="F56" s="864" t="n">
-        <v>7.46763841904257</v>
-      </c>
-      <c r="G56" s="864" t="n">
-        <v>38.4644591134795</v>
-      </c>
-      <c r="H56" s="864" t="n">
+        <v>782</v>
+      </c>
+      <c r="B56" s="867" t="n">
+        <v>14.0866643468269</v>
+      </c>
+      <c r="C56" s="867" t="n">
+        <v>36.8191441697328</v>
+      </c>
+      <c r="D56" s="878" t="n">
+        <v>-11.3793495893935</v>
+      </c>
+      <c r="E56" s="878" t="n">
+        <v>11.3531302335124</v>
+      </c>
+      <c r="F56" s="867" t="n">
+        <v>6.24509247368928</v>
+      </c>
+      <c r="G56" s="867" t="n">
+        <v>38.2566191156782</v>
+      </c>
+      <c r="H56" s="867" t="n">
         <v>15.8433893954659</v>
       </c>
-      <c r="I56" s="864" t="n">
+      <c r="I56" s="867" t="n">
         <v>40.4854887699201</v>
       </c>
-      <c r="J56" s="864" t="n">
+      <c r="J56" s="867" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="K56" s="864" t="n">
+      <c r="K56" s="867" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="L56" s="864" t="n">
+      <c r="L56" s="867" t="n">
         <v>11.5422897839273</v>
       </c>
-      <c r="M56" s="864" t="n">
+      <c r="M56" s="867" t="n">
         <v>15.2060022248553</v>
       </c>
       <c r="N56" s="781" t="s">
-        <v>774</v>
+        <v>783</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="46.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="783" t="s">
-        <v>775</v>
-      </c>
-      <c r="B57" s="864" t="n">
-        <v>21.6260696287263</v>
-      </c>
-      <c r="C57" s="864" t="n">
-        <v>31.198177127893</v>
-      </c>
-      <c r="D57" s="875" t="n">
+        <v>784</v>
+      </c>
+      <c r="B57" s="867" t="n">
+        <v>21.0845852085</v>
+      </c>
+      <c r="C57" s="867" t="n">
+        <v>30.6566927076667</v>
+      </c>
+      <c r="D57" s="878" t="n">
         <v>-4.38142872772042</v>
       </c>
-      <c r="E57" s="875" t="n">
+      <c r="E57" s="878" t="n">
         <v>5.19067877144628</v>
       </c>
-      <c r="F57" s="864" t="n">
-        <v>15.7283531504832</v>
-      </c>
-      <c r="G57" s="864" t="n">
-        <v>32.1506176525824</v>
-      </c>
-      <c r="H57" s="864" t="n">
+      <c r="F57" s="867" t="n">
+        <v>15.0131601789059</v>
+      </c>
+      <c r="G57" s="867" t="n">
+        <v>31.4354246810051</v>
+      </c>
+      <c r="H57" s="867" t="n">
         <v>24.4813370740213</v>
       </c>
-      <c r="I57" s="864" t="n">
+      <c r="I57" s="867" t="n">
         <v>31.9893413198388</v>
       </c>
-      <c r="J57" s="864" t="n">
+      <c r="J57" s="867" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="K57" s="864" t="n">
+      <c r="K57" s="867" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="L57" s="864" t="n">
+      <c r="L57" s="867" t="n">
         <v>13.0793877210432</v>
       </c>
-      <c r="M57" s="864" t="n">
+      <c r="M57" s="867" t="n">
         <v>13.6689042877394</v>
       </c>
       <c r="N57" s="781" t="s">
-        <v>776</v>
+        <v>785</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="30.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="783" t="s">
-        <v>777</v>
-      </c>
-      <c r="B58" s="864" t="n">
-        <v>21.7559343776643</v>
-      </c>
-      <c r="C58" s="864" t="n">
-        <v>31.259573190541</v>
-      </c>
-      <c r="D58" s="875" t="n">
+        <v>786</v>
+      </c>
+      <c r="B58" s="867" t="n">
+        <v>21.214449957438</v>
+      </c>
+      <c r="C58" s="867" t="n">
+        <v>30.7180887703147</v>
+      </c>
+      <c r="D58" s="878" t="n">
         <v>-4.25156397878245</v>
       </c>
-      <c r="E58" s="875" t="n">
+      <c r="E58" s="878" t="n">
         <v>5.25207483409425</v>
       </c>
-      <c r="F58" s="864" t="n">
-        <v>14.9782604607731</v>
-      </c>
-      <c r="G58" s="864" t="n">
-        <v>33.38364800817</v>
-      </c>
-      <c r="H58" s="864" t="n">
+      <c r="F58" s="867" t="n">
+        <v>14.2630674891958</v>
+      </c>
+      <c r="G58" s="867" t="n">
+        <v>32.6684550365927</v>
+      </c>
+      <c r="H58" s="867" t="n">
         <v>25.5560916360763</v>
       </c>
-      <c r="I58" s="864" t="n">
+      <c r="I58" s="867" t="n">
         <v>30.9098011208712</v>
       </c>
-      <c r="J58" s="864" t="n">
+      <c r="J58" s="867" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="K58" s="864" t="n">
+      <c r="K58" s="867" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="L58" s="864" t="n">
+      <c r="L58" s="867" t="n">
         <v>13.3741460043913</v>
       </c>
-      <c r="M58" s="864" t="n">
+      <c r="M58" s="867" t="n">
         <v>13.3741460043913</v>
       </c>
       <c r="N58" s="781" t="s">
-        <v>778</v>
+        <v>787</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="786" t="s">
-        <v>779</v>
-      </c>
-      <c r="B59" s="876" t="n">
-        <v>26.0074983564468</v>
-      </c>
-      <c r="C59" s="876" t="n">
-        <v>29.4860145263927</v>
-      </c>
-      <c r="D59" s="877" t="n">
-        <v>0</v>
-      </c>
-      <c r="E59" s="877" t="n">
-        <v>3.47851616994597</v>
-      </c>
-      <c r="F59" s="876" t="n">
-        <v>22.9947614067526</v>
-      </c>
-      <c r="G59" s="876" t="n">
-        <v>26.6177473961008</v>
-      </c>
-      <c r="H59" s="876" t="n">
+        <v>788</v>
+      </c>
+      <c r="B59" s="879" t="n">
+        <v>25.4660139362204</v>
+      </c>
+      <c r="C59" s="879" t="n">
+        <v>29.2723388763702</v>
+      </c>
+      <c r="D59" s="880" t="n">
+        <v>0</v>
+      </c>
+      <c r="E59" s="880" t="n">
+        <v>3.80632494014975</v>
+      </c>
+      <c r="F59" s="879" t="n">
+        <v>22.2795684351753</v>
+      </c>
+      <c r="G59" s="879" t="n">
+        <v>26.6000198930422</v>
+      </c>
+      <c r="H59" s="879" t="n">
         <v>28.1685006370529</v>
       </c>
-      <c r="I59" s="876" t="n">
+      <c r="I59" s="879" t="n">
         <v>33.2418050725696</v>
       </c>
-      <c r="J59" s="876" t="n">
+      <c r="J59" s="879" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="K59" s="876" t="n">
+      <c r="K59" s="879" t="n">
         <v>178.89220902969</v>
       </c>
-      <c r="L59" s="876" t="n">
+      <c r="L59" s="879" t="n">
         <v>13.3741460043913</v>
       </c>
-      <c r="M59" s="876" t="n">
+      <c r="M59" s="879" t="n">
         <v>13.3741460043913</v>
       </c>
       <c r="N59" s="804" t="s">
-        <v>780</v>
+        <v>789</v>
       </c>
     </row>
   </sheetData>
@@ -13707,7 +13789,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="790" t="s">
-        <v>781</v>
+        <v>790</v>
       </c>
       <c r="B1" s="226"/>
       <c r="C1" s="226"/>
@@ -13717,7 +13799,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="336" t="s">
-        <v>782</v>
+        <v>791</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -13735,7 +13817,7 @@
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="414" t="s">
-        <v>783</v>
+        <v>792</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -13745,164 +13827,164 @@
     </row>
     <row r="5" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="813" t="s">
-        <v>784</v>
-      </c>
-      <c r="B5" s="878" t="n">
+        <v>793</v>
+      </c>
+      <c r="B5" s="881" t="n">
         <f aca="false">Assumption!$B$14+(-0.02)</f>
         <v>0.03</v>
       </c>
-      <c r="C5" s="878" t="n">
+      <c r="C5" s="881" t="n">
         <f aca="false">Assumption!$B$14+(-0.01)</f>
         <v>0.04</v>
       </c>
-      <c r="D5" s="878" t="n">
+      <c r="D5" s="881" t="n">
         <f aca="false">Assumption!$B$14+(0)</f>
         <v>0.05</v>
       </c>
-      <c r="E5" s="878" t="n">
+      <c r="E5" s="881" t="n">
         <f aca="false">Assumption!$B$14+(0.01)</f>
         <v>0.06</v>
       </c>
-      <c r="F5" s="879" t="n">
+      <c r="F5" s="882" t="n">
         <f aca="false">Assumption!$B$14+(0.02)</f>
         <v>0.07</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="880" t="n">
+      <c r="A6" s="883" t="n">
         <f aca="false">Assumption!$B$16+(-0.02)</f>
         <v>0.121309839519679</v>
       </c>
-      <c r="B6" s="881" t="n">
+      <c r="B6" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A6)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+B$5)*(1-B$5/Assumption!$B$17)/($A6-B$5))/(1+$A6)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>43.6632784026025</v>
-      </c>
-      <c r="C6" s="881" t="n">
+        <v>42.9480854310252</v>
+      </c>
+      <c r="C6" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A6)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+C$5)*(1-C$5/Assumption!$B$17)/($A6-C$5))/(1+$A6)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>44.7004899324069</v>
-      </c>
-      <c r="D6" s="881" t="n">
+        <v>43.9852969608297</v>
+      </c>
+      <c r="D6" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A6)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+D$5)*(1-D$5/Assumption!$B$17)/($A6-D$5))/(1+$A6)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>45.8000450628265</v>
-      </c>
-      <c r="E6" s="881" t="n">
+        <v>45.0848520912492</v>
+      </c>
+      <c r="E6" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A6)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+E$5)*(1-E$5/Assumption!$B$17)/($A6-E$5))/(1+$A6)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>46.9924496316371</v>
-      </c>
-      <c r="F6" s="882" t="n">
+        <v>46.2772566600598</v>
+      </c>
+      <c r="F6" s="885" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A6)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+F$5)*(1-F$5/Assumption!$B$17)/($A6-F$5))/(1+$A6)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>48.3319911434931</v>
+        <v>47.6167981719158</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="880" t="n">
+      <c r="A7" s="883" t="n">
         <f aca="false">Assumption!$B$16+(-0.01)</f>
         <v>0.131309839519679</v>
       </c>
-      <c r="B7" s="881" t="n">
+      <c r="B7" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A7)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+B$5)*(1-B$5/Assumption!$B$17)/($A7-B$5))/(1+$A7)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>33.051201020086</v>
-      </c>
-      <c r="C7" s="881" t="n">
+        <v>32.3360080485087</v>
+      </c>
+      <c r="C7" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A7)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+C$5)*(1-C$5/Assumption!$B$17)/($A7-C$5))/(1+$A7)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>33.0495622160443</v>
-      </c>
-      <c r="D7" s="881" t="n">
+        <v>32.334369244467</v>
+      </c>
+      <c r="D7" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A7)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+D$5)*(1-D$5/Assumption!$B$17)/($A7-D$5))/(1+$A7)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>32.8544936419302</v>
-      </c>
-      <c r="E7" s="881" t="n">
+        <v>32.1393006703529</v>
+      </c>
+      <c r="E7" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A7)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+E$5)*(1-E$5/Assumption!$B$17)/($A7-E$5))/(1+$A7)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>32.3846195277062</v>
-      </c>
-      <c r="F7" s="882" t="n">
+        <v>31.6694265561289</v>
+      </c>
+      <c r="F7" s="885" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A7)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+F$5)*(1-F$5/Assumption!$B$17)/($A7-F$5))/(1+$A7)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>31.5054726121973</v>
+        <v>30.79027964062</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="880" t="n">
+      <c r="A8" s="883" t="n">
         <f aca="false">Assumption!$B$16+(0)</f>
         <v>0.141309839519679</v>
       </c>
-      <c r="B8" s="881" t="n">
+      <c r="B8" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A8)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+B$5)*(1-B$5/Assumption!$B$17)/($A8-B$5))/(1+$A8)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>24.5717305276797</v>
-      </c>
-      <c r="C8" s="881" t="n">
+        <v>23.8565375561025</v>
+      </c>
+      <c r="C8" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A8)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+C$5)*(1-C$5/Assumption!$B$17)/($A8-C$5))/(1+$A8)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>23.9356915628625</v>
-      </c>
-      <c r="D8" s="883" t="n">
+        <v>23.2204985912852</v>
+      </c>
+      <c r="D8" s="886" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A8)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+D$5)*(1-D$5/Assumption!$B$17)/($A8-D$5))/(1+$A8)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>22.9947614067526</v>
-      </c>
-      <c r="E8" s="881" t="n">
+        <v>22.2795684351753</v>
+      </c>
+      <c r="E8" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A8)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+E$5)*(1-E$5/Assumption!$B$17)/($A8-E$5))/(1+$A8)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>21.6364476993502</v>
-      </c>
-      <c r="F8" s="882" t="n">
+        <v>20.9212547277729</v>
+      </c>
+      <c r="F8" s="885" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A8)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+F$5)*(1-F$5/Assumption!$B$17)/($A8-F$5))/(1+$A8)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>19.6851574702728</v>
+        <v>18.9699644986955</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="880" t="n">
+      <c r="A9" s="883" t="n">
         <f aca="false">Assumption!$B$16+(0.01)</f>
         <v>0.151309839519679</v>
       </c>
-      <c r="B9" s="881" t="n">
+      <c r="B9" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A9)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+B$5)*(1-B$5/Assumption!$B$17)/($A9-B$5))/(1+$A9)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>17.6880241299027</v>
-      </c>
-      <c r="C9" s="881" t="n">
+        <v>16.9728311583254</v>
+      </c>
+      <c r="C9" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A9)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+C$5)*(1-C$5/Assumption!$B$17)/($A9-C$5))/(1+$A9)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>16.6653784440411</v>
-      </c>
-      <c r="D9" s="881" t="n">
+        <v>15.9501854724638</v>
+      </c>
+      <c r="D9" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A9)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+D$5)*(1-D$5/Assumption!$B$17)/($A9-D$5))/(1+$A9)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>15.2970464524351</v>
-      </c>
-      <c r="E9" s="881" t="n">
+        <v>14.5818534808578</v>
+      </c>
+      <c r="E9" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A9)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+E$5)*(1-E$5/Assumption!$B$17)/($A9-E$5))/(1+$A9)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>13.4694523430269</v>
-      </c>
-      <c r="F9" s="882" t="n">
+        <v>12.7542593714496</v>
+      </c>
+      <c r="F9" s="885" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A9)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+F$5)*(1-F$5/Assumption!$B$17)/($A9-F$5))/(1+$A9)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>11.0131472075974</v>
+        <v>10.2979542360202</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="880" t="n">
+      <c r="A10" s="883" t="n">
         <f aca="false">Assumption!$B$16+(0.02)</f>
         <v>0.161309839519679</v>
       </c>
-      <c r="B10" s="881" t="n">
+      <c r="B10" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A10)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+B$5)*(1-B$5/Assumption!$B$17)/($A10-B$5))/(1+$A10)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>12.0272360755729</v>
-      </c>
-      <c r="C10" s="881" t="n">
+        <v>11.3120431039956</v>
+      </c>
+      <c r="C10" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A10)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+C$5)*(1-C$5/Assumption!$B$17)/($A10-C$5))/(1+$A10)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>10.7742603486568</v>
-      </c>
-      <c r="D10" s="881" t="n">
+        <v>10.0590673770795</v>
+      </c>
+      <c r="D10" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A10)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+D$5)*(1-D$5/Assumption!$B$17)/($A10-D$5))/(1+$A10)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>9.16999241407187</v>
-      </c>
-      <c r="E10" s="881" t="n">
+        <v>8.45479944249458</v>
+      </c>
+      <c r="E10" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A10)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+E$5)*(1-E$5/Assumption!$B$17)/($A10-E$5))/(1+$A10)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>7.11040717139316</v>
-      </c>
-      <c r="F10" s="882" t="n">
+        <v>6.39521419981587</v>
+      </c>
+      <c r="F10" s="885" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A10)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+F$5)*(1-F$5/Assumption!$B$17)/($A10-F$5))/(1+$A10)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>4.44590935997118</v>
+        <v>3.73071638839389</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="825" t="s">
-        <v>785</v>
-      </c>
-      <c r="B11" s="884" t="n">
+        <v>794</v>
+      </c>
+      <c r="B11" s="887" t="n">
         <f aca="false">ROUND(D8-DCF!B22/1000000,6)</f>
         <v>0</v>
       </c>
@@ -13921,7 +14003,7 @@
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="414" t="s">
-        <v>786</v>
+        <v>795</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -13931,154 +14013,154 @@
     </row>
     <row r="14" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="813" t="s">
-        <v>787</v>
-      </c>
-      <c r="B14" s="885" t="n">
+        <v>796</v>
+      </c>
+      <c r="B14" s="888" t="n">
         <v>-0.3</v>
       </c>
-      <c r="C14" s="885" t="n">
+      <c r="C14" s="888" t="n">
         <v>-0.15</v>
       </c>
-      <c r="D14" s="885" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="885" t="n">
+      <c r="D14" s="888" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="888" t="n">
         <v>0.15</v>
       </c>
-      <c r="F14" s="886" t="n">
+      <c r="F14" s="889" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="887" t="n">
+      <c r="A15" s="890" t="n">
         <v>0.3</v>
       </c>
-      <c r="B15" s="881" t="n">
+      <c r="B15" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+B$14)*(1-$A15)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>15.5857524376136</v>
       </c>
-      <c r="C15" s="881" t="n">
+      <c r="C15" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+C$14)*(1-$A15)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>27.5965575370784</v>
       </c>
-      <c r="D15" s="881" t="n">
+      <c r="D15" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+D$14)*(1-$A15)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>39.6073626365432</v>
       </c>
-      <c r="E15" s="881" t="n">
+      <c r="E15" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+E$14)*(1-$A15)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>51.618167736008</v>
       </c>
-      <c r="F15" s="882" t="n">
+      <c r="F15" s="885" t="n">
         <f aca="false">(VCM!$E$4*(1+F$14)*(1-$A15)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>63.6289728354728</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="887" t="n">
+      <c r="A16" s="890" t="n">
         <v>0.35</v>
       </c>
-      <c r="B16" s="881" t="n">
+      <c r="B16" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+B$14)*(1-$A16)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>11.582150737792</v>
       </c>
-      <c r="C16" s="881" t="n">
+      <c r="C16" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+C$14)*(1-$A16)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>22.735041187295</v>
       </c>
-      <c r="D16" s="881" t="n">
+      <c r="D16" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+D$14)*(1-$A16)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>33.8879316367981</v>
       </c>
-      <c r="E16" s="881" t="n">
+      <c r="E16" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+E$14)*(1-$A16)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>45.0408220863011</v>
       </c>
-      <c r="F16" s="882" t="n">
+      <c r="F16" s="885" t="n">
         <f aca="false">(VCM!$E$4*(1+F$14)*(1-$A16)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>56.1937125358041</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="887" t="n">
+      <c r="A17" s="890" t="n">
         <v>0.4</v>
       </c>
-      <c r="B17" s="881" t="n">
+      <c r="B17" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+B$14)*(1-$A17)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>7.57854903797042</v>
       </c>
-      <c r="C17" s="881" t="n">
+      <c r="C17" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+C$14)*(1-$A17)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>17.8735248375117</v>
       </c>
-      <c r="D17" s="883" t="n">
+      <c r="D17" s="886" t="n">
         <f aca="false">(VCM!$E$4*(1+D$14)*(1-$A17)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>28.1685006370529</v>
       </c>
-      <c r="E17" s="881" t="n">
+      <c r="E17" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+E$14)*(1-$A17)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>38.4634764365942</v>
       </c>
-      <c r="F17" s="882" t="n">
+      <c r="F17" s="885" t="n">
         <f aca="false">(VCM!$E$4*(1+F$14)*(1-$A17)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>48.7584522361354</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="887" t="n">
+      <c r="A18" s="890" t="n">
         <v>0.45</v>
       </c>
-      <c r="B18" s="881" t="n">
+      <c r="B18" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+B$14)*(1-$A18)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>3.57494733814883</v>
       </c>
-      <c r="C18" s="881" t="n">
+      <c r="C18" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+C$14)*(1-$A18)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>13.0120084877283</v>
       </c>
-      <c r="D18" s="881" t="n">
+      <c r="D18" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+D$14)*(1-$A18)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>22.4490696373078</v>
       </c>
-      <c r="E18" s="881" t="n">
+      <c r="E18" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+E$14)*(1-$A18)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>31.8861307868873</v>
       </c>
-      <c r="F18" s="882" t="n">
+      <c r="F18" s="885" t="n">
         <f aca="false">(VCM!$E$4*(1+F$14)*(1-$A18)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>41.3231919364668</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="887" t="n">
+      <c r="A19" s="890" t="n">
         <v>0.5</v>
       </c>
-      <c r="B19" s="881" t="n">
+      <c r="B19" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+B$14)*(1-$A19)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>-0.428654361672774</v>
       </c>
-      <c r="C19" s="881" t="n">
+      <c r="C19" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+C$14)*(1-$A19)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>8.15049213794494</v>
       </c>
-      <c r="D19" s="881" t="n">
+      <c r="D19" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+D$14)*(1-$A19)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>16.7296386375626</v>
       </c>
-      <c r="E19" s="881" t="n">
+      <c r="E19" s="884" t="n">
         <f aca="false">(VCM!$E$4*(1+E$14)*(1-$A19)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>25.3087851371804</v>
       </c>
-      <c r="F19" s="882" t="n">
+      <c r="F19" s="885" t="n">
         <f aca="false">(VCM!$E$4*(1+F$14)*(1-$A19)/(1+VCM!$B$5)^VCM!$B$3-VCM!$E$3)/1000000</f>
         <v>33.8879316367981</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="825" t="s">
-        <v>788</v>
-      </c>
-      <c r="B20" s="884" t="n">
+        <v>797</v>
+      </c>
+      <c r="B20" s="887" t="n">
         <f aca="false">ROUND(D17-VCM!E7/1000000,6)</f>
         <v>0</v>
       </c>
@@ -14097,7 +14179,7 @@
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="414" t="s">
-        <v>789</v>
+        <v>798</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -14107,157 +14189,157 @@
     </row>
     <row r="23" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="813" t="s">
-        <v>790</v>
-      </c>
-      <c r="B23" s="878" t="n">
+        <v>799</v>
+      </c>
+      <c r="B23" s="881" t="n">
         <f aca="false">Assumption!$B$17+(-0.04)</f>
         <v>0.0831158832517256</v>
       </c>
-      <c r="C23" s="878" t="n">
+      <c r="C23" s="881" t="n">
         <f aca="false">Assumption!$B$17+(-0.02)</f>
         <v>0.103115883251726</v>
       </c>
-      <c r="D23" s="878" t="n">
+      <c r="D23" s="881" t="n">
         <f aca="false">Assumption!$B$17+(0)</f>
         <v>0.123115883251726</v>
       </c>
-      <c r="E23" s="878" t="n">
+      <c r="E23" s="881" t="n">
         <f aca="false">Assumption!$B$17+(0.02)</f>
         <v>0.143115883251726</v>
       </c>
-      <c r="F23" s="879" t="n">
+      <c r="F23" s="882" t="n">
         <f aca="false">Assumption!$B$17+(0.04)</f>
         <v>0.163115883251726</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="880" t="n">
+      <c r="A24" s="883" t="n">
         <f aca="false">Assumption!$B$16+(-0.02)</f>
         <v>0.121309839519679</v>
       </c>
-      <c r="B24" s="881" t="n">
+      <c r="B24" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A24)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/B$23)/($A24-Assumption!$B$14))/(1+$A24)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>16.9262450704033</v>
-      </c>
-      <c r="C24" s="881" t="n">
+        <v>16.211052098826</v>
+      </c>
+      <c r="C24" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A24)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/C$23)/($A24-Assumption!$B$14))/(1+$A24)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>34.1632762473697</v>
-      </c>
-      <c r="D24" s="881" t="n">
+        <v>33.4480832757925</v>
+      </c>
+      <c r="D24" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A24)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/D$23)/($A24-Assumption!$B$14))/(1+$A24)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>45.8000450628265</v>
-      </c>
-      <c r="E24" s="881" t="n">
+        <v>45.0848520912492</v>
+      </c>
+      <c r="E24" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A24)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/E$23)/($A24-Assumption!$B$14))/(1+$A24)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>54.1844093090465</v>
-      </c>
-      <c r="F24" s="882" t="n">
+        <v>53.4692163374692</v>
+      </c>
+      <c r="F24" s="885" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A24)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/F$23)/($A24-Assumption!$B$14))/(1+$A24)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>60.5127225860838</v>
+        <v>59.7975296145065</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="880" t="n">
+      <c r="A25" s="883" t="n">
         <f aca="false">Assumption!$B$16+(-0.01)</f>
         <v>0.131309839519679</v>
       </c>
-      <c r="B25" s="881" t="n">
+      <c r="B25" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A25)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/B$23)/($A25-Assumption!$B$14))/(1+$A25)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>8.46950312566897</v>
-      </c>
-      <c r="C25" s="881" t="n">
+        <v>7.75431015409168</v>
+      </c>
+      <c r="C25" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A25)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/C$23)/($A25-Assumption!$B$14))/(1+$A25)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>23.026812585772</v>
-      </c>
-      <c r="D25" s="881" t="n">
+        <v>22.3116196141947</v>
+      </c>
+      <c r="D25" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A25)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/D$23)/($A25-Assumption!$B$14))/(1+$A25)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>32.8544936419302</v>
-      </c>
-      <c r="E25" s="881" t="n">
+        <v>32.1393006703529</v>
+      </c>
+      <c r="E25" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A25)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/E$23)/($A25-Assumption!$B$14))/(1+$A25)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>39.9353989153131</v>
-      </c>
-      <c r="F25" s="882" t="n">
+        <v>39.2202059437358</v>
+      </c>
+      <c r="F25" s="885" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A25)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/F$23)/($A25-Assumption!$B$14))/(1+$A25)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>45.2798932071963</v>
+        <v>44.5647002356191</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="880" t="n">
+      <c r="A26" s="883" t="n">
         <f aca="false">Assumption!$B$16+(0)</f>
         <v>0.141309839519679</v>
       </c>
-      <c r="B26" s="881" t="n">
+      <c r="B26" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A26)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/B$23)/($A26-Assumption!$B$14))/(1+$A26)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>2.07750943539398</v>
-      </c>
-      <c r="C26" s="881" t="n">
+        <v>1.36231646381669</v>
+      </c>
+      <c r="C26" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A26)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/C$23)/($A26-Assumption!$B$14))/(1+$A26)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>14.5646543370482</v>
-      </c>
-      <c r="D26" s="883" t="n">
+        <v>13.8494613654709</v>
+      </c>
+      <c r="D26" s="886" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A26)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/D$23)/($A26-Assumption!$B$14))/(1+$A26)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>22.9947614067526</v>
-      </c>
-      <c r="E26" s="881" t="n">
+        <v>22.2795684351753</v>
+      </c>
+      <c r="E26" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A26)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/E$23)/($A26-Assumption!$B$14))/(1+$A26)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>29.0687059379142</v>
-      </c>
-      <c r="F26" s="882" t="n">
+        <v>28.3535129663369</v>
+      </c>
+      <c r="F26" s="885" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A26)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/F$23)/($A26-Assumption!$B$14))/(1+$A26)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>33.6531708647412</v>
+        <v>32.9379778931639</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="880" t="n">
+      <c r="A27" s="883" t="n">
         <f aca="false">Assumption!$B$16+(0.01)</f>
         <v>0.151309839519679</v>
       </c>
-      <c r="B27" s="881" t="n">
+      <c r="B27" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A27)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/B$23)/($A27-Assumption!$B$14))/(1+$A27)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>-2.86935038162652</v>
-      </c>
-      <c r="C27" s="881" t="n">
+        <v>-3.58454335320381</v>
+      </c>
+      <c r="C27" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A27)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/C$23)/($A27-Assumption!$B$14))/(1+$A27)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>7.9755937782705</v>
-      </c>
-      <c r="D27" s="881" t="n">
+        <v>7.26040080669321</v>
+      </c>
+      <c r="D27" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A27)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/D$23)/($A27-Assumption!$B$14))/(1+$A27)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>15.2970464524351</v>
-      </c>
-      <c r="E27" s="881" t="n">
+        <v>14.5818534808578</v>
+      </c>
+      <c r="E27" s="884" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A27)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/E$23)/($A27-Assumption!$B$14))/(1+$A27)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>20.5721986020697</v>
-      </c>
-      <c r="F27" s="882" t="n">
+        <v>19.8570056304924</v>
+      </c>
+      <c r="F27" s="885" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A27)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/F$23)/($A27-Assumption!$B$14))/(1+$A27)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>24.5537545562942</v>
+        <v>23.8385615847169</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="888" t="n">
+      <c r="A28" s="891" t="n">
         <f aca="false">Assumption!$B$16+(0.02)</f>
         <v>0.161309839519679</v>
       </c>
-      <c r="B28" s="889" t="n">
+      <c r="B28" s="892" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A28)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/B$23)/($A28-Assumption!$B$14))/(1+$A28)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>-6.76765950913217</v>
-      </c>
-      <c r="C28" s="889" t="n">
+        <v>-7.48285248070946</v>
+      </c>
+      <c r="C28" s="892" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A28)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/C$23)/($A28-Assumption!$B$14))/(1+$A28)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>2.74677236890245</v>
-      </c>
-      <c r="D28" s="889" t="n">
+        <v>2.03157939732516</v>
+      </c>
+      <c r="D28" s="892" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A28)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/D$23)/($A28-Assumption!$B$14))/(1+$A28)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>9.16999241407187</v>
-      </c>
-      <c r="E28" s="889" t="n">
+        <v>8.45479944249458</v>
+      </c>
+      <c r="E28" s="892" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A28)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/E$23)/($A28-Assumption!$B$14))/(1+$A28)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>13.7979623726044</v>
-      </c>
-      <c r="F28" s="890" t="n">
+        <v>13.0827694010271</v>
+      </c>
+      <c r="F28" s="893" t="n">
         <f aca="false">(SUMPRODUCT(DCF!$C$10:$G$10*DCF!$C$11:$G$11/(1+$A28)^DCF!$C$3:$G$3)+(DCF!$G$5*(1+Assumption!$B$14)*(1-Assumption!$B$14/F$23)/($A28-Assumption!$B$14))/(1+$A28)^DCF!$G$3+DCF!$B$31-DCF!$B$32)/1000000</f>
-        <v>17.2910410216522</v>
+        <v>16.5758480500749</v>
       </c>
     </row>
   </sheetData>
@@ -14285,13 +14367,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="329" t="s">
-        <v>791</v>
+        <v>800</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>792</v>
+        <v>801</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>292</v>
@@ -14309,12 +14391,12 @@
         <v>296</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>793</v>
+        <v>802</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>794</v>
+        <v>803</v>
       </c>
       <c r="B4" s="1" t="n">
         <f aca="false">ROUND('Balance Sheet'!G32-'Balance Sheet'!G75,0)</f>
@@ -14343,7 +14425,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>795</v>
+        <v>804</v>
       </c>
       <c r="B5" s="1" t="n">
         <f aca="false">ROUND('Cash Flow Statement'!F34-'Balance Sheet'!G6,0)</f>
@@ -14372,7 +14454,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>796</v>
+        <v>805</v>
       </c>
       <c r="B6" s="1" t="n">
         <f aca="false">ROUND('Income Statement'!E78-'Cash Flow Statement'!F4,0)</f>
@@ -14401,7 +14483,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>797</v>
+        <v>806</v>
       </c>
       <c r="B7" s="1" t="n">
         <f aca="false">ROUND('Pro Forma'!C4-'Income Statement'!E11,0)</f>
@@ -14430,7 +14512,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>798</v>
+        <v>807</v>
       </c>
       <c r="B8" s="1" t="n">
         <f aca="false">ROUND('Pro Forma'!C14-'Income Statement'!E78,0)</f>
@@ -14459,7 +14541,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>799</v>
+        <v>808</v>
       </c>
       <c r="B9" s="1" t="n">
         <f aca="false">ROUND('Pro Forma'!C36-Drivers!F115,0)</f>
@@ -14488,7 +14570,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>800</v>
+        <v>809</v>
       </c>
       <c r="B10" s="1" t="n">
         <f aca="false">ROUND('Pro Forma'!C9-'Income Statement'!E69,0)</f>
@@ -14517,7 +14599,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>801</v>
+        <v>810</v>
       </c>
       <c r="B11" s="1" t="n">
         <f aca="false">ROUND(SUM(Drivers!F96,'Cash Flow Statement'!F20),0)</f>
@@ -14546,7 +14628,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>802</v>
+        <v>811</v>
       </c>
       <c r="B12" s="1" t="n">
         <f aca="false">ROUND(MIN(0,'Balance Sheet'!G6-Drivers!F121),0)</f>
@@ -14575,7 +14657,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>803</v>
+        <v>812</v>
       </c>
       <c r="B13" s="1" t="n">
         <f aca="false">SUMPRODUCT((Drivers!F7:J7=Drivers!C156)*Drivers!F94:J94)</f>
@@ -14588,13 +14670,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>804</v>
-      </c>
-      <c r="B14" s="891" t="n">
+        <v>813</v>
+      </c>
+      <c r="B14" s="894" t="n">
         <f aca="false">Sensitivity!B11</f>
         <v>0</v>
       </c>
-      <c r="C14" s="891" t="n">
+      <c r="C14" s="894" t="n">
         <f aca="false">Sensitivity!B20</f>
         <v>0</v>
       </c>
@@ -14605,7 +14687,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>805</v>
+        <v>814</v>
       </c>
       <c r="G15" s="1" t="str">
         <f aca="false">IF(Assumption!B14&lt;Assumption!B16,"OK","LỖI")</f>
@@ -14614,7 +14696,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>806</v>
+        <v>815</v>
       </c>
       <c r="B16" s="1" t="n">
         <f aca="false">IF(Drivers!F$7=Drivers!$C$156,0,Drivers!F124)</f>
@@ -14643,7 +14725,7 @@
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>807</v>
+        <v>816</v>
       </c>
       <c r="G17" s="1" t="str">
         <f aca="false">IF(AND(COUNTIF(G4:G16,"LỖI")=0,SUMPRODUCT(ISERROR(G4:G16)*1)=0),"TẤT CẢ OK","CÓ LỖI")</f>

</xml_diff>